<commit_message>
📋 Planilha de custo agora é por funcionário/cargo
Planilha reformulada: aba Funcionários (um por linha — cargo, nome,
regime, salário, comissões, VT, VR, desconto) com custo total por
linha; aba Resumo por Cargo (COUNTIF/SUMIF) com quantidade, custo
total e custo médio por cargo + total geral. Texto do download
atualizado no post.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/downloads/planilha-custo-empregado-gestor-certo.xlsx
+++ b/assets/downloads/planilha-custo-empregado-gestor-certo.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instruções" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Custo Mensal" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funcionários" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo por Cargo" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,10 +19,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="R$ #,##0.00"/>
-    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="R$ #,##0.00"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -56,6 +57,8 @@
       <b val="1"/>
     </font>
     <font>
+      <i val="1"/>
+      <color rgb="006B7A88"/>
       <sz val="10"/>
     </font>
     <font>
@@ -63,15 +66,11 @@
       <color rgb="00FFFFFF"/>
     </font>
     <font>
-      <i val="1"/>
+      <b val="1"/>
       <sz val="10"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="000C8A67"/>
-    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -96,6 +95,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EAF2FE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E6F5F0"/>
       </patternFill>
     </fill>
   </fills>
@@ -125,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -139,18 +143,20 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -516,17 +522,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B20"/>
+  <dimension ref="B2:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="95" customWidth="1" min="2" max="2"/>
+    <col width="98" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>PLANILHA DE CUSTO MENSAL DO EMPREGADO</t>
+          <t>PLANILHA DE CUSTO DE FUNCIONÁRIOS POR CARGO</t>
         </is>
       </c>
     </row>
@@ -550,90 +556,83 @@
     <row r="7">
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>1) Vá na aba CUSTO MENSAL.</t>
+          <t>1) Na aba FUNCIONÁRIOS, defina RAT (%) e Terceiros (%) no topo (usados para quem não é Simples).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>2) Preencha as células amarelas: salário, comissões, RAT, Terceiros, VT e VR.</t>
+          <t>2) Cadastre um funcionário por linha: Cargo, Nome, Regime (escreva 'Simples' ou 'Presumido'), Salário, Comissões, VT, VR e o desconto do VR.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>3) Compare as colunas: empresa no SIMPLES (Anexos I, II, III e V) x LUCRO PRESUMIDO/REAL.</t>
+          <t>3) A coluna 'Custo total mensal' calcula sozinha cada linha.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="3" t="inlineStr"/>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>4) Na aba RESUMO POR CARGO, escreva os cargos que você usou — ela soma a quantidade e o custo total de cada cargo automaticamente.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>O que está incluído:</t>
-        </is>
-      </c>
+      <c r="B11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>• Remuneração (salário + comissões).</t>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>O que entra no custo:</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>• INSS patronal (20%), RAT e Terceiros (5,8%) — só fora do Simples (Anexos I/II/III/V).</t>
+          <t>• Remuneração (salário + comissões).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>• FGTS (8%) — sempre.</t>
+          <t>• INSS patronal 20% + RAT + Terceiros — só quando o Regime não é 'Simples'.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>• Provisões de 13º e de férias + 1/3 (com seus encargos e FGTS).</t>
+          <t>• FGTS 8% (sempre), provisões de 13º e férias + 1/3 (com encargos) e provisão da multa de 40% do FGTS.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>• Provisão da multa de 40% do FGTS (rescisão).</t>
+          <t>• VT (descontado até 6% do salário) e VR (descontado conforme a coluna).</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>• Custo de VT (descontado até 6% do salário) e VR (desconto conforme política).</t>
-        </is>
-      </c>
+      <c r="B17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="B18" s="3" t="inlineStr"/>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Dica: escreva o Cargo igual nas duas abas (ex.: 'Vendedor') para o resumo somar certo.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Observações: RAT varia de 1% a 3% (× FAP) conforme o risco; Terceiros padrão 5,8%. No Anexo IV do Simples há INSS patronal.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>Valores ilustrativos — a folha real depende da convenção coletiva e de adicionais. Fale com a Gestor Certo: (11) 91404-0532.</t>
+          <t>Valores ilustrativos — a folha real depende da convenção coletiva e de adicionais. Gestor Certo: (11) 91404-0532.</t>
         </is>
       </c>
     </row>
@@ -648,334 +647,900 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>CUSTO MENSAL DO EMPREGADO — SIMPLES x PRESUMIDO/REAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>ENTRADAS (edite as células amarelas)</t>
+          <t>CUSTO DE FUNCIONÁRIOS — UM POR LINHA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>RAT (%):</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Terceiros (%):</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="n">
+        <v>0.058</v>
+      </c>
+      <c r="F2" s="8" t="inlineStr">
+        <is>
+          <t>No Regime, escreva 'Simples' ou 'Presumido'</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>Cargo</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Nome</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>Regime</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>Salário</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>Comissões</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>VT (mês)</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>VR (mês)</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>Desc. VR (%)</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>Custo total mensal</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Vendedor</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Ana</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>Simples</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E5" s="11" t="n">
+        <v>800</v>
+      </c>
+      <c r="F5" s="11" t="n">
+        <v>250</v>
+      </c>
+      <c r="G5" s="11" t="n">
+        <v>500</v>
+      </c>
+      <c r="H5" s="12" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I5" s="13">
+        <f>IF(D5="","",(D5+E5)+(D5+E5)*IF(UPPER(C5)="SIMPLES",0,0.2+$B$2+$D$2)+(D5+E5)*0.08+((D5+E5)/12+(D5+E5)*4/3/12)+((D5+E5)/12+(D5+E5)*4/3/12)*IF(UPPER(C5)="SIMPLES",0,0.2+$B$2+$D$2)+((D5+E5)/12+(D5+E5)*4/3/12)*0.08+0.4*0.08*((D5+E5)+((D5+E5)/12+(D5+E5)*4/3/12))+(F5-MIN(F5,0.06*D5))+(G5-G5*H5))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Vendedor</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Bruno</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>Simples</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>500</v>
+      </c>
+      <c r="F6" s="11" t="n">
+        <v>250</v>
+      </c>
+      <c r="G6" s="11" t="n">
+        <v>500</v>
+      </c>
+      <c r="H6" s="12" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I6" s="13">
+        <f>IF(D6="","",(D6+E6)+(D6+E6)*IF(UPPER(C6)="SIMPLES",0,0.2+$B$2+$D$2)+(D6+E6)*0.08+((D6+E6)/12+(D6+E6)*4/3/12)+((D6+E6)/12+(D6+E6)*4/3/12)*IF(UPPER(C6)="SIMPLES",0,0.2+$B$2+$D$2)+((D6+E6)/12+(D6+E6)*4/3/12)*0.08+0.4*0.08*((D6+E6)+((D6+E6)/12+(D6+E6)*4/3/12))+(F6-MIN(F6,0.06*D6))+(G6-G6*H6))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Gerente</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Carla</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>Presumido</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>6000</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="11" t="n">
+        <v>800</v>
+      </c>
+      <c r="H7" s="12" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I7" s="13">
+        <f>IF(D7="","",(D7+E7)+(D7+E7)*IF(UPPER(C7)="SIMPLES",0,0.2+$B$2+$D$2)+(D7+E7)*0.08+((D7+E7)/12+(D7+E7)*4/3/12)+((D7+E7)/12+(D7+E7)*4/3/12)*IF(UPPER(C7)="SIMPLES",0,0.2+$B$2+$D$2)+((D7+E7)/12+(D7+E7)*4/3/12)*0.08+0.4*0.08*((D7+E7)+((D7+E7)/12+(D7+E7)*4/3/12))+(F7-MIN(F7,0.06*D7))+(G7-G7*H7))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="n"/>
+      <c r="B8" s="10" t="n"/>
+      <c r="C8" s="10" t="n"/>
+      <c r="D8" s="11" t="n"/>
+      <c r="E8" s="11" t="n"/>
+      <c r="F8" s="11" t="n"/>
+      <c r="G8" s="11" t="n"/>
+      <c r="H8" s="12" t="n"/>
+      <c r="I8" s="13">
+        <f>IF(D8="","",(D8+E8)+(D8+E8)*IF(UPPER(C8)="SIMPLES",0,0.2+$B$2+$D$2)+(D8+E8)*0.08+((D8+E8)/12+(D8+E8)*4/3/12)+((D8+E8)/12+(D8+E8)*4/3/12)*IF(UPPER(C8)="SIMPLES",0,0.2+$B$2+$D$2)+((D8+E8)/12+(D8+E8)*4/3/12)*0.08+0.4*0.08*((D8+E8)+((D8+E8)/12+(D8+E8)*4/3/12))+(F8-MIN(F8,0.06*D8))+(G8-G8*H8))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="n"/>
+      <c r="B9" s="10" t="n"/>
+      <c r="C9" s="10" t="n"/>
+      <c r="D9" s="11" t="n"/>
+      <c r="E9" s="11" t="n"/>
+      <c r="F9" s="11" t="n"/>
+      <c r="G9" s="11" t="n"/>
+      <c r="H9" s="12" t="n"/>
+      <c r="I9" s="13">
+        <f>IF(D9="","",(D9+E9)+(D9+E9)*IF(UPPER(C9)="SIMPLES",0,0.2+$B$2+$D$2)+(D9+E9)*0.08+((D9+E9)/12+(D9+E9)*4/3/12)+((D9+E9)/12+(D9+E9)*4/3/12)*IF(UPPER(C9)="SIMPLES",0,0.2+$B$2+$D$2)+((D9+E9)/12+(D9+E9)*4/3/12)*0.08+0.4*0.08*((D9+E9)+((D9+E9)/12+(D9+E9)*4/3/12))+(F9-MIN(F9,0.06*D9))+(G9-G9*H9))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="n"/>
+      <c r="B10" s="10" t="n"/>
+      <c r="C10" s="10" t="n"/>
+      <c r="D10" s="11" t="n"/>
+      <c r="E10" s="11" t="n"/>
+      <c r="F10" s="11" t="n"/>
+      <c r="G10" s="11" t="n"/>
+      <c r="H10" s="12" t="n"/>
+      <c r="I10" s="13">
+        <f>IF(D10="","",(D10+E10)+(D10+E10)*IF(UPPER(C10)="SIMPLES",0,0.2+$B$2+$D$2)+(D10+E10)*0.08+((D10+E10)/12+(D10+E10)*4/3/12)+((D10+E10)/12+(D10+E10)*4/3/12)*IF(UPPER(C10)="SIMPLES",0,0.2+$B$2+$D$2)+((D10+E10)/12+(D10+E10)*4/3/12)*0.08+0.4*0.08*((D10+E10)+((D10+E10)/12+(D10+E10)*4/3/12))+(F10-MIN(F10,0.06*D10))+(G10-G10*H10))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="n"/>
+      <c r="B11" s="10" t="n"/>
+      <c r="C11" s="10" t="n"/>
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="11" t="n"/>
+      <c r="F11" s="11" t="n"/>
+      <c r="G11" s="11" t="n"/>
+      <c r="H11" s="12" t="n"/>
+      <c r="I11" s="13">
+        <f>IF(D11="","",(D11+E11)+(D11+E11)*IF(UPPER(C11)="SIMPLES",0,0.2+$B$2+$D$2)+(D11+E11)*0.08+((D11+E11)/12+(D11+E11)*4/3/12)+((D11+E11)/12+(D11+E11)*4/3/12)*IF(UPPER(C11)="SIMPLES",0,0.2+$B$2+$D$2)+((D11+E11)/12+(D11+E11)*4/3/12)*0.08+0.4*0.08*((D11+E11)+((D11+E11)/12+(D11+E11)*4/3/12))+(F11-MIN(F11,0.06*D11))+(G11-G11*H11))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="n"/>
+      <c r="B12" s="10" t="n"/>
+      <c r="C12" s="10" t="n"/>
+      <c r="D12" s="11" t="n"/>
+      <c r="E12" s="11" t="n"/>
+      <c r="F12" s="11" t="n"/>
+      <c r="G12" s="11" t="n"/>
+      <c r="H12" s="12" t="n"/>
+      <c r="I12" s="13">
+        <f>IF(D12="","",(D12+E12)+(D12+E12)*IF(UPPER(C12)="SIMPLES",0,0.2+$B$2+$D$2)+(D12+E12)*0.08+((D12+E12)/12+(D12+E12)*4/3/12)+((D12+E12)/12+(D12+E12)*4/3/12)*IF(UPPER(C12)="SIMPLES",0,0.2+$B$2+$D$2)+((D12+E12)/12+(D12+E12)*4/3/12)*0.08+0.4*0.08*((D12+E12)+((D12+E12)/12+(D12+E12)*4/3/12))+(F12-MIN(F12,0.06*D12))+(G12-G12*H12))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="n"/>
+      <c r="B13" s="10" t="n"/>
+      <c r="C13" s="10" t="n"/>
+      <c r="D13" s="11" t="n"/>
+      <c r="E13" s="11" t="n"/>
+      <c r="F13" s="11" t="n"/>
+      <c r="G13" s="11" t="n"/>
+      <c r="H13" s="12" t="n"/>
+      <c r="I13" s="13">
+        <f>IF(D13="","",(D13+E13)+(D13+E13)*IF(UPPER(C13)="SIMPLES",0,0.2+$B$2+$D$2)+(D13+E13)*0.08+((D13+E13)/12+(D13+E13)*4/3/12)+((D13+E13)/12+(D13+E13)*4/3/12)*IF(UPPER(C13)="SIMPLES",0,0.2+$B$2+$D$2)+((D13+E13)/12+(D13+E13)*4/3/12)*0.08+0.4*0.08*((D13+E13)+((D13+E13)/12+(D13+E13)*4/3/12))+(F13-MIN(F13,0.06*D13))+(G13-G13*H13))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="n"/>
+      <c r="B14" s="10" t="n"/>
+      <c r="C14" s="10" t="n"/>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="11" t="n"/>
+      <c r="F14" s="11" t="n"/>
+      <c r="G14" s="11" t="n"/>
+      <c r="H14" s="12" t="n"/>
+      <c r="I14" s="13">
+        <f>IF(D14="","",(D14+E14)+(D14+E14)*IF(UPPER(C14)="SIMPLES",0,0.2+$B$2+$D$2)+(D14+E14)*0.08+((D14+E14)/12+(D14+E14)*4/3/12)+((D14+E14)/12+(D14+E14)*4/3/12)*IF(UPPER(C14)="SIMPLES",0,0.2+$B$2+$D$2)+((D14+E14)/12+(D14+E14)*4/3/12)*0.08+0.4*0.08*((D14+E14)+((D14+E14)/12+(D14+E14)*4/3/12))+(F14-MIN(F14,0.06*D14))+(G14-G14*H14))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="n"/>
+      <c r="B15" s="10" t="n"/>
+      <c r="C15" s="10" t="n"/>
+      <c r="D15" s="11" t="n"/>
+      <c r="E15" s="11" t="n"/>
+      <c r="F15" s="11" t="n"/>
+      <c r="G15" s="11" t="n"/>
+      <c r="H15" s="12" t="n"/>
+      <c r="I15" s="13">
+        <f>IF(D15="","",(D15+E15)+(D15+E15)*IF(UPPER(C15)="SIMPLES",0,0.2+$B$2+$D$2)+(D15+E15)*0.08+((D15+E15)/12+(D15+E15)*4/3/12)+((D15+E15)/12+(D15+E15)*4/3/12)*IF(UPPER(C15)="SIMPLES",0,0.2+$B$2+$D$2)+((D15+E15)/12+(D15+E15)*4/3/12)*0.08+0.4*0.08*((D15+E15)+((D15+E15)/12+(D15+E15)*4/3/12))+(F15-MIN(F15,0.06*D15))+(G15-G15*H15))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="n"/>
+      <c r="B16" s="10" t="n"/>
+      <c r="C16" s="10" t="n"/>
+      <c r="D16" s="11" t="n"/>
+      <c r="E16" s="11" t="n"/>
+      <c r="F16" s="11" t="n"/>
+      <c r="G16" s="11" t="n"/>
+      <c r="H16" s="12" t="n"/>
+      <c r="I16" s="13">
+        <f>IF(D16="","",(D16+E16)+(D16+E16)*IF(UPPER(C16)="SIMPLES",0,0.2+$B$2+$D$2)+(D16+E16)*0.08+((D16+E16)/12+(D16+E16)*4/3/12)+((D16+E16)/12+(D16+E16)*4/3/12)*IF(UPPER(C16)="SIMPLES",0,0.2+$B$2+$D$2)+((D16+E16)/12+(D16+E16)*4/3/12)*0.08+0.4*0.08*((D16+E16)+((D16+E16)/12+(D16+E16)*4/3/12))+(F16-MIN(F16,0.06*D16))+(G16-G16*H16))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="n"/>
+      <c r="B17" s="10" t="n"/>
+      <c r="C17" s="10" t="n"/>
+      <c r="D17" s="11" t="n"/>
+      <c r="E17" s="11" t="n"/>
+      <c r="F17" s="11" t="n"/>
+      <c r="G17" s="11" t="n"/>
+      <c r="H17" s="12" t="n"/>
+      <c r="I17" s="13">
+        <f>IF(D17="","",(D17+E17)+(D17+E17)*IF(UPPER(C17)="SIMPLES",0,0.2+$B$2+$D$2)+(D17+E17)*0.08+((D17+E17)/12+(D17+E17)*4/3/12)+((D17+E17)/12+(D17+E17)*4/3/12)*IF(UPPER(C17)="SIMPLES",0,0.2+$B$2+$D$2)+((D17+E17)/12+(D17+E17)*4/3/12)*0.08+0.4*0.08*((D17+E17)+((D17+E17)/12+(D17+E17)*4/3/12))+(F17-MIN(F17,0.06*D17))+(G17-G17*H17))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="n"/>
+      <c r="B18" s="10" t="n"/>
+      <c r="C18" s="10" t="n"/>
+      <c r="D18" s="11" t="n"/>
+      <c r="E18" s="11" t="n"/>
+      <c r="F18" s="11" t="n"/>
+      <c r="G18" s="11" t="n"/>
+      <c r="H18" s="12" t="n"/>
+      <c r="I18" s="13">
+        <f>IF(D18="","",(D18+E18)+(D18+E18)*IF(UPPER(C18)="SIMPLES",0,0.2+$B$2+$D$2)+(D18+E18)*0.08+((D18+E18)/12+(D18+E18)*4/3/12)+((D18+E18)/12+(D18+E18)*4/3/12)*IF(UPPER(C18)="SIMPLES",0,0.2+$B$2+$D$2)+((D18+E18)/12+(D18+E18)*4/3/12)*0.08+0.4*0.08*((D18+E18)+((D18+E18)/12+(D18+E18)*4/3/12))+(F18-MIN(F18,0.06*D18))+(G18-G18*H18))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="n"/>
+      <c r="B19" s="10" t="n"/>
+      <c r="C19" s="10" t="n"/>
+      <c r="D19" s="11" t="n"/>
+      <c r="E19" s="11" t="n"/>
+      <c r="F19" s="11" t="n"/>
+      <c r="G19" s="11" t="n"/>
+      <c r="H19" s="12" t="n"/>
+      <c r="I19" s="13">
+        <f>IF(D19="","",(D19+E19)+(D19+E19)*IF(UPPER(C19)="SIMPLES",0,0.2+$B$2+$D$2)+(D19+E19)*0.08+((D19+E19)/12+(D19+E19)*4/3/12)+((D19+E19)/12+(D19+E19)*4/3/12)*IF(UPPER(C19)="SIMPLES",0,0.2+$B$2+$D$2)+((D19+E19)/12+(D19+E19)*4/3/12)*0.08+0.4*0.08*((D19+E19)+((D19+E19)/12+(D19+E19)*4/3/12))+(F19-MIN(F19,0.06*D19))+(G19-G19*H19))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="n"/>
+      <c r="B20" s="10" t="n"/>
+      <c r="C20" s="10" t="n"/>
+      <c r="D20" s="11" t="n"/>
+      <c r="E20" s="11" t="n"/>
+      <c r="F20" s="11" t="n"/>
+      <c r="G20" s="11" t="n"/>
+      <c r="H20" s="12" t="n"/>
+      <c r="I20" s="13">
+        <f>IF(D20="","",(D20+E20)+(D20+E20)*IF(UPPER(C20)="SIMPLES",0,0.2+$B$2+$D$2)+(D20+E20)*0.08+((D20+E20)/12+(D20+E20)*4/3/12)+((D20+E20)/12+(D20+E20)*4/3/12)*IF(UPPER(C20)="SIMPLES",0,0.2+$B$2+$D$2)+((D20+E20)/12+(D20+E20)*4/3/12)*0.08+0.4*0.08*((D20+E20)+((D20+E20)/12+(D20+E20)*4/3/12))+(F20-MIN(F20,0.06*D20))+(G20-G20*H20))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="n"/>
+      <c r="B21" s="10" t="n"/>
+      <c r="C21" s="10" t="n"/>
+      <c r="D21" s="11" t="n"/>
+      <c r="E21" s="11" t="n"/>
+      <c r="F21" s="11" t="n"/>
+      <c r="G21" s="11" t="n"/>
+      <c r="H21" s="12" t="n"/>
+      <c r="I21" s="13">
+        <f>IF(D21="","",(D21+E21)+(D21+E21)*IF(UPPER(C21)="SIMPLES",0,0.2+$B$2+$D$2)+(D21+E21)*0.08+((D21+E21)/12+(D21+E21)*4/3/12)+((D21+E21)/12+(D21+E21)*4/3/12)*IF(UPPER(C21)="SIMPLES",0,0.2+$B$2+$D$2)+((D21+E21)/12+(D21+E21)*4/3/12)*0.08+0.4*0.08*((D21+E21)+((D21+E21)/12+(D21+E21)*4/3/12))+(F21-MIN(F21,0.06*D21))+(G21-G21*H21))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="n"/>
+      <c r="B22" s="10" t="n"/>
+      <c r="C22" s="10" t="n"/>
+      <c r="D22" s="11" t="n"/>
+      <c r="E22" s="11" t="n"/>
+      <c r="F22" s="11" t="n"/>
+      <c r="G22" s="11" t="n"/>
+      <c r="H22" s="12" t="n"/>
+      <c r="I22" s="13">
+        <f>IF(D22="","",(D22+E22)+(D22+E22)*IF(UPPER(C22)="SIMPLES",0,0.2+$B$2+$D$2)+(D22+E22)*0.08+((D22+E22)/12+(D22+E22)*4/3/12)+((D22+E22)/12+(D22+E22)*4/3/12)*IF(UPPER(C22)="SIMPLES",0,0.2+$B$2+$D$2)+((D22+E22)/12+(D22+E22)*4/3/12)*0.08+0.4*0.08*((D22+E22)+((D22+E22)/12+(D22+E22)*4/3/12))+(F22-MIN(F22,0.06*D22))+(G22-G22*H22))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="n"/>
+      <c r="B23" s="10" t="n"/>
+      <c r="C23" s="10" t="n"/>
+      <c r="D23" s="11" t="n"/>
+      <c r="E23" s="11" t="n"/>
+      <c r="F23" s="11" t="n"/>
+      <c r="G23" s="11" t="n"/>
+      <c r="H23" s="12" t="n"/>
+      <c r="I23" s="13">
+        <f>IF(D23="","",(D23+E23)+(D23+E23)*IF(UPPER(C23)="SIMPLES",0,0.2+$B$2+$D$2)+(D23+E23)*0.08+((D23+E23)/12+(D23+E23)*4/3/12)+((D23+E23)/12+(D23+E23)*4/3/12)*IF(UPPER(C23)="SIMPLES",0,0.2+$B$2+$D$2)+((D23+E23)/12+(D23+E23)*4/3/12)*0.08+0.4*0.08*((D23+E23)+((D23+E23)/12+(D23+E23)*4/3/12))+(F23-MIN(F23,0.06*D23))+(G23-G23*H23))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="n"/>
+      <c r="B24" s="10" t="n"/>
+      <c r="C24" s="10" t="n"/>
+      <c r="D24" s="11" t="n"/>
+      <c r="E24" s="11" t="n"/>
+      <c r="F24" s="11" t="n"/>
+      <c r="G24" s="11" t="n"/>
+      <c r="H24" s="12" t="n"/>
+      <c r="I24" s="13">
+        <f>IF(D24="","",(D24+E24)+(D24+E24)*IF(UPPER(C24)="SIMPLES",0,0.2+$B$2+$D$2)+(D24+E24)*0.08+((D24+E24)/12+(D24+E24)*4/3/12)+((D24+E24)/12+(D24+E24)*4/3/12)*IF(UPPER(C24)="SIMPLES",0,0.2+$B$2+$D$2)+((D24+E24)/12+(D24+E24)*4/3/12)*0.08+0.4*0.08*((D24+E24)+((D24+E24)/12+(D24+E24)*4/3/12))+(F24-MIN(F24,0.06*D24))+(G24-G24*H24))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="n"/>
+      <c r="B25" s="10" t="n"/>
+      <c r="C25" s="10" t="n"/>
+      <c r="D25" s="11" t="n"/>
+      <c r="E25" s="11" t="n"/>
+      <c r="F25" s="11" t="n"/>
+      <c r="G25" s="11" t="n"/>
+      <c r="H25" s="12" t="n"/>
+      <c r="I25" s="13">
+        <f>IF(D25="","",(D25+E25)+(D25+E25)*IF(UPPER(C25)="SIMPLES",0,0.2+$B$2+$D$2)+(D25+E25)*0.08+((D25+E25)/12+(D25+E25)*4/3/12)+((D25+E25)/12+(D25+E25)*4/3/12)*IF(UPPER(C25)="SIMPLES",0,0.2+$B$2+$D$2)+((D25+E25)/12+(D25+E25)*4/3/12)*0.08+0.4*0.08*((D25+E25)+((D25+E25)/12+(D25+E25)*4/3/12))+(F25-MIN(F25,0.06*D25))+(G25-G25*H25))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="n"/>
+      <c r="B26" s="10" t="n"/>
+      <c r="C26" s="10" t="n"/>
+      <c r="D26" s="11" t="n"/>
+      <c r="E26" s="11" t="n"/>
+      <c r="F26" s="11" t="n"/>
+      <c r="G26" s="11" t="n"/>
+      <c r="H26" s="12" t="n"/>
+      <c r="I26" s="13">
+        <f>IF(D26="","",(D26+E26)+(D26+E26)*IF(UPPER(C26)="SIMPLES",0,0.2+$B$2+$D$2)+(D26+E26)*0.08+((D26+E26)/12+(D26+E26)*4/3/12)+((D26+E26)/12+(D26+E26)*4/3/12)*IF(UPPER(C26)="SIMPLES",0,0.2+$B$2+$D$2)+((D26+E26)/12+(D26+E26)*4/3/12)*0.08+0.4*0.08*((D26+E26)+((D26+E26)/12+(D26+E26)*4/3/12))+(F26-MIN(F26,0.06*D26))+(G26-G26*H26))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="n"/>
+      <c r="B27" s="10" t="n"/>
+      <c r="C27" s="10" t="n"/>
+      <c r="D27" s="11" t="n"/>
+      <c r="E27" s="11" t="n"/>
+      <c r="F27" s="11" t="n"/>
+      <c r="G27" s="11" t="n"/>
+      <c r="H27" s="12" t="n"/>
+      <c r="I27" s="13">
+        <f>IF(D27="","",(D27+E27)+(D27+E27)*IF(UPPER(C27)="SIMPLES",0,0.2+$B$2+$D$2)+(D27+E27)*0.08+((D27+E27)/12+(D27+E27)*4/3/12)+((D27+E27)/12+(D27+E27)*4/3/12)*IF(UPPER(C27)="SIMPLES",0,0.2+$B$2+$D$2)+((D27+E27)/12+(D27+E27)*4/3/12)*0.08+0.4*0.08*((D27+E27)+((D27+E27)/12+(D27+E27)*4/3/12))+(F27-MIN(F27,0.06*D27))+(G27-G27*H27))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="n"/>
+      <c r="B28" s="10" t="n"/>
+      <c r="C28" s="10" t="n"/>
+      <c r="D28" s="11" t="n"/>
+      <c r="E28" s="11" t="n"/>
+      <c r="F28" s="11" t="n"/>
+      <c r="G28" s="11" t="n"/>
+      <c r="H28" s="12" t="n"/>
+      <c r="I28" s="13">
+        <f>IF(D28="","",(D28+E28)+(D28+E28)*IF(UPPER(C28)="SIMPLES",0,0.2+$B$2+$D$2)+(D28+E28)*0.08+((D28+E28)/12+(D28+E28)*4/3/12)+((D28+E28)/12+(D28+E28)*4/3/12)*IF(UPPER(C28)="SIMPLES",0,0.2+$B$2+$D$2)+((D28+E28)/12+(D28+E28)*4/3/12)*0.08+0.4*0.08*((D28+E28)+((D28+E28)/12+(D28+E28)*4/3/12))+(F28-MIN(F28,0.06*D28))+(G28-G28*H28))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="n"/>
+      <c r="B29" s="10" t="n"/>
+      <c r="C29" s="10" t="n"/>
+      <c r="D29" s="11" t="n"/>
+      <c r="E29" s="11" t="n"/>
+      <c r="F29" s="11" t="n"/>
+      <c r="G29" s="11" t="n"/>
+      <c r="H29" s="12" t="n"/>
+      <c r="I29" s="13">
+        <f>IF(D29="","",(D29+E29)+(D29+E29)*IF(UPPER(C29)="SIMPLES",0,0.2+$B$2+$D$2)+(D29+E29)*0.08+((D29+E29)/12+(D29+E29)*4/3/12)+((D29+E29)/12+(D29+E29)*4/3/12)*IF(UPPER(C29)="SIMPLES",0,0.2+$B$2+$D$2)+((D29+E29)/12+(D29+E29)*4/3/12)*0.08+0.4*0.08*((D29+E29)+((D29+E29)/12+(D29+E29)*4/3/12))+(F29-MIN(F29,0.06*D29))+(G29-G29*H29))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="n"/>
+      <c r="B30" s="10" t="n"/>
+      <c r="C30" s="10" t="n"/>
+      <c r="D30" s="11" t="n"/>
+      <c r="E30" s="11" t="n"/>
+      <c r="F30" s="11" t="n"/>
+      <c r="G30" s="11" t="n"/>
+      <c r="H30" s="12" t="n"/>
+      <c r="I30" s="13">
+        <f>IF(D30="","",(D30+E30)+(D30+E30)*IF(UPPER(C30)="SIMPLES",0,0.2+$B$2+$D$2)+(D30+E30)*0.08+((D30+E30)/12+(D30+E30)*4/3/12)+((D30+E30)/12+(D30+E30)*4/3/12)*IF(UPPER(C30)="SIMPLES",0,0.2+$B$2+$D$2)+((D30+E30)/12+(D30+E30)*4/3/12)*0.08+0.4*0.08*((D30+E30)+((D30+E30)/12+(D30+E30)*4/3/12))+(F30-MIN(F30,0.06*D30))+(G30-G30*H30))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="n"/>
+      <c r="B31" s="10" t="n"/>
+      <c r="C31" s="10" t="n"/>
+      <c r="D31" s="11" t="n"/>
+      <c r="E31" s="11" t="n"/>
+      <c r="F31" s="11" t="n"/>
+      <c r="G31" s="11" t="n"/>
+      <c r="H31" s="12" t="n"/>
+      <c r="I31" s="13">
+        <f>IF(D31="","",(D31+E31)+(D31+E31)*IF(UPPER(C31)="SIMPLES",0,0.2+$B$2+$D$2)+(D31+E31)*0.08+((D31+E31)/12+(D31+E31)*4/3/12)+((D31+E31)/12+(D31+E31)*4/3/12)*IF(UPPER(C31)="SIMPLES",0,0.2+$B$2+$D$2)+((D31+E31)/12+(D31+E31)*4/3/12)*0.08+0.4*0.08*((D31+E31)+((D31+E31)/12+(D31+E31)*4/3/12))+(F31-MIN(F31,0.06*D31))+(G31-G31*H31))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="n"/>
+      <c r="B32" s="10" t="n"/>
+      <c r="C32" s="10" t="n"/>
+      <c r="D32" s="11" t="n"/>
+      <c r="E32" s="11" t="n"/>
+      <c r="F32" s="11" t="n"/>
+      <c r="G32" s="11" t="n"/>
+      <c r="H32" s="12" t="n"/>
+      <c r="I32" s="13">
+        <f>IF(D32="","",(D32+E32)+(D32+E32)*IF(UPPER(C32)="SIMPLES",0,0.2+$B$2+$D$2)+(D32+E32)*0.08+((D32+E32)/12+(D32+E32)*4/3/12)+((D32+E32)/12+(D32+E32)*4/3/12)*IF(UPPER(C32)="SIMPLES",0,0.2+$B$2+$D$2)+((D32+E32)/12+(D32+E32)*4/3/12)*0.08+0.4*0.08*((D32+E32)+((D32+E32)/12+(D32+E32)*4/3/12))+(F32-MIN(F32,0.06*D32))+(G32-G32*H32))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="n"/>
+      <c r="B33" s="10" t="n"/>
+      <c r="C33" s="10" t="n"/>
+      <c r="D33" s="11" t="n"/>
+      <c r="E33" s="11" t="n"/>
+      <c r="F33" s="11" t="n"/>
+      <c r="G33" s="11" t="n"/>
+      <c r="H33" s="12" t="n"/>
+      <c r="I33" s="13">
+        <f>IF(D33="","",(D33+E33)+(D33+E33)*IF(UPPER(C33)="SIMPLES",0,0.2+$B$2+$D$2)+(D33+E33)*0.08+((D33+E33)/12+(D33+E33)*4/3/12)+((D33+E33)/12+(D33+E33)*4/3/12)*IF(UPPER(C33)="SIMPLES",0,0.2+$B$2+$D$2)+((D33+E33)/12+(D33+E33)*4/3/12)*0.08+0.4*0.08*((D33+E33)+((D33+E33)/12+(D33+E33)*4/3/12))+(F33-MIN(F33,0.06*D33))+(G33-G33*H33))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="n"/>
+      <c r="B34" s="10" t="n"/>
+      <c r="C34" s="10" t="n"/>
+      <c r="D34" s="11" t="n"/>
+      <c r="E34" s="11" t="n"/>
+      <c r="F34" s="11" t="n"/>
+      <c r="G34" s="11" t="n"/>
+      <c r="H34" s="12" t="n"/>
+      <c r="I34" s="13">
+        <f>IF(D34="","",(D34+E34)+(D34+E34)*IF(UPPER(C34)="SIMPLES",0,0.2+$B$2+$D$2)+(D34+E34)*0.08+((D34+E34)/12+(D34+E34)*4/3/12)+((D34+E34)/12+(D34+E34)*4/3/12)*IF(UPPER(C34)="SIMPLES",0,0.2+$B$2+$D$2)+((D34+E34)/12+(D34+E34)*4/3/12)*0.08+0.4*0.08*((D34+E34)+((D34+E34)/12+(D34+E34)*4/3/12))+(F34-MIN(F34,0.06*D34))+(G34-G34*H34))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="D35" s="14">
+        <f>COUNT(D5:D34)</f>
+        <v/>
+      </c>
+      <c r="H35" s="15" t="inlineStr">
+        <is>
+          <t>Funcionários:</t>
+        </is>
+      </c>
+      <c r="I35" s="16">
+        <f>SUM(I5:I34)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:I1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>RESUMO POR CARGO</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="26" customHeight="1">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>Cargo</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Funcionários</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>Custo total/mês</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>Custo médio</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>Salário base</t>
-        </is>
-      </c>
-      <c r="B4" s="8" t="n">
-        <v>3000</v>
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Vendedor</t>
+        </is>
+      </c>
+      <c r="B4" s="17">
+        <f>IF(A4="","",COUNTIF(Funcionários!$A$5:$A$34,A4))</f>
+        <v/>
+      </c>
+      <c r="C4" s="11">
+        <f>IF(A4="","",SUMIF(Funcionários!$A$5:$A$34,A4,Funcionários!$I$5:$I$34))</f>
+        <v/>
+      </c>
+      <c r="D4" s="11">
+        <f>IF(OR(A4="",B4=0),"",C4/B4)</f>
+        <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>Comissões / médias</t>
-        </is>
-      </c>
-      <c r="B5" s="8" t="n">
-        <v>0</v>
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Gerente</t>
+        </is>
+      </c>
+      <c r="B5" s="17">
+        <f>IF(A5="","",COUNTIF(Funcionários!$A$5:$A$34,A5))</f>
+        <v/>
+      </c>
+      <c r="C5" s="11">
+        <f>IF(A5="","",SUMIF(Funcionários!$A$5:$A$34,A5,Funcionários!$I$5:$I$34))</f>
+        <v/>
+      </c>
+      <c r="D5" s="11">
+        <f>IF(OR(A5="",B5=0),"",C5/B5)</f>
+        <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>RAT (%) — fora do Simples</t>
-        </is>
-      </c>
-      <c r="B6" s="9" t="n">
-        <v>0.02</v>
+      <c r="A6" s="10" t="n"/>
+      <c r="B6" s="17">
+        <f>IF(A6="","",COUNTIF(Funcionários!$A$5:$A$34,A6))</f>
+        <v/>
+      </c>
+      <c r="C6" s="11">
+        <f>IF(A6="","",SUMIF(Funcionários!$A$5:$A$34,A6,Funcionários!$I$5:$I$34))</f>
+        <v/>
+      </c>
+      <c r="D6" s="11">
+        <f>IF(OR(A6="",B6=0),"",C6/B6)</f>
+        <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>Terceiros (%) — fora do Simples</t>
-        </is>
-      </c>
-      <c r="B7" s="9" t="n">
-        <v>0.058</v>
+      <c r="A7" s="10" t="n"/>
+      <c r="B7" s="17">
+        <f>IF(A7="","",COUNTIF(Funcionários!$A$5:$A$34,A7))</f>
+        <v/>
+      </c>
+      <c r="C7" s="11">
+        <f>IF(A7="","",SUMIF(Funcionários!$A$5:$A$34,A7,Funcionários!$I$5:$I$34))</f>
+        <v/>
+      </c>
+      <c r="D7" s="11">
+        <f>IF(OR(A7="",B7=0),"",C7/B7)</f>
+        <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>Vale-transporte (VT) mensal</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="n">
-        <v>300</v>
+      <c r="A8" s="10" t="n"/>
+      <c r="B8" s="17">
+        <f>IF(A8="","",COUNTIF(Funcionários!$A$5:$A$34,A8))</f>
+        <v/>
+      </c>
+      <c r="C8" s="11">
+        <f>IF(A8="","",SUMIF(Funcionários!$A$5:$A$34,A8,Funcionários!$I$5:$I$34))</f>
+        <v/>
+      </c>
+      <c r="D8" s="11">
+        <f>IF(OR(A8="",B8=0),"",C8/B8)</f>
+        <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>Vale-refeição (VR) mensal</t>
-        </is>
-      </c>
-      <c r="B9" s="8" t="n">
-        <v>600</v>
+      <c r="A9" s="10" t="n"/>
+      <c r="B9" s="17">
+        <f>IF(A9="","",COUNTIF(Funcionários!$A$5:$A$34,A9))</f>
+        <v/>
+      </c>
+      <c r="C9" s="11">
+        <f>IF(A9="","",SUMIF(Funcionários!$A$5:$A$34,A9,Funcionários!$I$5:$I$34))</f>
+        <v/>
+      </c>
+      <c r="D9" s="11">
+        <f>IF(OR(A9="",B9=0),"",C9/B9)</f>
+        <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>Desconto do VR (%)</t>
-        </is>
-      </c>
-      <c r="B10" s="9" t="n">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="12" ht="28" customHeight="1">
-      <c r="A12" s="10" t="inlineStr">
-        <is>
-          <t>Componente</t>
-        </is>
-      </c>
-      <c r="B12" s="10" t="inlineStr">
-        <is>
-          <t>Simples (I/II/III/V)</t>
-        </is>
-      </c>
-      <c r="C12" s="10" t="inlineStr">
-        <is>
-          <t>Presumido / Real</t>
-        </is>
+      <c r="A10" s="10" t="n"/>
+      <c r="B10" s="17">
+        <f>IF(A10="","",COUNTIF(Funcionários!$A$5:$A$34,A10))</f>
+        <v/>
+      </c>
+      <c r="C10" s="11">
+        <f>IF(A10="","",SUMIF(Funcionários!$A$5:$A$34,A10,Funcionários!$I$5:$I$34))</f>
+        <v/>
+      </c>
+      <c r="D10" s="11">
+        <f>IF(OR(A10="",B10=0),"",C10/B10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="n"/>
+      <c r="B11" s="17">
+        <f>IF(A11="","",COUNTIF(Funcionários!$A$5:$A$34,A11))</f>
+        <v/>
+      </c>
+      <c r="C11" s="11">
+        <f>IF(A11="","",SUMIF(Funcionários!$A$5:$A$34,A11,Funcionários!$I$5:$I$34))</f>
+        <v/>
+      </c>
+      <c r="D11" s="11">
+        <f>IF(OR(A11="",B11=0),"",C11/B11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="n"/>
+      <c r="B12" s="17">
+        <f>IF(A12="","",COUNTIF(Funcionários!$A$5:$A$34,A12))</f>
+        <v/>
+      </c>
+      <c r="C12" s="11">
+        <f>IF(A12="","",SUMIF(Funcionários!$A$5:$A$34,A12,Funcionários!$I$5:$I$34))</f>
+        <v/>
+      </c>
+      <c r="D12" s="11">
+        <f>IF(OR(A12="",B12=0),"",C12/B12)</f>
+        <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="inlineStr">
-        <is>
-          <t>Remuneração (salário + comissões)</t>
-        </is>
-      </c>
-      <c r="B13" s="12">
-        <f>($B$4+$B$5)</f>
-        <v/>
-      </c>
-      <c r="C13" s="12">
-        <f>($B$4+$B$5)</f>
+      <c r="A13" s="10" t="n"/>
+      <c r="B13" s="17">
+        <f>IF(A13="","",COUNTIF(Funcionários!$A$5:$A$34,A13))</f>
+        <v/>
+      </c>
+      <c r="C13" s="11">
+        <f>IF(A13="","",SUMIF(Funcionários!$A$5:$A$34,A13,Funcionários!$I$5:$I$34))</f>
+        <v/>
+      </c>
+      <c r="D13" s="11">
+        <f>IF(OR(A13="",B13=0),"",C13/B13)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="inlineStr">
-        <is>
-          <t>INSS patronal (20%)</t>
-        </is>
-      </c>
-      <c r="B14" s="12">
-        <f>0</f>
-        <v/>
-      </c>
-      <c r="C14" s="12">
-        <f>0.20*($B$4+$B$5)</f>
+      <c r="A14" s="10" t="n"/>
+      <c r="B14" s="17">
+        <f>IF(A14="","",COUNTIF(Funcionários!$A$5:$A$34,A14))</f>
+        <v/>
+      </c>
+      <c r="C14" s="11">
+        <f>IF(A14="","",SUMIF(Funcionários!$A$5:$A$34,A14,Funcionários!$I$5:$I$34))</f>
+        <v/>
+      </c>
+      <c r="D14" s="11">
+        <f>IF(OR(A14="",B14=0),"",C14/B14)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="inlineStr">
-        <is>
-          <t>RAT</t>
-        </is>
-      </c>
-      <c r="B15" s="12">
-        <f>0</f>
-        <v/>
-      </c>
-      <c r="C15" s="12">
-        <f>$B$6*($B$4+$B$5)</f>
+      <c r="A15" s="10" t="n"/>
+      <c r="B15" s="17">
+        <f>IF(A15="","",COUNTIF(Funcionários!$A$5:$A$34,A15))</f>
+        <v/>
+      </c>
+      <c r="C15" s="11">
+        <f>IF(A15="","",SUMIF(Funcionários!$A$5:$A$34,A15,Funcionários!$I$5:$I$34))</f>
+        <v/>
+      </c>
+      <c r="D15" s="11">
+        <f>IF(OR(A15="",B15=0),"",C15/B15)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="inlineStr">
-        <is>
-          <t>Terceiros (Sistema S)</t>
-        </is>
-      </c>
-      <c r="B16" s="12">
-        <f>0</f>
-        <v/>
-      </c>
-      <c r="C16" s="12">
-        <f>$B$7*($B$4+$B$5)</f>
+      <c r="A16" s="10" t="n"/>
+      <c r="B16" s="17">
+        <f>IF(A16="","",COUNTIF(Funcionários!$A$5:$A$34,A16))</f>
+        <v/>
+      </c>
+      <c r="C16" s="11">
+        <f>IF(A16="","",SUMIF(Funcionários!$A$5:$A$34,A16,Funcionários!$I$5:$I$34))</f>
+        <v/>
+      </c>
+      <c r="D16" s="11">
+        <f>IF(OR(A16="",B16=0),"",C16/B16)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="inlineStr">
-        <is>
-          <t>FGTS (8%)</t>
-        </is>
-      </c>
-      <c r="B17" s="12">
-        <f>0.08*($B$4+$B$5)</f>
-        <v/>
-      </c>
-      <c r="C17" s="12">
-        <f>0.08*($B$4+$B$5)</f>
+      <c r="A17" s="10" t="n"/>
+      <c r="B17" s="17">
+        <f>IF(A17="","",COUNTIF(Funcionários!$A$5:$A$34,A17))</f>
+        <v/>
+      </c>
+      <c r="C17" s="11">
+        <f>IF(A17="","",SUMIF(Funcionários!$A$5:$A$34,A17,Funcionários!$I$5:$I$34))</f>
+        <v/>
+      </c>
+      <c r="D17" s="11">
+        <f>IF(OR(A17="",B17=0),"",C17/B17)</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="inlineStr">
-        <is>
-          <t>Provisão 13º</t>
-        </is>
-      </c>
-      <c r="B18" s="12">
-        <f>($B$4+$B$5)/12</f>
-        <v/>
-      </c>
-      <c r="C18" s="12">
-        <f>($B$4+$B$5)/12</f>
+      <c r="A18" s="10" t="n"/>
+      <c r="B18" s="17">
+        <f>IF(A18="","",COUNTIF(Funcionários!$A$5:$A$34,A18))</f>
+        <v/>
+      </c>
+      <c r="C18" s="11">
+        <f>IF(A18="","",SUMIF(Funcionários!$A$5:$A$34,A18,Funcionários!$I$5:$I$34))</f>
+        <v/>
+      </c>
+      <c r="D18" s="11">
+        <f>IF(OR(A18="",B18=0),"",C18/B18)</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="inlineStr">
-        <is>
-          <t>Provisão férias + 1/3</t>
-        </is>
-      </c>
-      <c r="B19" s="12">
-        <f>($B$4+$B$5)*4/3/12</f>
-        <v/>
-      </c>
-      <c r="C19" s="12">
-        <f>($B$4+$B$5)*4/3/12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="11" t="inlineStr">
-        <is>
-          <t>Encargos s/ provisões (INSS+RAT+Terc)</t>
-        </is>
-      </c>
-      <c r="B20" s="12">
-        <f>0</f>
-        <v/>
-      </c>
-      <c r="C20" s="12">
-        <f>(0.20+$B$6+$B$7)*(($B$4+$B$5)/12+($B$4+$B$5)*4/3/12)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="11" t="inlineStr">
-        <is>
-          <t>FGTS s/ provisões (8%)</t>
-        </is>
-      </c>
-      <c r="B21" s="12">
-        <f>0.08*(($B$4+$B$5)/12+($B$4+$B$5)*4/3/12)</f>
-        <v/>
-      </c>
-      <c r="C21" s="12">
-        <f>0.08*(($B$4+$B$5)/12+($B$4+$B$5)*4/3/12)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="11" t="inlineStr">
-        <is>
-          <t>Provisão multa FGTS (40%)</t>
-        </is>
-      </c>
-      <c r="B22" s="12">
-        <f>0.40*0.08*(($B$4+$B$5)+(($B$4+$B$5)/12+($B$4+$B$5)*4/3/12))</f>
-        <v/>
-      </c>
-      <c r="C22" s="12">
-        <f>0.40*0.08*(($B$4+$B$5)+(($B$4+$B$5)/12+($B$4+$B$5)*4/3/12))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="11" t="inlineStr">
-        <is>
-          <t>Custo VT (líquido do desconto 6%)</t>
-        </is>
-      </c>
-      <c r="B23" s="12">
-        <f>$B$8-MIN($B$8,0.06*$B$4)</f>
-        <v/>
-      </c>
-      <c r="C23" s="12">
-        <f>$B$8-MIN($B$8,0.06*$B$4)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="11" t="inlineStr">
-        <is>
-          <t>Custo VR (líquido do desconto)</t>
-        </is>
-      </c>
-      <c r="B24" s="12">
-        <f>$B$9-$B$9*$B$10</f>
-        <v/>
-      </c>
-      <c r="C24" s="12">
-        <f>$B$9-$B$9*$B$10</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="13" t="inlineStr">
-        <is>
-          <t>CUSTO TOTAL MENSAL</t>
-        </is>
-      </c>
-      <c r="B25" s="13">
-        <f>SUM(B13:B24)</f>
-        <v/>
-      </c>
-      <c r="C25" s="13">
-        <f>SUM(C13:C24)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="14" t="inlineStr">
-        <is>
-          <t>% sobre o salário</t>
-        </is>
-      </c>
-      <c r="B26" s="15">
-        <f>B25/$B$4</f>
-        <v/>
-      </c>
-      <c r="C26" s="15">
-        <f>C25/$B$4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t>Economia no Simples (R$)</t>
-        </is>
-      </c>
-      <c r="B27" s="16">
-        <f>C25-B25</f>
+      <c r="A19" s="18" t="inlineStr">
+        <is>
+          <t>TOTAL GERAL</t>
+        </is>
+      </c>
+      <c r="B19" s="14">
+        <f>SUM(B4:B18)</f>
+        <v/>
+      </c>
+      <c r="C19" s="16">
+        <f>SUM(C4:C18)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
🧮 Planilha de custo: uma coluna por encargo
Aba Funcionários agora detalha cada encargo em coluna própria: INSS
patronal 20%, RAT, Terceiros, FGTS 8%, provisão 13º, provisão
férias+1/3, multa FGTS 40%, custo VT, custo VR e plano/outros, além do
custo total. Linha de total soma cada encargo (folha por componente).
Mantém Resumo por Cargo (gráfico) e Dashboard (KPIs + pizza por regime
+ barras por cargo).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/downloads/planilha-custo-empregado-gestor-certo.xlsx
+++ b/assets/downloads/planilha-custo-empregado-gestor-certo.xlsx
@@ -23,7 +23,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="R$ #,##0.00"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -68,15 +68,11 @@
     </font>
     <font>
       <b val="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <b val="1"/>
       <color rgb="006B7A88"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -96,6 +92,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001A56A5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E7DD1"/>
       </patternFill>
     </fill>
     <fill>
@@ -135,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -148,7 +149,7 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -160,13 +161,16 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="6" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -827,7 +831,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="98" customWidth="1" min="2" max="2"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -864,14 +868,14 @@
     <row r="8">
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>2) Cadastre um funcionário por linha: Cargo, Nome, Regime ('Simples' ou 'Presumido'), Salário, Comissões, VT, VR, Desconto do VR e Plano de saúde/outros benefícios.</t>
+          <t>2) Preencha as colunas amarelas de cada funcionário: Cargo, Nome, Regime ('Simples' ou 'Presumido'), Salário, Comissões, VT, VR, Desconto do VR e Plano de saúde/outros.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>3) A coluna 'Custo total mensal' calcula sozinha.</t>
+          <t>3) As colunas azuis são calculadas: há UMA COLUNA PARA CADA ENCARGO (INSS, RAT, Terceiros, FGTS, 13º, férias, multa FGTS, VT, VR) e o Custo total.</t>
         </is>
       </c>
     </row>
@@ -885,7 +889,7 @@
     <row r="11">
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>5) Veja a aba DASHBOARD para os indicadores e gráficos da folha.</t>
+          <t>5) Veja a aba DASHBOARD para indicadores e gráficos da folha.</t>
         </is>
       </c>
     </row>
@@ -895,7 +899,7 @@
     <row r="13">
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>O que entra no custo: remuneração (salário+comissões); INSS patronal 20% + RAT + Terceiros (só fora do Simples); FGTS 8%; provisões de 13º e férias+1/3 (com encargos); provisão da multa de 40% do FGTS; VT (desconto até 6% do salário); VR (desconto da coluna); e plano de saúde/outros benefícios.</t>
+          <t>Bases: INSS patronal 20% + RAT + Terceiros incidem sobre salário + 13º + férias (só fora do Simples). FGTS 8% e a multa de 40% também sobre essa base. 13º = 1/12; férias = (1+1/3)/12. VT desconta até 6% do salário; VR conforme a coluna.</t>
         </is>
       </c>
     </row>
@@ -905,7 +909,7 @@
     <row r="15">
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Dica: escreva o Cargo igual nas abas para o resumo somar certo. Valores ilustrativos — a folha real depende da convenção coletiva. Gestor Certo: (11) 91404-0532.</t>
+          <t>Dica: escreva o Cargo igual nas abas. Valores ilustrativos — a folha real depende da convenção coletiva. Gestor Certo: (11) 91404-0532.</t>
         </is>
       </c>
     </row>
@@ -966,15 +970,15 @@
         <v/>
       </c>
       <c r="B4" s="8">
-        <f>SUM('Funcionários'!J5:J34)</f>
+        <f>SUM('Funcionários'!S5:S34)</f>
         <v/>
       </c>
       <c r="D4" s="8">
-        <f>IFERROR(SUM('Funcionários'!J5:J34)/COUNT('Funcionários'!D5:D34),0)</f>
+        <f>IFERROR(SUM('Funcionários'!S5:S34)/COUNT('Funcionários'!D5:D34),0)</f>
         <v/>
       </c>
       <c r="E4" s="9">
-        <f>IFERROR(SUM('Funcionários'!J5:J34)/SUM('Funcionários'!D5:D34),0)</f>
+        <f>IFERROR(SUM('Funcionários'!S5:S34)/SUM('Funcionários'!D5:D34),0)</f>
         <v/>
       </c>
     </row>
@@ -1004,7 +1008,7 @@
         </is>
       </c>
       <c r="B10" s="13">
-        <f>SUMIF('Funcionários'!$C$5:$C$34,"Simples",'Funcionários'!$J$5:$J$34)</f>
+        <f>SUMIF('Funcionários'!$C$5:$C$34,"Simples",'Funcionários'!$S$5:$S$34)</f>
         <v/>
       </c>
     </row>
@@ -1015,7 +1019,7 @@
         </is>
       </c>
       <c r="B11" s="13">
-        <f>SUM('Funcionários'!$J$5:$J$34)-B10</f>
+        <f>SUM('Funcionários'!$S$5:$S$34)-B10</f>
         <v/>
       </c>
     </row>
@@ -1034,25 +1038,34 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J35"/>
+  <dimension ref="A1:S35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="9" customWidth="1" min="17" max="17"/>
+    <col width="9" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>CUSTO DE FUNCIONÁRIOS — UM POR LINHA</t>
+          <t>CUSTO DE FUNCIONÁRIOS — UMA COLUNA POR ENCARGO</t>
         </is>
       </c>
     </row>
@@ -1075,11 +1088,11 @@
       </c>
       <c r="F2" s="15" t="inlineStr">
         <is>
-          <t>Regime: escreva 'Simples' ou 'Presumido' em cada linha</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
+          <t>Amarelo = preencher · Azul = calculado</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
       <c r="A4" s="11" t="inlineStr">
         <is>
           <t>Cargo</t>
@@ -1122,12 +1135,57 @@
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>Plano saúde/outros</t>
-        </is>
-      </c>
-      <c r="J4" s="11" t="inlineStr">
-        <is>
-          <t>Custo total mensal</t>
+          <t>Plano/outros</t>
+        </is>
+      </c>
+      <c r="J4" s="16" t="inlineStr">
+        <is>
+          <t>INSS patr. 20%</t>
+        </is>
+      </c>
+      <c r="K4" s="16" t="inlineStr">
+        <is>
+          <t>RAT</t>
+        </is>
+      </c>
+      <c r="L4" s="16" t="inlineStr">
+        <is>
+          <t>Terceiros</t>
+        </is>
+      </c>
+      <c r="M4" s="16" t="inlineStr">
+        <is>
+          <t>FGTS 8%</t>
+        </is>
+      </c>
+      <c r="N4" s="16" t="inlineStr">
+        <is>
+          <t>Prov. 13º</t>
+        </is>
+      </c>
+      <c r="O4" s="16" t="inlineStr">
+        <is>
+          <t>Prov. férias+1/3</t>
+        </is>
+      </c>
+      <c r="P4" s="16" t="inlineStr">
+        <is>
+          <t>Multa FGTS 40%</t>
+        </is>
+      </c>
+      <c r="Q4" s="16" t="inlineStr">
+        <is>
+          <t>Custo VT</t>
+        </is>
+      </c>
+      <c r="R4" s="16" t="inlineStr">
+        <is>
+          <t>Custo VR</t>
+        </is>
+      </c>
+      <c r="S4" s="16" t="inlineStr">
+        <is>
+          <t>CUSTO TOTAL</t>
         </is>
       </c>
     </row>
@@ -1159,12 +1217,50 @@
       <c r="G5" s="13" t="n">
         <v>500</v>
       </c>
-      <c r="H5" s="16" t="n">
+      <c r="H5" s="17" t="n">
         <v>0.2</v>
       </c>
-      <c r="I5" s="13" t="n"/>
-      <c r="J5" s="17">
-        <f>IF(D5="","",(D5+E5)+(D5+E5)*IF(UPPER(C5)="SIMPLES",0,0.2+$B$2+$D$2)+(D5+E5)*0.08+((D5+E5)/12+(D5+E5)*4/3/12)+((D5+E5)/12+(D5+E5)*4/3/12)*IF(UPPER(C5)="SIMPLES",0,0.2+$B$2+$D$2)+((D5+E5)/12+(D5+E5)*4/3/12)*0.08+0.4*0.08*((D5+E5)+((D5+E5)/12+(D5+E5)*4/3/12))+(F5-MIN(F5,0.06*D5))+(G5-G5*H5)+I5)</f>
+      <c r="I5" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="18">
+        <f>IF(D5="","",IF(UPPER(C5)="SIMPLES",0,0.2*((D5+E5)+(D5+E5)/12+(D5+E5)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="K5" s="18">
+        <f>IF(D5="","",IF(UPPER(C5)="SIMPLES",0,$B$2*((D5+E5)+(D5+E5)/12+(D5+E5)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="L5" s="18">
+        <f>IF(D5="","",IF(UPPER(C5)="SIMPLES",0,$D$2*((D5+E5)+(D5+E5)/12+(D5+E5)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="M5" s="18">
+        <f>IF(D5="","",0.08*((D5+E5)+(D5+E5)/12+(D5+E5)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="N5" s="18">
+        <f>IF(D5="","",(D5+E5)/12)</f>
+        <v/>
+      </c>
+      <c r="O5" s="18">
+        <f>IF(D5="","",(D5+E5)*4/3/12)</f>
+        <v/>
+      </c>
+      <c r="P5" s="18">
+        <f>IF(D5="","",0.4*0.08*((D5+E5)+(D5+E5)/12+(D5+E5)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="Q5" s="18">
+        <f>IF(D5="","",F5-MIN(F5,0.06*D5))</f>
+        <v/>
+      </c>
+      <c r="R5" s="18">
+        <f>IF(D5="","",G5-G5*H5)</f>
+        <v/>
+      </c>
+      <c r="S5" s="19">
+        <f>IF(D5="","",D5+E5+J5+K5+L5+M5+N5+O5+P5+Q5+R5+I5)</f>
         <v/>
       </c>
     </row>
@@ -1196,12 +1292,50 @@
       <c r="G6" s="13" t="n">
         <v>500</v>
       </c>
-      <c r="H6" s="16" t="n">
+      <c r="H6" s="17" t="n">
         <v>0.2</v>
       </c>
-      <c r="I6" s="13" t="n"/>
-      <c r="J6" s="17">
-        <f>IF(D6="","",(D6+E6)+(D6+E6)*IF(UPPER(C6)="SIMPLES",0,0.2+$B$2+$D$2)+(D6+E6)*0.08+((D6+E6)/12+(D6+E6)*4/3/12)+((D6+E6)/12+(D6+E6)*4/3/12)*IF(UPPER(C6)="SIMPLES",0,0.2+$B$2+$D$2)+((D6+E6)/12+(D6+E6)*4/3/12)*0.08+0.4*0.08*((D6+E6)+((D6+E6)/12+(D6+E6)*4/3/12))+(F6-MIN(F6,0.06*D6))+(G6-G6*H6)+I6)</f>
+      <c r="I6" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="18">
+        <f>IF(D6="","",IF(UPPER(C6)="SIMPLES",0,0.2*((D6+E6)+(D6+E6)/12+(D6+E6)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="K6" s="18">
+        <f>IF(D6="","",IF(UPPER(C6)="SIMPLES",0,$B$2*((D6+E6)+(D6+E6)/12+(D6+E6)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="L6" s="18">
+        <f>IF(D6="","",IF(UPPER(C6)="SIMPLES",0,$D$2*((D6+E6)+(D6+E6)/12+(D6+E6)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="M6" s="18">
+        <f>IF(D6="","",0.08*((D6+E6)+(D6+E6)/12+(D6+E6)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="N6" s="18">
+        <f>IF(D6="","",(D6+E6)/12)</f>
+        <v/>
+      </c>
+      <c r="O6" s="18">
+        <f>IF(D6="","",(D6+E6)*4/3/12)</f>
+        <v/>
+      </c>
+      <c r="P6" s="18">
+        <f>IF(D6="","",0.4*0.08*((D6+E6)+(D6+E6)/12+(D6+E6)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="Q6" s="18">
+        <f>IF(D6="","",F6-MIN(F6,0.06*D6))</f>
+        <v/>
+      </c>
+      <c r="R6" s="18">
+        <f>IF(D6="","",G6-G6*H6)</f>
+        <v/>
+      </c>
+      <c r="S6" s="19">
+        <f>IF(D6="","",D6+E6+J6+K6+L6+M6+N6+O6+P6+Q6+R6+I6)</f>
         <v/>
       </c>
     </row>
@@ -1233,12 +1367,50 @@
       <c r="G7" s="13" t="n">
         <v>800</v>
       </c>
-      <c r="H7" s="16" t="n">
+      <c r="H7" s="17" t="n">
         <v>0.2</v>
       </c>
-      <c r="I7" s="13" t="n"/>
-      <c r="J7" s="17">
-        <f>IF(D7="","",(D7+E7)+(D7+E7)*IF(UPPER(C7)="SIMPLES",0,0.2+$B$2+$D$2)+(D7+E7)*0.08+((D7+E7)/12+(D7+E7)*4/3/12)+((D7+E7)/12+(D7+E7)*4/3/12)*IF(UPPER(C7)="SIMPLES",0,0.2+$B$2+$D$2)+((D7+E7)/12+(D7+E7)*4/3/12)*0.08+0.4*0.08*((D7+E7)+((D7+E7)/12+(D7+E7)*4/3/12))+(F7-MIN(F7,0.06*D7))+(G7-G7*H7)+I7)</f>
+      <c r="I7" s="13" t="n">
+        <v>500</v>
+      </c>
+      <c r="J7" s="18">
+        <f>IF(D7="","",IF(UPPER(C7)="SIMPLES",0,0.2*((D7+E7)+(D7+E7)/12+(D7+E7)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="K7" s="18">
+        <f>IF(D7="","",IF(UPPER(C7)="SIMPLES",0,$B$2*((D7+E7)+(D7+E7)/12+(D7+E7)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="L7" s="18">
+        <f>IF(D7="","",IF(UPPER(C7)="SIMPLES",0,$D$2*((D7+E7)+(D7+E7)/12+(D7+E7)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="M7" s="18">
+        <f>IF(D7="","",0.08*((D7+E7)+(D7+E7)/12+(D7+E7)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="N7" s="18">
+        <f>IF(D7="","",(D7+E7)/12)</f>
+        <v/>
+      </c>
+      <c r="O7" s="18">
+        <f>IF(D7="","",(D7+E7)*4/3/12)</f>
+        <v/>
+      </c>
+      <c r="P7" s="18">
+        <f>IF(D7="","",0.4*0.08*((D7+E7)+(D7+E7)/12+(D7+E7)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="Q7" s="18">
+        <f>IF(D7="","",F7-MIN(F7,0.06*D7))</f>
+        <v/>
+      </c>
+      <c r="R7" s="18">
+        <f>IF(D7="","",G7-G7*H7)</f>
+        <v/>
+      </c>
+      <c r="S7" s="19">
+        <f>IF(D7="","",D7+E7+J7+K7+L7+M7+N7+O7+P7+Q7+R7+I7)</f>
         <v/>
       </c>
     </row>
@@ -1250,10 +1422,46 @@
       <c r="E8" s="13" t="n"/>
       <c r="F8" s="13" t="n"/>
       <c r="G8" s="13" t="n"/>
-      <c r="H8" s="16" t="n"/>
+      <c r="H8" s="17" t="n"/>
       <c r="I8" s="13" t="n"/>
-      <c r="J8" s="17">
-        <f>IF(D8="","",(D8+E8)+(D8+E8)*IF(UPPER(C8)="SIMPLES",0,0.2+$B$2+$D$2)+(D8+E8)*0.08+((D8+E8)/12+(D8+E8)*4/3/12)+((D8+E8)/12+(D8+E8)*4/3/12)*IF(UPPER(C8)="SIMPLES",0,0.2+$B$2+$D$2)+((D8+E8)/12+(D8+E8)*4/3/12)*0.08+0.4*0.08*((D8+E8)+((D8+E8)/12+(D8+E8)*4/3/12))+(F8-MIN(F8,0.06*D8))+(G8-G8*H8)+I8)</f>
+      <c r="J8" s="18">
+        <f>IF(D8="","",IF(UPPER(C8)="SIMPLES",0,0.2*((D8+E8)+(D8+E8)/12+(D8+E8)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="K8" s="18">
+        <f>IF(D8="","",IF(UPPER(C8)="SIMPLES",0,$B$2*((D8+E8)+(D8+E8)/12+(D8+E8)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="L8" s="18">
+        <f>IF(D8="","",IF(UPPER(C8)="SIMPLES",0,$D$2*((D8+E8)+(D8+E8)/12+(D8+E8)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="M8" s="18">
+        <f>IF(D8="","",0.08*((D8+E8)+(D8+E8)/12+(D8+E8)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="N8" s="18">
+        <f>IF(D8="","",(D8+E8)/12)</f>
+        <v/>
+      </c>
+      <c r="O8" s="18">
+        <f>IF(D8="","",(D8+E8)*4/3/12)</f>
+        <v/>
+      </c>
+      <c r="P8" s="18">
+        <f>IF(D8="","",0.4*0.08*((D8+E8)+(D8+E8)/12+(D8+E8)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="Q8" s="18">
+        <f>IF(D8="","",F8-MIN(F8,0.06*D8))</f>
+        <v/>
+      </c>
+      <c r="R8" s="18">
+        <f>IF(D8="","",G8-G8*H8)</f>
+        <v/>
+      </c>
+      <c r="S8" s="19">
+        <f>IF(D8="","",D8+E8+J8+K8+L8+M8+N8+O8+P8+Q8+R8+I8)</f>
         <v/>
       </c>
     </row>
@@ -1265,10 +1473,46 @@
       <c r="E9" s="13" t="n"/>
       <c r="F9" s="13" t="n"/>
       <c r="G9" s="13" t="n"/>
-      <c r="H9" s="16" t="n"/>
+      <c r="H9" s="17" t="n"/>
       <c r="I9" s="13" t="n"/>
-      <c r="J9" s="17">
-        <f>IF(D9="","",(D9+E9)+(D9+E9)*IF(UPPER(C9)="SIMPLES",0,0.2+$B$2+$D$2)+(D9+E9)*0.08+((D9+E9)/12+(D9+E9)*4/3/12)+((D9+E9)/12+(D9+E9)*4/3/12)*IF(UPPER(C9)="SIMPLES",0,0.2+$B$2+$D$2)+((D9+E9)/12+(D9+E9)*4/3/12)*0.08+0.4*0.08*((D9+E9)+((D9+E9)/12+(D9+E9)*4/3/12))+(F9-MIN(F9,0.06*D9))+(G9-G9*H9)+I9)</f>
+      <c r="J9" s="18">
+        <f>IF(D9="","",IF(UPPER(C9)="SIMPLES",0,0.2*((D9+E9)+(D9+E9)/12+(D9+E9)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="K9" s="18">
+        <f>IF(D9="","",IF(UPPER(C9)="SIMPLES",0,$B$2*((D9+E9)+(D9+E9)/12+(D9+E9)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="L9" s="18">
+        <f>IF(D9="","",IF(UPPER(C9)="SIMPLES",0,$D$2*((D9+E9)+(D9+E9)/12+(D9+E9)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="M9" s="18">
+        <f>IF(D9="","",0.08*((D9+E9)+(D9+E9)/12+(D9+E9)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="N9" s="18">
+        <f>IF(D9="","",(D9+E9)/12)</f>
+        <v/>
+      </c>
+      <c r="O9" s="18">
+        <f>IF(D9="","",(D9+E9)*4/3/12)</f>
+        <v/>
+      </c>
+      <c r="P9" s="18">
+        <f>IF(D9="","",0.4*0.08*((D9+E9)+(D9+E9)/12+(D9+E9)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="Q9" s="18">
+        <f>IF(D9="","",F9-MIN(F9,0.06*D9))</f>
+        <v/>
+      </c>
+      <c r="R9" s="18">
+        <f>IF(D9="","",G9-G9*H9)</f>
+        <v/>
+      </c>
+      <c r="S9" s="19">
+        <f>IF(D9="","",D9+E9+J9+K9+L9+M9+N9+O9+P9+Q9+R9+I9)</f>
         <v/>
       </c>
     </row>
@@ -1280,10 +1524,46 @@
       <c r="E10" s="13" t="n"/>
       <c r="F10" s="13" t="n"/>
       <c r="G10" s="13" t="n"/>
-      <c r="H10" s="16" t="n"/>
+      <c r="H10" s="17" t="n"/>
       <c r="I10" s="13" t="n"/>
-      <c r="J10" s="17">
-        <f>IF(D10="","",(D10+E10)+(D10+E10)*IF(UPPER(C10)="SIMPLES",0,0.2+$B$2+$D$2)+(D10+E10)*0.08+((D10+E10)/12+(D10+E10)*4/3/12)+((D10+E10)/12+(D10+E10)*4/3/12)*IF(UPPER(C10)="SIMPLES",0,0.2+$B$2+$D$2)+((D10+E10)/12+(D10+E10)*4/3/12)*0.08+0.4*0.08*((D10+E10)+((D10+E10)/12+(D10+E10)*4/3/12))+(F10-MIN(F10,0.06*D10))+(G10-G10*H10)+I10)</f>
+      <c r="J10" s="18">
+        <f>IF(D10="","",IF(UPPER(C10)="SIMPLES",0,0.2*((D10+E10)+(D10+E10)/12+(D10+E10)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="K10" s="18">
+        <f>IF(D10="","",IF(UPPER(C10)="SIMPLES",0,$B$2*((D10+E10)+(D10+E10)/12+(D10+E10)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="L10" s="18">
+        <f>IF(D10="","",IF(UPPER(C10)="SIMPLES",0,$D$2*((D10+E10)+(D10+E10)/12+(D10+E10)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="M10" s="18">
+        <f>IF(D10="","",0.08*((D10+E10)+(D10+E10)/12+(D10+E10)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="N10" s="18">
+        <f>IF(D10="","",(D10+E10)/12)</f>
+        <v/>
+      </c>
+      <c r="O10" s="18">
+        <f>IF(D10="","",(D10+E10)*4/3/12)</f>
+        <v/>
+      </c>
+      <c r="P10" s="18">
+        <f>IF(D10="","",0.4*0.08*((D10+E10)+(D10+E10)/12+(D10+E10)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="Q10" s="18">
+        <f>IF(D10="","",F10-MIN(F10,0.06*D10))</f>
+        <v/>
+      </c>
+      <c r="R10" s="18">
+        <f>IF(D10="","",G10-G10*H10)</f>
+        <v/>
+      </c>
+      <c r="S10" s="19">
+        <f>IF(D10="","",D10+E10+J10+K10+L10+M10+N10+O10+P10+Q10+R10+I10)</f>
         <v/>
       </c>
     </row>
@@ -1295,10 +1575,46 @@
       <c r="E11" s="13" t="n"/>
       <c r="F11" s="13" t="n"/>
       <c r="G11" s="13" t="n"/>
-      <c r="H11" s="16" t="n"/>
+      <c r="H11" s="17" t="n"/>
       <c r="I11" s="13" t="n"/>
-      <c r="J11" s="17">
-        <f>IF(D11="","",(D11+E11)+(D11+E11)*IF(UPPER(C11)="SIMPLES",0,0.2+$B$2+$D$2)+(D11+E11)*0.08+((D11+E11)/12+(D11+E11)*4/3/12)+((D11+E11)/12+(D11+E11)*4/3/12)*IF(UPPER(C11)="SIMPLES",0,0.2+$B$2+$D$2)+((D11+E11)/12+(D11+E11)*4/3/12)*0.08+0.4*0.08*((D11+E11)+((D11+E11)/12+(D11+E11)*4/3/12))+(F11-MIN(F11,0.06*D11))+(G11-G11*H11)+I11)</f>
+      <c r="J11" s="18">
+        <f>IF(D11="","",IF(UPPER(C11)="SIMPLES",0,0.2*((D11+E11)+(D11+E11)/12+(D11+E11)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="K11" s="18">
+        <f>IF(D11="","",IF(UPPER(C11)="SIMPLES",0,$B$2*((D11+E11)+(D11+E11)/12+(D11+E11)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="L11" s="18">
+        <f>IF(D11="","",IF(UPPER(C11)="SIMPLES",0,$D$2*((D11+E11)+(D11+E11)/12+(D11+E11)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="M11" s="18">
+        <f>IF(D11="","",0.08*((D11+E11)+(D11+E11)/12+(D11+E11)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="N11" s="18">
+        <f>IF(D11="","",(D11+E11)/12)</f>
+        <v/>
+      </c>
+      <c r="O11" s="18">
+        <f>IF(D11="","",(D11+E11)*4/3/12)</f>
+        <v/>
+      </c>
+      <c r="P11" s="18">
+        <f>IF(D11="","",0.4*0.08*((D11+E11)+(D11+E11)/12+(D11+E11)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="Q11" s="18">
+        <f>IF(D11="","",F11-MIN(F11,0.06*D11))</f>
+        <v/>
+      </c>
+      <c r="R11" s="18">
+        <f>IF(D11="","",G11-G11*H11)</f>
+        <v/>
+      </c>
+      <c r="S11" s="19">
+        <f>IF(D11="","",D11+E11+J11+K11+L11+M11+N11+O11+P11+Q11+R11+I11)</f>
         <v/>
       </c>
     </row>
@@ -1310,10 +1626,46 @@
       <c r="E12" s="13" t="n"/>
       <c r="F12" s="13" t="n"/>
       <c r="G12" s="13" t="n"/>
-      <c r="H12" s="16" t="n"/>
+      <c r="H12" s="17" t="n"/>
       <c r="I12" s="13" t="n"/>
-      <c r="J12" s="17">
-        <f>IF(D12="","",(D12+E12)+(D12+E12)*IF(UPPER(C12)="SIMPLES",0,0.2+$B$2+$D$2)+(D12+E12)*0.08+((D12+E12)/12+(D12+E12)*4/3/12)+((D12+E12)/12+(D12+E12)*4/3/12)*IF(UPPER(C12)="SIMPLES",0,0.2+$B$2+$D$2)+((D12+E12)/12+(D12+E12)*4/3/12)*0.08+0.4*0.08*((D12+E12)+((D12+E12)/12+(D12+E12)*4/3/12))+(F12-MIN(F12,0.06*D12))+(G12-G12*H12)+I12)</f>
+      <c r="J12" s="18">
+        <f>IF(D12="","",IF(UPPER(C12)="SIMPLES",0,0.2*((D12+E12)+(D12+E12)/12+(D12+E12)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="K12" s="18">
+        <f>IF(D12="","",IF(UPPER(C12)="SIMPLES",0,$B$2*((D12+E12)+(D12+E12)/12+(D12+E12)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="L12" s="18">
+        <f>IF(D12="","",IF(UPPER(C12)="SIMPLES",0,$D$2*((D12+E12)+(D12+E12)/12+(D12+E12)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="M12" s="18">
+        <f>IF(D12="","",0.08*((D12+E12)+(D12+E12)/12+(D12+E12)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="N12" s="18">
+        <f>IF(D12="","",(D12+E12)/12)</f>
+        <v/>
+      </c>
+      <c r="O12" s="18">
+        <f>IF(D12="","",(D12+E12)*4/3/12)</f>
+        <v/>
+      </c>
+      <c r="P12" s="18">
+        <f>IF(D12="","",0.4*0.08*((D12+E12)+(D12+E12)/12+(D12+E12)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="Q12" s="18">
+        <f>IF(D12="","",F12-MIN(F12,0.06*D12))</f>
+        <v/>
+      </c>
+      <c r="R12" s="18">
+        <f>IF(D12="","",G12-G12*H12)</f>
+        <v/>
+      </c>
+      <c r="S12" s="19">
+        <f>IF(D12="","",D12+E12+J12+K12+L12+M12+N12+O12+P12+Q12+R12+I12)</f>
         <v/>
       </c>
     </row>
@@ -1325,10 +1677,46 @@
       <c r="E13" s="13" t="n"/>
       <c r="F13" s="13" t="n"/>
       <c r="G13" s="13" t="n"/>
-      <c r="H13" s="16" t="n"/>
+      <c r="H13" s="17" t="n"/>
       <c r="I13" s="13" t="n"/>
-      <c r="J13" s="17">
-        <f>IF(D13="","",(D13+E13)+(D13+E13)*IF(UPPER(C13)="SIMPLES",0,0.2+$B$2+$D$2)+(D13+E13)*0.08+((D13+E13)/12+(D13+E13)*4/3/12)+((D13+E13)/12+(D13+E13)*4/3/12)*IF(UPPER(C13)="SIMPLES",0,0.2+$B$2+$D$2)+((D13+E13)/12+(D13+E13)*4/3/12)*0.08+0.4*0.08*((D13+E13)+((D13+E13)/12+(D13+E13)*4/3/12))+(F13-MIN(F13,0.06*D13))+(G13-G13*H13)+I13)</f>
+      <c r="J13" s="18">
+        <f>IF(D13="","",IF(UPPER(C13)="SIMPLES",0,0.2*((D13+E13)+(D13+E13)/12+(D13+E13)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="K13" s="18">
+        <f>IF(D13="","",IF(UPPER(C13)="SIMPLES",0,$B$2*((D13+E13)+(D13+E13)/12+(D13+E13)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="L13" s="18">
+        <f>IF(D13="","",IF(UPPER(C13)="SIMPLES",0,$D$2*((D13+E13)+(D13+E13)/12+(D13+E13)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="M13" s="18">
+        <f>IF(D13="","",0.08*((D13+E13)+(D13+E13)/12+(D13+E13)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="N13" s="18">
+        <f>IF(D13="","",(D13+E13)/12)</f>
+        <v/>
+      </c>
+      <c r="O13" s="18">
+        <f>IF(D13="","",(D13+E13)*4/3/12)</f>
+        <v/>
+      </c>
+      <c r="P13" s="18">
+        <f>IF(D13="","",0.4*0.08*((D13+E13)+(D13+E13)/12+(D13+E13)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="Q13" s="18">
+        <f>IF(D13="","",F13-MIN(F13,0.06*D13))</f>
+        <v/>
+      </c>
+      <c r="R13" s="18">
+        <f>IF(D13="","",G13-G13*H13)</f>
+        <v/>
+      </c>
+      <c r="S13" s="19">
+        <f>IF(D13="","",D13+E13+J13+K13+L13+M13+N13+O13+P13+Q13+R13+I13)</f>
         <v/>
       </c>
     </row>
@@ -1340,10 +1728,46 @@
       <c r="E14" s="13" t="n"/>
       <c r="F14" s="13" t="n"/>
       <c r="G14" s="13" t="n"/>
-      <c r="H14" s="16" t="n"/>
+      <c r="H14" s="17" t="n"/>
       <c r="I14" s="13" t="n"/>
-      <c r="J14" s="17">
-        <f>IF(D14="","",(D14+E14)+(D14+E14)*IF(UPPER(C14)="SIMPLES",0,0.2+$B$2+$D$2)+(D14+E14)*0.08+((D14+E14)/12+(D14+E14)*4/3/12)+((D14+E14)/12+(D14+E14)*4/3/12)*IF(UPPER(C14)="SIMPLES",0,0.2+$B$2+$D$2)+((D14+E14)/12+(D14+E14)*4/3/12)*0.08+0.4*0.08*((D14+E14)+((D14+E14)/12+(D14+E14)*4/3/12))+(F14-MIN(F14,0.06*D14))+(G14-G14*H14)+I14)</f>
+      <c r="J14" s="18">
+        <f>IF(D14="","",IF(UPPER(C14)="SIMPLES",0,0.2*((D14+E14)+(D14+E14)/12+(D14+E14)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="K14" s="18">
+        <f>IF(D14="","",IF(UPPER(C14)="SIMPLES",0,$B$2*((D14+E14)+(D14+E14)/12+(D14+E14)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="L14" s="18">
+        <f>IF(D14="","",IF(UPPER(C14)="SIMPLES",0,$D$2*((D14+E14)+(D14+E14)/12+(D14+E14)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="M14" s="18">
+        <f>IF(D14="","",0.08*((D14+E14)+(D14+E14)/12+(D14+E14)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="N14" s="18">
+        <f>IF(D14="","",(D14+E14)/12)</f>
+        <v/>
+      </c>
+      <c r="O14" s="18">
+        <f>IF(D14="","",(D14+E14)*4/3/12)</f>
+        <v/>
+      </c>
+      <c r="P14" s="18">
+        <f>IF(D14="","",0.4*0.08*((D14+E14)+(D14+E14)/12+(D14+E14)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="Q14" s="18">
+        <f>IF(D14="","",F14-MIN(F14,0.06*D14))</f>
+        <v/>
+      </c>
+      <c r="R14" s="18">
+        <f>IF(D14="","",G14-G14*H14)</f>
+        <v/>
+      </c>
+      <c r="S14" s="19">
+        <f>IF(D14="","",D14+E14+J14+K14+L14+M14+N14+O14+P14+Q14+R14+I14)</f>
         <v/>
       </c>
     </row>
@@ -1355,10 +1779,46 @@
       <c r="E15" s="13" t="n"/>
       <c r="F15" s="13" t="n"/>
       <c r="G15" s="13" t="n"/>
-      <c r="H15" s="16" t="n"/>
+      <c r="H15" s="17" t="n"/>
       <c r="I15" s="13" t="n"/>
-      <c r="J15" s="17">
-        <f>IF(D15="","",(D15+E15)+(D15+E15)*IF(UPPER(C15)="SIMPLES",0,0.2+$B$2+$D$2)+(D15+E15)*0.08+((D15+E15)/12+(D15+E15)*4/3/12)+((D15+E15)/12+(D15+E15)*4/3/12)*IF(UPPER(C15)="SIMPLES",0,0.2+$B$2+$D$2)+((D15+E15)/12+(D15+E15)*4/3/12)*0.08+0.4*0.08*((D15+E15)+((D15+E15)/12+(D15+E15)*4/3/12))+(F15-MIN(F15,0.06*D15))+(G15-G15*H15)+I15)</f>
+      <c r="J15" s="18">
+        <f>IF(D15="","",IF(UPPER(C15)="SIMPLES",0,0.2*((D15+E15)+(D15+E15)/12+(D15+E15)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="K15" s="18">
+        <f>IF(D15="","",IF(UPPER(C15)="SIMPLES",0,$B$2*((D15+E15)+(D15+E15)/12+(D15+E15)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="L15" s="18">
+        <f>IF(D15="","",IF(UPPER(C15)="SIMPLES",0,$D$2*((D15+E15)+(D15+E15)/12+(D15+E15)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="M15" s="18">
+        <f>IF(D15="","",0.08*((D15+E15)+(D15+E15)/12+(D15+E15)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="N15" s="18">
+        <f>IF(D15="","",(D15+E15)/12)</f>
+        <v/>
+      </c>
+      <c r="O15" s="18">
+        <f>IF(D15="","",(D15+E15)*4/3/12)</f>
+        <v/>
+      </c>
+      <c r="P15" s="18">
+        <f>IF(D15="","",0.4*0.08*((D15+E15)+(D15+E15)/12+(D15+E15)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="Q15" s="18">
+        <f>IF(D15="","",F15-MIN(F15,0.06*D15))</f>
+        <v/>
+      </c>
+      <c r="R15" s="18">
+        <f>IF(D15="","",G15-G15*H15)</f>
+        <v/>
+      </c>
+      <c r="S15" s="19">
+        <f>IF(D15="","",D15+E15+J15+K15+L15+M15+N15+O15+P15+Q15+R15+I15)</f>
         <v/>
       </c>
     </row>
@@ -1370,10 +1830,46 @@
       <c r="E16" s="13" t="n"/>
       <c r="F16" s="13" t="n"/>
       <c r="G16" s="13" t="n"/>
-      <c r="H16" s="16" t="n"/>
+      <c r="H16" s="17" t="n"/>
       <c r="I16" s="13" t="n"/>
-      <c r="J16" s="17">
-        <f>IF(D16="","",(D16+E16)+(D16+E16)*IF(UPPER(C16)="SIMPLES",0,0.2+$B$2+$D$2)+(D16+E16)*0.08+((D16+E16)/12+(D16+E16)*4/3/12)+((D16+E16)/12+(D16+E16)*4/3/12)*IF(UPPER(C16)="SIMPLES",0,0.2+$B$2+$D$2)+((D16+E16)/12+(D16+E16)*4/3/12)*0.08+0.4*0.08*((D16+E16)+((D16+E16)/12+(D16+E16)*4/3/12))+(F16-MIN(F16,0.06*D16))+(G16-G16*H16)+I16)</f>
+      <c r="J16" s="18">
+        <f>IF(D16="","",IF(UPPER(C16)="SIMPLES",0,0.2*((D16+E16)+(D16+E16)/12+(D16+E16)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="K16" s="18">
+        <f>IF(D16="","",IF(UPPER(C16)="SIMPLES",0,$B$2*((D16+E16)+(D16+E16)/12+(D16+E16)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="L16" s="18">
+        <f>IF(D16="","",IF(UPPER(C16)="SIMPLES",0,$D$2*((D16+E16)+(D16+E16)/12+(D16+E16)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="M16" s="18">
+        <f>IF(D16="","",0.08*((D16+E16)+(D16+E16)/12+(D16+E16)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="N16" s="18">
+        <f>IF(D16="","",(D16+E16)/12)</f>
+        <v/>
+      </c>
+      <c r="O16" s="18">
+        <f>IF(D16="","",(D16+E16)*4/3/12)</f>
+        <v/>
+      </c>
+      <c r="P16" s="18">
+        <f>IF(D16="","",0.4*0.08*((D16+E16)+(D16+E16)/12+(D16+E16)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="Q16" s="18">
+        <f>IF(D16="","",F16-MIN(F16,0.06*D16))</f>
+        <v/>
+      </c>
+      <c r="R16" s="18">
+        <f>IF(D16="","",G16-G16*H16)</f>
+        <v/>
+      </c>
+      <c r="S16" s="19">
+        <f>IF(D16="","",D16+E16+J16+K16+L16+M16+N16+O16+P16+Q16+R16+I16)</f>
         <v/>
       </c>
     </row>
@@ -1385,10 +1881,46 @@
       <c r="E17" s="13" t="n"/>
       <c r="F17" s="13" t="n"/>
       <c r="G17" s="13" t="n"/>
-      <c r="H17" s="16" t="n"/>
+      <c r="H17" s="17" t="n"/>
       <c r="I17" s="13" t="n"/>
-      <c r="J17" s="17">
-        <f>IF(D17="","",(D17+E17)+(D17+E17)*IF(UPPER(C17)="SIMPLES",0,0.2+$B$2+$D$2)+(D17+E17)*0.08+((D17+E17)/12+(D17+E17)*4/3/12)+((D17+E17)/12+(D17+E17)*4/3/12)*IF(UPPER(C17)="SIMPLES",0,0.2+$B$2+$D$2)+((D17+E17)/12+(D17+E17)*4/3/12)*0.08+0.4*0.08*((D17+E17)+((D17+E17)/12+(D17+E17)*4/3/12))+(F17-MIN(F17,0.06*D17))+(G17-G17*H17)+I17)</f>
+      <c r="J17" s="18">
+        <f>IF(D17="","",IF(UPPER(C17)="SIMPLES",0,0.2*((D17+E17)+(D17+E17)/12+(D17+E17)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="K17" s="18">
+        <f>IF(D17="","",IF(UPPER(C17)="SIMPLES",0,$B$2*((D17+E17)+(D17+E17)/12+(D17+E17)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="L17" s="18">
+        <f>IF(D17="","",IF(UPPER(C17)="SIMPLES",0,$D$2*((D17+E17)+(D17+E17)/12+(D17+E17)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="M17" s="18">
+        <f>IF(D17="","",0.08*((D17+E17)+(D17+E17)/12+(D17+E17)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="N17" s="18">
+        <f>IF(D17="","",(D17+E17)/12)</f>
+        <v/>
+      </c>
+      <c r="O17" s="18">
+        <f>IF(D17="","",(D17+E17)*4/3/12)</f>
+        <v/>
+      </c>
+      <c r="P17" s="18">
+        <f>IF(D17="","",0.4*0.08*((D17+E17)+(D17+E17)/12+(D17+E17)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="Q17" s="18">
+        <f>IF(D17="","",F17-MIN(F17,0.06*D17))</f>
+        <v/>
+      </c>
+      <c r="R17" s="18">
+        <f>IF(D17="","",G17-G17*H17)</f>
+        <v/>
+      </c>
+      <c r="S17" s="19">
+        <f>IF(D17="","",D17+E17+J17+K17+L17+M17+N17+O17+P17+Q17+R17+I17)</f>
         <v/>
       </c>
     </row>
@@ -1400,10 +1932,46 @@
       <c r="E18" s="13" t="n"/>
       <c r="F18" s="13" t="n"/>
       <c r="G18" s="13" t="n"/>
-      <c r="H18" s="16" t="n"/>
+      <c r="H18" s="17" t="n"/>
       <c r="I18" s="13" t="n"/>
-      <c r="J18" s="17">
-        <f>IF(D18="","",(D18+E18)+(D18+E18)*IF(UPPER(C18)="SIMPLES",0,0.2+$B$2+$D$2)+(D18+E18)*0.08+((D18+E18)/12+(D18+E18)*4/3/12)+((D18+E18)/12+(D18+E18)*4/3/12)*IF(UPPER(C18)="SIMPLES",0,0.2+$B$2+$D$2)+((D18+E18)/12+(D18+E18)*4/3/12)*0.08+0.4*0.08*((D18+E18)+((D18+E18)/12+(D18+E18)*4/3/12))+(F18-MIN(F18,0.06*D18))+(G18-G18*H18)+I18)</f>
+      <c r="J18" s="18">
+        <f>IF(D18="","",IF(UPPER(C18)="SIMPLES",0,0.2*((D18+E18)+(D18+E18)/12+(D18+E18)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="K18" s="18">
+        <f>IF(D18="","",IF(UPPER(C18)="SIMPLES",0,$B$2*((D18+E18)+(D18+E18)/12+(D18+E18)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="L18" s="18">
+        <f>IF(D18="","",IF(UPPER(C18)="SIMPLES",0,$D$2*((D18+E18)+(D18+E18)/12+(D18+E18)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="M18" s="18">
+        <f>IF(D18="","",0.08*((D18+E18)+(D18+E18)/12+(D18+E18)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="N18" s="18">
+        <f>IF(D18="","",(D18+E18)/12)</f>
+        <v/>
+      </c>
+      <c r="O18" s="18">
+        <f>IF(D18="","",(D18+E18)*4/3/12)</f>
+        <v/>
+      </c>
+      <c r="P18" s="18">
+        <f>IF(D18="","",0.4*0.08*((D18+E18)+(D18+E18)/12+(D18+E18)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="Q18" s="18">
+        <f>IF(D18="","",F18-MIN(F18,0.06*D18))</f>
+        <v/>
+      </c>
+      <c r="R18" s="18">
+        <f>IF(D18="","",G18-G18*H18)</f>
+        <v/>
+      </c>
+      <c r="S18" s="19">
+        <f>IF(D18="","",D18+E18+J18+K18+L18+M18+N18+O18+P18+Q18+R18+I18)</f>
         <v/>
       </c>
     </row>
@@ -1415,10 +1983,46 @@
       <c r="E19" s="13" t="n"/>
       <c r="F19" s="13" t="n"/>
       <c r="G19" s="13" t="n"/>
-      <c r="H19" s="16" t="n"/>
+      <c r="H19" s="17" t="n"/>
       <c r="I19" s="13" t="n"/>
-      <c r="J19" s="17">
-        <f>IF(D19="","",(D19+E19)+(D19+E19)*IF(UPPER(C19)="SIMPLES",0,0.2+$B$2+$D$2)+(D19+E19)*0.08+((D19+E19)/12+(D19+E19)*4/3/12)+((D19+E19)/12+(D19+E19)*4/3/12)*IF(UPPER(C19)="SIMPLES",0,0.2+$B$2+$D$2)+((D19+E19)/12+(D19+E19)*4/3/12)*0.08+0.4*0.08*((D19+E19)+((D19+E19)/12+(D19+E19)*4/3/12))+(F19-MIN(F19,0.06*D19))+(G19-G19*H19)+I19)</f>
+      <c r="J19" s="18">
+        <f>IF(D19="","",IF(UPPER(C19)="SIMPLES",0,0.2*((D19+E19)+(D19+E19)/12+(D19+E19)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="K19" s="18">
+        <f>IF(D19="","",IF(UPPER(C19)="SIMPLES",0,$B$2*((D19+E19)+(D19+E19)/12+(D19+E19)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="L19" s="18">
+        <f>IF(D19="","",IF(UPPER(C19)="SIMPLES",0,$D$2*((D19+E19)+(D19+E19)/12+(D19+E19)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="M19" s="18">
+        <f>IF(D19="","",0.08*((D19+E19)+(D19+E19)/12+(D19+E19)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="N19" s="18">
+        <f>IF(D19="","",(D19+E19)/12)</f>
+        <v/>
+      </c>
+      <c r="O19" s="18">
+        <f>IF(D19="","",(D19+E19)*4/3/12)</f>
+        <v/>
+      </c>
+      <c r="P19" s="18">
+        <f>IF(D19="","",0.4*0.08*((D19+E19)+(D19+E19)/12+(D19+E19)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="Q19" s="18">
+        <f>IF(D19="","",F19-MIN(F19,0.06*D19))</f>
+        <v/>
+      </c>
+      <c r="R19" s="18">
+        <f>IF(D19="","",G19-G19*H19)</f>
+        <v/>
+      </c>
+      <c r="S19" s="19">
+        <f>IF(D19="","",D19+E19+J19+K19+L19+M19+N19+O19+P19+Q19+R19+I19)</f>
         <v/>
       </c>
     </row>
@@ -1430,10 +2034,46 @@
       <c r="E20" s="13" t="n"/>
       <c r="F20" s="13" t="n"/>
       <c r="G20" s="13" t="n"/>
-      <c r="H20" s="16" t="n"/>
+      <c r="H20" s="17" t="n"/>
       <c r="I20" s="13" t="n"/>
-      <c r="J20" s="17">
-        <f>IF(D20="","",(D20+E20)+(D20+E20)*IF(UPPER(C20)="SIMPLES",0,0.2+$B$2+$D$2)+(D20+E20)*0.08+((D20+E20)/12+(D20+E20)*4/3/12)+((D20+E20)/12+(D20+E20)*4/3/12)*IF(UPPER(C20)="SIMPLES",0,0.2+$B$2+$D$2)+((D20+E20)/12+(D20+E20)*4/3/12)*0.08+0.4*0.08*((D20+E20)+((D20+E20)/12+(D20+E20)*4/3/12))+(F20-MIN(F20,0.06*D20))+(G20-G20*H20)+I20)</f>
+      <c r="J20" s="18">
+        <f>IF(D20="","",IF(UPPER(C20)="SIMPLES",0,0.2*((D20+E20)+(D20+E20)/12+(D20+E20)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="K20" s="18">
+        <f>IF(D20="","",IF(UPPER(C20)="SIMPLES",0,$B$2*((D20+E20)+(D20+E20)/12+(D20+E20)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="L20" s="18">
+        <f>IF(D20="","",IF(UPPER(C20)="SIMPLES",0,$D$2*((D20+E20)+(D20+E20)/12+(D20+E20)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="M20" s="18">
+        <f>IF(D20="","",0.08*((D20+E20)+(D20+E20)/12+(D20+E20)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="N20" s="18">
+        <f>IF(D20="","",(D20+E20)/12)</f>
+        <v/>
+      </c>
+      <c r="O20" s="18">
+        <f>IF(D20="","",(D20+E20)*4/3/12)</f>
+        <v/>
+      </c>
+      <c r="P20" s="18">
+        <f>IF(D20="","",0.4*0.08*((D20+E20)+(D20+E20)/12+(D20+E20)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="Q20" s="18">
+        <f>IF(D20="","",F20-MIN(F20,0.06*D20))</f>
+        <v/>
+      </c>
+      <c r="R20" s="18">
+        <f>IF(D20="","",G20-G20*H20)</f>
+        <v/>
+      </c>
+      <c r="S20" s="19">
+        <f>IF(D20="","",D20+E20+J20+K20+L20+M20+N20+O20+P20+Q20+R20+I20)</f>
         <v/>
       </c>
     </row>
@@ -1445,10 +2085,46 @@
       <c r="E21" s="13" t="n"/>
       <c r="F21" s="13" t="n"/>
       <c r="G21" s="13" t="n"/>
-      <c r="H21" s="16" t="n"/>
+      <c r="H21" s="17" t="n"/>
       <c r="I21" s="13" t="n"/>
-      <c r="J21" s="17">
-        <f>IF(D21="","",(D21+E21)+(D21+E21)*IF(UPPER(C21)="SIMPLES",0,0.2+$B$2+$D$2)+(D21+E21)*0.08+((D21+E21)/12+(D21+E21)*4/3/12)+((D21+E21)/12+(D21+E21)*4/3/12)*IF(UPPER(C21)="SIMPLES",0,0.2+$B$2+$D$2)+((D21+E21)/12+(D21+E21)*4/3/12)*0.08+0.4*0.08*((D21+E21)+((D21+E21)/12+(D21+E21)*4/3/12))+(F21-MIN(F21,0.06*D21))+(G21-G21*H21)+I21)</f>
+      <c r="J21" s="18">
+        <f>IF(D21="","",IF(UPPER(C21)="SIMPLES",0,0.2*((D21+E21)+(D21+E21)/12+(D21+E21)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="K21" s="18">
+        <f>IF(D21="","",IF(UPPER(C21)="SIMPLES",0,$B$2*((D21+E21)+(D21+E21)/12+(D21+E21)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="L21" s="18">
+        <f>IF(D21="","",IF(UPPER(C21)="SIMPLES",0,$D$2*((D21+E21)+(D21+E21)/12+(D21+E21)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="M21" s="18">
+        <f>IF(D21="","",0.08*((D21+E21)+(D21+E21)/12+(D21+E21)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="N21" s="18">
+        <f>IF(D21="","",(D21+E21)/12)</f>
+        <v/>
+      </c>
+      <c r="O21" s="18">
+        <f>IF(D21="","",(D21+E21)*4/3/12)</f>
+        <v/>
+      </c>
+      <c r="P21" s="18">
+        <f>IF(D21="","",0.4*0.08*((D21+E21)+(D21+E21)/12+(D21+E21)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="Q21" s="18">
+        <f>IF(D21="","",F21-MIN(F21,0.06*D21))</f>
+        <v/>
+      </c>
+      <c r="R21" s="18">
+        <f>IF(D21="","",G21-G21*H21)</f>
+        <v/>
+      </c>
+      <c r="S21" s="19">
+        <f>IF(D21="","",D21+E21+J21+K21+L21+M21+N21+O21+P21+Q21+R21+I21)</f>
         <v/>
       </c>
     </row>
@@ -1460,10 +2136,46 @@
       <c r="E22" s="13" t="n"/>
       <c r="F22" s="13" t="n"/>
       <c r="G22" s="13" t="n"/>
-      <c r="H22" s="16" t="n"/>
+      <c r="H22" s="17" t="n"/>
       <c r="I22" s="13" t="n"/>
-      <c r="J22" s="17">
-        <f>IF(D22="","",(D22+E22)+(D22+E22)*IF(UPPER(C22)="SIMPLES",0,0.2+$B$2+$D$2)+(D22+E22)*0.08+((D22+E22)/12+(D22+E22)*4/3/12)+((D22+E22)/12+(D22+E22)*4/3/12)*IF(UPPER(C22)="SIMPLES",0,0.2+$B$2+$D$2)+((D22+E22)/12+(D22+E22)*4/3/12)*0.08+0.4*0.08*((D22+E22)+((D22+E22)/12+(D22+E22)*4/3/12))+(F22-MIN(F22,0.06*D22))+(G22-G22*H22)+I22)</f>
+      <c r="J22" s="18">
+        <f>IF(D22="","",IF(UPPER(C22)="SIMPLES",0,0.2*((D22+E22)+(D22+E22)/12+(D22+E22)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="K22" s="18">
+        <f>IF(D22="","",IF(UPPER(C22)="SIMPLES",0,$B$2*((D22+E22)+(D22+E22)/12+(D22+E22)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="L22" s="18">
+        <f>IF(D22="","",IF(UPPER(C22)="SIMPLES",0,$D$2*((D22+E22)+(D22+E22)/12+(D22+E22)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="M22" s="18">
+        <f>IF(D22="","",0.08*((D22+E22)+(D22+E22)/12+(D22+E22)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="N22" s="18">
+        <f>IF(D22="","",(D22+E22)/12)</f>
+        <v/>
+      </c>
+      <c r="O22" s="18">
+        <f>IF(D22="","",(D22+E22)*4/3/12)</f>
+        <v/>
+      </c>
+      <c r="P22" s="18">
+        <f>IF(D22="","",0.4*0.08*((D22+E22)+(D22+E22)/12+(D22+E22)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="Q22" s="18">
+        <f>IF(D22="","",F22-MIN(F22,0.06*D22))</f>
+        <v/>
+      </c>
+      <c r="R22" s="18">
+        <f>IF(D22="","",G22-G22*H22)</f>
+        <v/>
+      </c>
+      <c r="S22" s="19">
+        <f>IF(D22="","",D22+E22+J22+K22+L22+M22+N22+O22+P22+Q22+R22+I22)</f>
         <v/>
       </c>
     </row>
@@ -1475,10 +2187,46 @@
       <c r="E23" s="13" t="n"/>
       <c r="F23" s="13" t="n"/>
       <c r="G23" s="13" t="n"/>
-      <c r="H23" s="16" t="n"/>
+      <c r="H23" s="17" t="n"/>
       <c r="I23" s="13" t="n"/>
-      <c r="J23" s="17">
-        <f>IF(D23="","",(D23+E23)+(D23+E23)*IF(UPPER(C23)="SIMPLES",0,0.2+$B$2+$D$2)+(D23+E23)*0.08+((D23+E23)/12+(D23+E23)*4/3/12)+((D23+E23)/12+(D23+E23)*4/3/12)*IF(UPPER(C23)="SIMPLES",0,0.2+$B$2+$D$2)+((D23+E23)/12+(D23+E23)*4/3/12)*0.08+0.4*0.08*((D23+E23)+((D23+E23)/12+(D23+E23)*4/3/12))+(F23-MIN(F23,0.06*D23))+(G23-G23*H23)+I23)</f>
+      <c r="J23" s="18">
+        <f>IF(D23="","",IF(UPPER(C23)="SIMPLES",0,0.2*((D23+E23)+(D23+E23)/12+(D23+E23)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="K23" s="18">
+        <f>IF(D23="","",IF(UPPER(C23)="SIMPLES",0,$B$2*((D23+E23)+(D23+E23)/12+(D23+E23)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="L23" s="18">
+        <f>IF(D23="","",IF(UPPER(C23)="SIMPLES",0,$D$2*((D23+E23)+(D23+E23)/12+(D23+E23)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="M23" s="18">
+        <f>IF(D23="","",0.08*((D23+E23)+(D23+E23)/12+(D23+E23)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="N23" s="18">
+        <f>IF(D23="","",(D23+E23)/12)</f>
+        <v/>
+      </c>
+      <c r="O23" s="18">
+        <f>IF(D23="","",(D23+E23)*4/3/12)</f>
+        <v/>
+      </c>
+      <c r="P23" s="18">
+        <f>IF(D23="","",0.4*0.08*((D23+E23)+(D23+E23)/12+(D23+E23)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="Q23" s="18">
+        <f>IF(D23="","",F23-MIN(F23,0.06*D23))</f>
+        <v/>
+      </c>
+      <c r="R23" s="18">
+        <f>IF(D23="","",G23-G23*H23)</f>
+        <v/>
+      </c>
+      <c r="S23" s="19">
+        <f>IF(D23="","",D23+E23+J23+K23+L23+M23+N23+O23+P23+Q23+R23+I23)</f>
         <v/>
       </c>
     </row>
@@ -1490,10 +2238,46 @@
       <c r="E24" s="13" t="n"/>
       <c r="F24" s="13" t="n"/>
       <c r="G24" s="13" t="n"/>
-      <c r="H24" s="16" t="n"/>
+      <c r="H24" s="17" t="n"/>
       <c r="I24" s="13" t="n"/>
-      <c r="J24" s="17">
-        <f>IF(D24="","",(D24+E24)+(D24+E24)*IF(UPPER(C24)="SIMPLES",0,0.2+$B$2+$D$2)+(D24+E24)*0.08+((D24+E24)/12+(D24+E24)*4/3/12)+((D24+E24)/12+(D24+E24)*4/3/12)*IF(UPPER(C24)="SIMPLES",0,0.2+$B$2+$D$2)+((D24+E24)/12+(D24+E24)*4/3/12)*0.08+0.4*0.08*((D24+E24)+((D24+E24)/12+(D24+E24)*4/3/12))+(F24-MIN(F24,0.06*D24))+(G24-G24*H24)+I24)</f>
+      <c r="J24" s="18">
+        <f>IF(D24="","",IF(UPPER(C24)="SIMPLES",0,0.2*((D24+E24)+(D24+E24)/12+(D24+E24)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="K24" s="18">
+        <f>IF(D24="","",IF(UPPER(C24)="SIMPLES",0,$B$2*((D24+E24)+(D24+E24)/12+(D24+E24)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="L24" s="18">
+        <f>IF(D24="","",IF(UPPER(C24)="SIMPLES",0,$D$2*((D24+E24)+(D24+E24)/12+(D24+E24)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="M24" s="18">
+        <f>IF(D24="","",0.08*((D24+E24)+(D24+E24)/12+(D24+E24)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="N24" s="18">
+        <f>IF(D24="","",(D24+E24)/12)</f>
+        <v/>
+      </c>
+      <c r="O24" s="18">
+        <f>IF(D24="","",(D24+E24)*4/3/12)</f>
+        <v/>
+      </c>
+      <c r="P24" s="18">
+        <f>IF(D24="","",0.4*0.08*((D24+E24)+(D24+E24)/12+(D24+E24)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="Q24" s="18">
+        <f>IF(D24="","",F24-MIN(F24,0.06*D24))</f>
+        <v/>
+      </c>
+      <c r="R24" s="18">
+        <f>IF(D24="","",G24-G24*H24)</f>
+        <v/>
+      </c>
+      <c r="S24" s="19">
+        <f>IF(D24="","",D24+E24+J24+K24+L24+M24+N24+O24+P24+Q24+R24+I24)</f>
         <v/>
       </c>
     </row>
@@ -1505,10 +2289,46 @@
       <c r="E25" s="13" t="n"/>
       <c r="F25" s="13" t="n"/>
       <c r="G25" s="13" t="n"/>
-      <c r="H25" s="16" t="n"/>
+      <c r="H25" s="17" t="n"/>
       <c r="I25" s="13" t="n"/>
-      <c r="J25" s="17">
-        <f>IF(D25="","",(D25+E25)+(D25+E25)*IF(UPPER(C25)="SIMPLES",0,0.2+$B$2+$D$2)+(D25+E25)*0.08+((D25+E25)/12+(D25+E25)*4/3/12)+((D25+E25)/12+(D25+E25)*4/3/12)*IF(UPPER(C25)="SIMPLES",0,0.2+$B$2+$D$2)+((D25+E25)/12+(D25+E25)*4/3/12)*0.08+0.4*0.08*((D25+E25)+((D25+E25)/12+(D25+E25)*4/3/12))+(F25-MIN(F25,0.06*D25))+(G25-G25*H25)+I25)</f>
+      <c r="J25" s="18">
+        <f>IF(D25="","",IF(UPPER(C25)="SIMPLES",0,0.2*((D25+E25)+(D25+E25)/12+(D25+E25)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="K25" s="18">
+        <f>IF(D25="","",IF(UPPER(C25)="SIMPLES",0,$B$2*((D25+E25)+(D25+E25)/12+(D25+E25)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="L25" s="18">
+        <f>IF(D25="","",IF(UPPER(C25)="SIMPLES",0,$D$2*((D25+E25)+(D25+E25)/12+(D25+E25)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="M25" s="18">
+        <f>IF(D25="","",0.08*((D25+E25)+(D25+E25)/12+(D25+E25)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="N25" s="18">
+        <f>IF(D25="","",(D25+E25)/12)</f>
+        <v/>
+      </c>
+      <c r="O25" s="18">
+        <f>IF(D25="","",(D25+E25)*4/3/12)</f>
+        <v/>
+      </c>
+      <c r="P25" s="18">
+        <f>IF(D25="","",0.4*0.08*((D25+E25)+(D25+E25)/12+(D25+E25)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="Q25" s="18">
+        <f>IF(D25="","",F25-MIN(F25,0.06*D25))</f>
+        <v/>
+      </c>
+      <c r="R25" s="18">
+        <f>IF(D25="","",G25-G25*H25)</f>
+        <v/>
+      </c>
+      <c r="S25" s="19">
+        <f>IF(D25="","",D25+E25+J25+K25+L25+M25+N25+O25+P25+Q25+R25+I25)</f>
         <v/>
       </c>
     </row>
@@ -1520,10 +2340,46 @@
       <c r="E26" s="13" t="n"/>
       <c r="F26" s="13" t="n"/>
       <c r="G26" s="13" t="n"/>
-      <c r="H26" s="16" t="n"/>
+      <c r="H26" s="17" t="n"/>
       <c r="I26" s="13" t="n"/>
-      <c r="J26" s="17">
-        <f>IF(D26="","",(D26+E26)+(D26+E26)*IF(UPPER(C26)="SIMPLES",0,0.2+$B$2+$D$2)+(D26+E26)*0.08+((D26+E26)/12+(D26+E26)*4/3/12)+((D26+E26)/12+(D26+E26)*4/3/12)*IF(UPPER(C26)="SIMPLES",0,0.2+$B$2+$D$2)+((D26+E26)/12+(D26+E26)*4/3/12)*0.08+0.4*0.08*((D26+E26)+((D26+E26)/12+(D26+E26)*4/3/12))+(F26-MIN(F26,0.06*D26))+(G26-G26*H26)+I26)</f>
+      <c r="J26" s="18">
+        <f>IF(D26="","",IF(UPPER(C26)="SIMPLES",0,0.2*((D26+E26)+(D26+E26)/12+(D26+E26)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="K26" s="18">
+        <f>IF(D26="","",IF(UPPER(C26)="SIMPLES",0,$B$2*((D26+E26)+(D26+E26)/12+(D26+E26)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="L26" s="18">
+        <f>IF(D26="","",IF(UPPER(C26)="SIMPLES",0,$D$2*((D26+E26)+(D26+E26)/12+(D26+E26)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="M26" s="18">
+        <f>IF(D26="","",0.08*((D26+E26)+(D26+E26)/12+(D26+E26)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="N26" s="18">
+        <f>IF(D26="","",(D26+E26)/12)</f>
+        <v/>
+      </c>
+      <c r="O26" s="18">
+        <f>IF(D26="","",(D26+E26)*4/3/12)</f>
+        <v/>
+      </c>
+      <c r="P26" s="18">
+        <f>IF(D26="","",0.4*0.08*((D26+E26)+(D26+E26)/12+(D26+E26)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="Q26" s="18">
+        <f>IF(D26="","",F26-MIN(F26,0.06*D26))</f>
+        <v/>
+      </c>
+      <c r="R26" s="18">
+        <f>IF(D26="","",G26-G26*H26)</f>
+        <v/>
+      </c>
+      <c r="S26" s="19">
+        <f>IF(D26="","",D26+E26+J26+K26+L26+M26+N26+O26+P26+Q26+R26+I26)</f>
         <v/>
       </c>
     </row>
@@ -1535,10 +2391,46 @@
       <c r="E27" s="13" t="n"/>
       <c r="F27" s="13" t="n"/>
       <c r="G27" s="13" t="n"/>
-      <c r="H27" s="16" t="n"/>
+      <c r="H27" s="17" t="n"/>
       <c r="I27" s="13" t="n"/>
-      <c r="J27" s="17">
-        <f>IF(D27="","",(D27+E27)+(D27+E27)*IF(UPPER(C27)="SIMPLES",0,0.2+$B$2+$D$2)+(D27+E27)*0.08+((D27+E27)/12+(D27+E27)*4/3/12)+((D27+E27)/12+(D27+E27)*4/3/12)*IF(UPPER(C27)="SIMPLES",0,0.2+$B$2+$D$2)+((D27+E27)/12+(D27+E27)*4/3/12)*0.08+0.4*0.08*((D27+E27)+((D27+E27)/12+(D27+E27)*4/3/12))+(F27-MIN(F27,0.06*D27))+(G27-G27*H27)+I27)</f>
+      <c r="J27" s="18">
+        <f>IF(D27="","",IF(UPPER(C27)="SIMPLES",0,0.2*((D27+E27)+(D27+E27)/12+(D27+E27)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="K27" s="18">
+        <f>IF(D27="","",IF(UPPER(C27)="SIMPLES",0,$B$2*((D27+E27)+(D27+E27)/12+(D27+E27)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="L27" s="18">
+        <f>IF(D27="","",IF(UPPER(C27)="SIMPLES",0,$D$2*((D27+E27)+(D27+E27)/12+(D27+E27)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="M27" s="18">
+        <f>IF(D27="","",0.08*((D27+E27)+(D27+E27)/12+(D27+E27)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="N27" s="18">
+        <f>IF(D27="","",(D27+E27)/12)</f>
+        <v/>
+      </c>
+      <c r="O27" s="18">
+        <f>IF(D27="","",(D27+E27)*4/3/12)</f>
+        <v/>
+      </c>
+      <c r="P27" s="18">
+        <f>IF(D27="","",0.4*0.08*((D27+E27)+(D27+E27)/12+(D27+E27)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="Q27" s="18">
+        <f>IF(D27="","",F27-MIN(F27,0.06*D27))</f>
+        <v/>
+      </c>
+      <c r="R27" s="18">
+        <f>IF(D27="","",G27-G27*H27)</f>
+        <v/>
+      </c>
+      <c r="S27" s="19">
+        <f>IF(D27="","",D27+E27+J27+K27+L27+M27+N27+O27+P27+Q27+R27+I27)</f>
         <v/>
       </c>
     </row>
@@ -1550,10 +2442,46 @@
       <c r="E28" s="13" t="n"/>
       <c r="F28" s="13" t="n"/>
       <c r="G28" s="13" t="n"/>
-      <c r="H28" s="16" t="n"/>
+      <c r="H28" s="17" t="n"/>
       <c r="I28" s="13" t="n"/>
-      <c r="J28" s="17">
-        <f>IF(D28="","",(D28+E28)+(D28+E28)*IF(UPPER(C28)="SIMPLES",0,0.2+$B$2+$D$2)+(D28+E28)*0.08+((D28+E28)/12+(D28+E28)*4/3/12)+((D28+E28)/12+(D28+E28)*4/3/12)*IF(UPPER(C28)="SIMPLES",0,0.2+$B$2+$D$2)+((D28+E28)/12+(D28+E28)*4/3/12)*0.08+0.4*0.08*((D28+E28)+((D28+E28)/12+(D28+E28)*4/3/12))+(F28-MIN(F28,0.06*D28))+(G28-G28*H28)+I28)</f>
+      <c r="J28" s="18">
+        <f>IF(D28="","",IF(UPPER(C28)="SIMPLES",0,0.2*((D28+E28)+(D28+E28)/12+(D28+E28)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="K28" s="18">
+        <f>IF(D28="","",IF(UPPER(C28)="SIMPLES",0,$B$2*((D28+E28)+(D28+E28)/12+(D28+E28)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="L28" s="18">
+        <f>IF(D28="","",IF(UPPER(C28)="SIMPLES",0,$D$2*((D28+E28)+(D28+E28)/12+(D28+E28)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="M28" s="18">
+        <f>IF(D28="","",0.08*((D28+E28)+(D28+E28)/12+(D28+E28)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="N28" s="18">
+        <f>IF(D28="","",(D28+E28)/12)</f>
+        <v/>
+      </c>
+      <c r="O28" s="18">
+        <f>IF(D28="","",(D28+E28)*4/3/12)</f>
+        <v/>
+      </c>
+      <c r="P28" s="18">
+        <f>IF(D28="","",0.4*0.08*((D28+E28)+(D28+E28)/12+(D28+E28)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="Q28" s="18">
+        <f>IF(D28="","",F28-MIN(F28,0.06*D28))</f>
+        <v/>
+      </c>
+      <c r="R28" s="18">
+        <f>IF(D28="","",G28-G28*H28)</f>
+        <v/>
+      </c>
+      <c r="S28" s="19">
+        <f>IF(D28="","",D28+E28+J28+K28+L28+M28+N28+O28+P28+Q28+R28+I28)</f>
         <v/>
       </c>
     </row>
@@ -1565,10 +2493,46 @@
       <c r="E29" s="13" t="n"/>
       <c r="F29" s="13" t="n"/>
       <c r="G29" s="13" t="n"/>
-      <c r="H29" s="16" t="n"/>
+      <c r="H29" s="17" t="n"/>
       <c r="I29" s="13" t="n"/>
-      <c r="J29" s="17">
-        <f>IF(D29="","",(D29+E29)+(D29+E29)*IF(UPPER(C29)="SIMPLES",0,0.2+$B$2+$D$2)+(D29+E29)*0.08+((D29+E29)/12+(D29+E29)*4/3/12)+((D29+E29)/12+(D29+E29)*4/3/12)*IF(UPPER(C29)="SIMPLES",0,0.2+$B$2+$D$2)+((D29+E29)/12+(D29+E29)*4/3/12)*0.08+0.4*0.08*((D29+E29)+((D29+E29)/12+(D29+E29)*4/3/12))+(F29-MIN(F29,0.06*D29))+(G29-G29*H29)+I29)</f>
+      <c r="J29" s="18">
+        <f>IF(D29="","",IF(UPPER(C29)="SIMPLES",0,0.2*((D29+E29)+(D29+E29)/12+(D29+E29)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="K29" s="18">
+        <f>IF(D29="","",IF(UPPER(C29)="SIMPLES",0,$B$2*((D29+E29)+(D29+E29)/12+(D29+E29)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="L29" s="18">
+        <f>IF(D29="","",IF(UPPER(C29)="SIMPLES",0,$D$2*((D29+E29)+(D29+E29)/12+(D29+E29)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="M29" s="18">
+        <f>IF(D29="","",0.08*((D29+E29)+(D29+E29)/12+(D29+E29)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="N29" s="18">
+        <f>IF(D29="","",(D29+E29)/12)</f>
+        <v/>
+      </c>
+      <c r="O29" s="18">
+        <f>IF(D29="","",(D29+E29)*4/3/12)</f>
+        <v/>
+      </c>
+      <c r="P29" s="18">
+        <f>IF(D29="","",0.4*0.08*((D29+E29)+(D29+E29)/12+(D29+E29)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="Q29" s="18">
+        <f>IF(D29="","",F29-MIN(F29,0.06*D29))</f>
+        <v/>
+      </c>
+      <c r="R29" s="18">
+        <f>IF(D29="","",G29-G29*H29)</f>
+        <v/>
+      </c>
+      <c r="S29" s="19">
+        <f>IF(D29="","",D29+E29+J29+K29+L29+M29+N29+O29+P29+Q29+R29+I29)</f>
         <v/>
       </c>
     </row>
@@ -1580,10 +2544,46 @@
       <c r="E30" s="13" t="n"/>
       <c r="F30" s="13" t="n"/>
       <c r="G30" s="13" t="n"/>
-      <c r="H30" s="16" t="n"/>
+      <c r="H30" s="17" t="n"/>
       <c r="I30" s="13" t="n"/>
-      <c r="J30" s="17">
-        <f>IF(D30="","",(D30+E30)+(D30+E30)*IF(UPPER(C30)="SIMPLES",0,0.2+$B$2+$D$2)+(D30+E30)*0.08+((D30+E30)/12+(D30+E30)*4/3/12)+((D30+E30)/12+(D30+E30)*4/3/12)*IF(UPPER(C30)="SIMPLES",0,0.2+$B$2+$D$2)+((D30+E30)/12+(D30+E30)*4/3/12)*0.08+0.4*0.08*((D30+E30)+((D30+E30)/12+(D30+E30)*4/3/12))+(F30-MIN(F30,0.06*D30))+(G30-G30*H30)+I30)</f>
+      <c r="J30" s="18">
+        <f>IF(D30="","",IF(UPPER(C30)="SIMPLES",0,0.2*((D30+E30)+(D30+E30)/12+(D30+E30)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="K30" s="18">
+        <f>IF(D30="","",IF(UPPER(C30)="SIMPLES",0,$B$2*((D30+E30)+(D30+E30)/12+(D30+E30)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="L30" s="18">
+        <f>IF(D30="","",IF(UPPER(C30)="SIMPLES",0,$D$2*((D30+E30)+(D30+E30)/12+(D30+E30)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="M30" s="18">
+        <f>IF(D30="","",0.08*((D30+E30)+(D30+E30)/12+(D30+E30)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="N30" s="18">
+        <f>IF(D30="","",(D30+E30)/12)</f>
+        <v/>
+      </c>
+      <c r="O30" s="18">
+        <f>IF(D30="","",(D30+E30)*4/3/12)</f>
+        <v/>
+      </c>
+      <c r="P30" s="18">
+        <f>IF(D30="","",0.4*0.08*((D30+E30)+(D30+E30)/12+(D30+E30)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="Q30" s="18">
+        <f>IF(D30="","",F30-MIN(F30,0.06*D30))</f>
+        <v/>
+      </c>
+      <c r="R30" s="18">
+        <f>IF(D30="","",G30-G30*H30)</f>
+        <v/>
+      </c>
+      <c r="S30" s="19">
+        <f>IF(D30="","",D30+E30+J30+K30+L30+M30+N30+O30+P30+Q30+R30+I30)</f>
         <v/>
       </c>
     </row>
@@ -1595,10 +2595,46 @@
       <c r="E31" s="13" t="n"/>
       <c r="F31" s="13" t="n"/>
       <c r="G31" s="13" t="n"/>
-      <c r="H31" s="16" t="n"/>
+      <c r="H31" s="17" t="n"/>
       <c r="I31" s="13" t="n"/>
-      <c r="J31" s="17">
-        <f>IF(D31="","",(D31+E31)+(D31+E31)*IF(UPPER(C31)="SIMPLES",0,0.2+$B$2+$D$2)+(D31+E31)*0.08+((D31+E31)/12+(D31+E31)*4/3/12)+((D31+E31)/12+(D31+E31)*4/3/12)*IF(UPPER(C31)="SIMPLES",0,0.2+$B$2+$D$2)+((D31+E31)/12+(D31+E31)*4/3/12)*0.08+0.4*0.08*((D31+E31)+((D31+E31)/12+(D31+E31)*4/3/12))+(F31-MIN(F31,0.06*D31))+(G31-G31*H31)+I31)</f>
+      <c r="J31" s="18">
+        <f>IF(D31="","",IF(UPPER(C31)="SIMPLES",0,0.2*((D31+E31)+(D31+E31)/12+(D31+E31)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="K31" s="18">
+        <f>IF(D31="","",IF(UPPER(C31)="SIMPLES",0,$B$2*((D31+E31)+(D31+E31)/12+(D31+E31)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="L31" s="18">
+        <f>IF(D31="","",IF(UPPER(C31)="SIMPLES",0,$D$2*((D31+E31)+(D31+E31)/12+(D31+E31)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="M31" s="18">
+        <f>IF(D31="","",0.08*((D31+E31)+(D31+E31)/12+(D31+E31)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="N31" s="18">
+        <f>IF(D31="","",(D31+E31)/12)</f>
+        <v/>
+      </c>
+      <c r="O31" s="18">
+        <f>IF(D31="","",(D31+E31)*4/3/12)</f>
+        <v/>
+      </c>
+      <c r="P31" s="18">
+        <f>IF(D31="","",0.4*0.08*((D31+E31)+(D31+E31)/12+(D31+E31)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="Q31" s="18">
+        <f>IF(D31="","",F31-MIN(F31,0.06*D31))</f>
+        <v/>
+      </c>
+      <c r="R31" s="18">
+        <f>IF(D31="","",G31-G31*H31)</f>
+        <v/>
+      </c>
+      <c r="S31" s="19">
+        <f>IF(D31="","",D31+E31+J31+K31+L31+M31+N31+O31+P31+Q31+R31+I31)</f>
         <v/>
       </c>
     </row>
@@ -1610,10 +2646,46 @@
       <c r="E32" s="13" t="n"/>
       <c r="F32" s="13" t="n"/>
       <c r="G32" s="13" t="n"/>
-      <c r="H32" s="16" t="n"/>
+      <c r="H32" s="17" t="n"/>
       <c r="I32" s="13" t="n"/>
-      <c r="J32" s="17">
-        <f>IF(D32="","",(D32+E32)+(D32+E32)*IF(UPPER(C32)="SIMPLES",0,0.2+$B$2+$D$2)+(D32+E32)*0.08+((D32+E32)/12+(D32+E32)*4/3/12)+((D32+E32)/12+(D32+E32)*4/3/12)*IF(UPPER(C32)="SIMPLES",0,0.2+$B$2+$D$2)+((D32+E32)/12+(D32+E32)*4/3/12)*0.08+0.4*0.08*((D32+E32)+((D32+E32)/12+(D32+E32)*4/3/12))+(F32-MIN(F32,0.06*D32))+(G32-G32*H32)+I32)</f>
+      <c r="J32" s="18">
+        <f>IF(D32="","",IF(UPPER(C32)="SIMPLES",0,0.2*((D32+E32)+(D32+E32)/12+(D32+E32)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="K32" s="18">
+        <f>IF(D32="","",IF(UPPER(C32)="SIMPLES",0,$B$2*((D32+E32)+(D32+E32)/12+(D32+E32)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="L32" s="18">
+        <f>IF(D32="","",IF(UPPER(C32)="SIMPLES",0,$D$2*((D32+E32)+(D32+E32)/12+(D32+E32)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="M32" s="18">
+        <f>IF(D32="","",0.08*((D32+E32)+(D32+E32)/12+(D32+E32)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="N32" s="18">
+        <f>IF(D32="","",(D32+E32)/12)</f>
+        <v/>
+      </c>
+      <c r="O32" s="18">
+        <f>IF(D32="","",(D32+E32)*4/3/12)</f>
+        <v/>
+      </c>
+      <c r="P32" s="18">
+        <f>IF(D32="","",0.4*0.08*((D32+E32)+(D32+E32)/12+(D32+E32)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="Q32" s="18">
+        <f>IF(D32="","",F32-MIN(F32,0.06*D32))</f>
+        <v/>
+      </c>
+      <c r="R32" s="18">
+        <f>IF(D32="","",G32-G32*H32)</f>
+        <v/>
+      </c>
+      <c r="S32" s="19">
+        <f>IF(D32="","",D32+E32+J32+K32+L32+M32+N32+O32+P32+Q32+R32+I32)</f>
         <v/>
       </c>
     </row>
@@ -1625,10 +2697,46 @@
       <c r="E33" s="13" t="n"/>
       <c r="F33" s="13" t="n"/>
       <c r="G33" s="13" t="n"/>
-      <c r="H33" s="16" t="n"/>
+      <c r="H33" s="17" t="n"/>
       <c r="I33" s="13" t="n"/>
-      <c r="J33" s="17">
-        <f>IF(D33="","",(D33+E33)+(D33+E33)*IF(UPPER(C33)="SIMPLES",0,0.2+$B$2+$D$2)+(D33+E33)*0.08+((D33+E33)/12+(D33+E33)*4/3/12)+((D33+E33)/12+(D33+E33)*4/3/12)*IF(UPPER(C33)="SIMPLES",0,0.2+$B$2+$D$2)+((D33+E33)/12+(D33+E33)*4/3/12)*0.08+0.4*0.08*((D33+E33)+((D33+E33)/12+(D33+E33)*4/3/12))+(F33-MIN(F33,0.06*D33))+(G33-G33*H33)+I33)</f>
+      <c r="J33" s="18">
+        <f>IF(D33="","",IF(UPPER(C33)="SIMPLES",0,0.2*((D33+E33)+(D33+E33)/12+(D33+E33)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="K33" s="18">
+        <f>IF(D33="","",IF(UPPER(C33)="SIMPLES",0,$B$2*((D33+E33)+(D33+E33)/12+(D33+E33)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="L33" s="18">
+        <f>IF(D33="","",IF(UPPER(C33)="SIMPLES",0,$D$2*((D33+E33)+(D33+E33)/12+(D33+E33)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="M33" s="18">
+        <f>IF(D33="","",0.08*((D33+E33)+(D33+E33)/12+(D33+E33)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="N33" s="18">
+        <f>IF(D33="","",(D33+E33)/12)</f>
+        <v/>
+      </c>
+      <c r="O33" s="18">
+        <f>IF(D33="","",(D33+E33)*4/3/12)</f>
+        <v/>
+      </c>
+      <c r="P33" s="18">
+        <f>IF(D33="","",0.4*0.08*((D33+E33)+(D33+E33)/12+(D33+E33)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="Q33" s="18">
+        <f>IF(D33="","",F33-MIN(F33,0.06*D33))</f>
+        <v/>
+      </c>
+      <c r="R33" s="18">
+        <f>IF(D33="","",G33-G33*H33)</f>
+        <v/>
+      </c>
+      <c r="S33" s="19">
+        <f>IF(D33="","",D33+E33+J33+K33+L33+M33+N33+O33+P33+Q33+R33+I33)</f>
         <v/>
       </c>
     </row>
@@ -1640,36 +2748,112 @@
       <c r="E34" s="13" t="n"/>
       <c r="F34" s="13" t="n"/>
       <c r="G34" s="13" t="n"/>
-      <c r="H34" s="16" t="n"/>
+      <c r="H34" s="17" t="n"/>
       <c r="I34" s="13" t="n"/>
-      <c r="J34" s="17">
-        <f>IF(D34="","",(D34+E34)+(D34+E34)*IF(UPPER(C34)="SIMPLES",0,0.2+$B$2+$D$2)+(D34+E34)*0.08+((D34+E34)/12+(D34+E34)*4/3/12)+((D34+E34)/12+(D34+E34)*4/3/12)*IF(UPPER(C34)="SIMPLES",0,0.2+$B$2+$D$2)+((D34+E34)/12+(D34+E34)*4/3/12)*0.08+0.4*0.08*((D34+E34)+((D34+E34)/12+(D34+E34)*4/3/12))+(F34-MIN(F34,0.06*D34))+(G34-G34*H34)+I34)</f>
+      <c r="J34" s="18">
+        <f>IF(D34="","",IF(UPPER(C34)="SIMPLES",0,0.2*((D34+E34)+(D34+E34)/12+(D34+E34)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="K34" s="18">
+        <f>IF(D34="","",IF(UPPER(C34)="SIMPLES",0,$B$2*((D34+E34)+(D34+E34)/12+(D34+E34)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="L34" s="18">
+        <f>IF(D34="","",IF(UPPER(C34)="SIMPLES",0,$D$2*((D34+E34)+(D34+E34)/12+(D34+E34)*4/3/12)))</f>
+        <v/>
+      </c>
+      <c r="M34" s="18">
+        <f>IF(D34="","",0.08*((D34+E34)+(D34+E34)/12+(D34+E34)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="N34" s="18">
+        <f>IF(D34="","",(D34+E34)/12)</f>
+        <v/>
+      </c>
+      <c r="O34" s="18">
+        <f>IF(D34="","",(D34+E34)*4/3/12)</f>
+        <v/>
+      </c>
+      <c r="P34" s="18">
+        <f>IF(D34="","",0.4*0.08*((D34+E34)+(D34+E34)/12+(D34+E34)*4/3/12))</f>
+        <v/>
+      </c>
+      <c r="Q34" s="18">
+        <f>IF(D34="","",F34-MIN(F34,0.06*D34))</f>
+        <v/>
+      </c>
+      <c r="R34" s="18">
+        <f>IF(D34="","",G34-G34*H34)</f>
+        <v/>
+      </c>
+      <c r="S34" s="19">
+        <f>IF(D34="","",D34+E34+J34+K34+L34+M34+N34+O34+P34+Q34+R34+I34)</f>
         <v/>
       </c>
     </row>
     <row r="35">
+      <c r="B35" s="10" t="inlineStr"/>
       <c r="C35" s="10" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="D35" s="18">
+      <c r="D35" s="20">
         <f>COUNT(D5:D34)</f>
         <v/>
       </c>
-      <c r="I35" s="19" t="inlineStr">
-        <is>
-          <t>Funcionários:</t>
-        </is>
-      </c>
-      <c r="J35" s="20">
+      <c r="E35" s="21">
+        <f>SUM(E5:E34)</f>
+        <v/>
+      </c>
+      <c r="I35" s="21">
+        <f>SUM(I5:I34)</f>
+        <v/>
+      </c>
+      <c r="J35" s="21">
         <f>SUM(J5:J34)</f>
+        <v/>
+      </c>
+      <c r="K35" s="21">
+        <f>SUM(K5:K34)</f>
+        <v/>
+      </c>
+      <c r="L35" s="21">
+        <f>SUM(L5:L34)</f>
+        <v/>
+      </c>
+      <c r="M35" s="21">
+        <f>SUM(M5:M34)</f>
+        <v/>
+      </c>
+      <c r="N35" s="21">
+        <f>SUM(N5:N34)</f>
+        <v/>
+      </c>
+      <c r="O35" s="21">
+        <f>SUM(O5:O34)</f>
+        <v/>
+      </c>
+      <c r="P35" s="21">
+        <f>SUM(P5:P34)</f>
+        <v/>
+      </c>
+      <c r="Q35" s="21">
+        <f>SUM(Q5:Q34)</f>
+        <v/>
+      </c>
+      <c r="R35" s="21">
+        <f>SUM(R5:R34)</f>
+        <v/>
+      </c>
+      <c r="S35" s="21">
+        <f>SUM(S5:S34)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A1:S1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1725,12 +2909,12 @@
           <t>Vendedor</t>
         </is>
       </c>
-      <c r="B4" s="21">
+      <c r="B4" s="22">
         <f>IF(A4="","",COUNTIF('Funcionários'!$A$5:$A$34,A4))</f>
         <v/>
       </c>
       <c r="C4" s="13">
-        <f>IF(A4="","",SUMIF('Funcionários'!$A$5:$A$34,A4,'Funcionários'!$J$5:$J$34))</f>
+        <f>IF(A4="","",SUMIF('Funcionários'!$A$5:$A$34,A4,'Funcionários'!$S$5:$S$34))</f>
         <v/>
       </c>
       <c r="D4" s="13">
@@ -1744,12 +2928,12 @@
           <t>Gerente</t>
         </is>
       </c>
-      <c r="B5" s="21">
+      <c r="B5" s="22">
         <f>IF(A5="","",COUNTIF('Funcionários'!$A$5:$A$34,A5))</f>
         <v/>
       </c>
       <c r="C5" s="13">
-        <f>IF(A5="","",SUMIF('Funcionários'!$A$5:$A$34,A5,'Funcionários'!$J$5:$J$34))</f>
+        <f>IF(A5="","",SUMIF('Funcionários'!$A$5:$A$34,A5,'Funcionários'!$S$5:$S$34))</f>
         <v/>
       </c>
       <c r="D5" s="13">
@@ -1759,12 +2943,12 @@
     </row>
     <row r="6">
       <c r="A6" s="12" t="n"/>
-      <c r="B6" s="21">
+      <c r="B6" s="22">
         <f>IF(A6="","",COUNTIF('Funcionários'!$A$5:$A$34,A6))</f>
         <v/>
       </c>
       <c r="C6" s="13">
-        <f>IF(A6="","",SUMIF('Funcionários'!$A$5:$A$34,A6,'Funcionários'!$J$5:$J$34))</f>
+        <f>IF(A6="","",SUMIF('Funcionários'!$A$5:$A$34,A6,'Funcionários'!$S$5:$S$34))</f>
         <v/>
       </c>
       <c r="D6" s="13">
@@ -1774,12 +2958,12 @@
     </row>
     <row r="7">
       <c r="A7" s="12" t="n"/>
-      <c r="B7" s="21">
+      <c r="B7" s="22">
         <f>IF(A7="","",COUNTIF('Funcionários'!$A$5:$A$34,A7))</f>
         <v/>
       </c>
       <c r="C7" s="13">
-        <f>IF(A7="","",SUMIF('Funcionários'!$A$5:$A$34,A7,'Funcionários'!$J$5:$J$34))</f>
+        <f>IF(A7="","",SUMIF('Funcionários'!$A$5:$A$34,A7,'Funcionários'!$S$5:$S$34))</f>
         <v/>
       </c>
       <c r="D7" s="13">
@@ -1789,12 +2973,12 @@
     </row>
     <row r="8">
       <c r="A8" s="12" t="n"/>
-      <c r="B8" s="21">
+      <c r="B8" s="22">
         <f>IF(A8="","",COUNTIF('Funcionários'!$A$5:$A$34,A8))</f>
         <v/>
       </c>
       <c r="C8" s="13">
-        <f>IF(A8="","",SUMIF('Funcionários'!$A$5:$A$34,A8,'Funcionários'!$J$5:$J$34))</f>
+        <f>IF(A8="","",SUMIF('Funcionários'!$A$5:$A$34,A8,'Funcionários'!$S$5:$S$34))</f>
         <v/>
       </c>
       <c r="D8" s="13">
@@ -1804,12 +2988,12 @@
     </row>
     <row r="9">
       <c r="A9" s="12" t="n"/>
-      <c r="B9" s="21">
+      <c r="B9" s="22">
         <f>IF(A9="","",COUNTIF('Funcionários'!$A$5:$A$34,A9))</f>
         <v/>
       </c>
       <c r="C9" s="13">
-        <f>IF(A9="","",SUMIF('Funcionários'!$A$5:$A$34,A9,'Funcionários'!$J$5:$J$34))</f>
+        <f>IF(A9="","",SUMIF('Funcionários'!$A$5:$A$34,A9,'Funcionários'!$S$5:$S$34))</f>
         <v/>
       </c>
       <c r="D9" s="13">
@@ -1819,12 +3003,12 @@
     </row>
     <row r="10">
       <c r="A10" s="12" t="n"/>
-      <c r="B10" s="21">
+      <c r="B10" s="22">
         <f>IF(A10="","",COUNTIF('Funcionários'!$A$5:$A$34,A10))</f>
         <v/>
       </c>
       <c r="C10" s="13">
-        <f>IF(A10="","",SUMIF('Funcionários'!$A$5:$A$34,A10,'Funcionários'!$J$5:$J$34))</f>
+        <f>IF(A10="","",SUMIF('Funcionários'!$A$5:$A$34,A10,'Funcionários'!$S$5:$S$34))</f>
         <v/>
       </c>
       <c r="D10" s="13">
@@ -1834,12 +3018,12 @@
     </row>
     <row r="11">
       <c r="A11" s="12" t="n"/>
-      <c r="B11" s="21">
+      <c r="B11" s="22">
         <f>IF(A11="","",COUNTIF('Funcionários'!$A$5:$A$34,A11))</f>
         <v/>
       </c>
       <c r="C11" s="13">
-        <f>IF(A11="","",SUMIF('Funcionários'!$A$5:$A$34,A11,'Funcionários'!$J$5:$J$34))</f>
+        <f>IF(A11="","",SUMIF('Funcionários'!$A$5:$A$34,A11,'Funcionários'!$S$5:$S$34))</f>
         <v/>
       </c>
       <c r="D11" s="13">
@@ -1849,12 +3033,12 @@
     </row>
     <row r="12">
       <c r="A12" s="12" t="n"/>
-      <c r="B12" s="21">
+      <c r="B12" s="22">
         <f>IF(A12="","",COUNTIF('Funcionários'!$A$5:$A$34,A12))</f>
         <v/>
       </c>
       <c r="C12" s="13">
-        <f>IF(A12="","",SUMIF('Funcionários'!$A$5:$A$34,A12,'Funcionários'!$J$5:$J$34))</f>
+        <f>IF(A12="","",SUMIF('Funcionários'!$A$5:$A$34,A12,'Funcionários'!$S$5:$S$34))</f>
         <v/>
       </c>
       <c r="D12" s="13">
@@ -1864,12 +3048,12 @@
     </row>
     <row r="13">
       <c r="A13" s="12" t="n"/>
-      <c r="B13" s="21">
+      <c r="B13" s="22">
         <f>IF(A13="","",COUNTIF('Funcionários'!$A$5:$A$34,A13))</f>
         <v/>
       </c>
       <c r="C13" s="13">
-        <f>IF(A13="","",SUMIF('Funcionários'!$A$5:$A$34,A13,'Funcionários'!$J$5:$J$34))</f>
+        <f>IF(A13="","",SUMIF('Funcionários'!$A$5:$A$34,A13,'Funcionários'!$S$5:$S$34))</f>
         <v/>
       </c>
       <c r="D13" s="13">
@@ -1879,12 +3063,12 @@
     </row>
     <row r="14">
       <c r="A14" s="12" t="n"/>
-      <c r="B14" s="21">
+      <c r="B14" s="22">
         <f>IF(A14="","",COUNTIF('Funcionários'!$A$5:$A$34,A14))</f>
         <v/>
       </c>
       <c r="C14" s="13">
-        <f>IF(A14="","",SUMIF('Funcionários'!$A$5:$A$34,A14,'Funcionários'!$J$5:$J$34))</f>
+        <f>IF(A14="","",SUMIF('Funcionários'!$A$5:$A$34,A14,'Funcionários'!$S$5:$S$34))</f>
         <v/>
       </c>
       <c r="D14" s="13">
@@ -1894,12 +3078,12 @@
     </row>
     <row r="15">
       <c r="A15" s="12" t="n"/>
-      <c r="B15" s="21">
+      <c r="B15" s="22">
         <f>IF(A15="","",COUNTIF('Funcionários'!$A$5:$A$34,A15))</f>
         <v/>
       </c>
       <c r="C15" s="13">
-        <f>IF(A15="","",SUMIF('Funcionários'!$A$5:$A$34,A15,'Funcionários'!$J$5:$J$34))</f>
+        <f>IF(A15="","",SUMIF('Funcionários'!$A$5:$A$34,A15,'Funcionários'!$S$5:$S$34))</f>
         <v/>
       </c>
       <c r="D15" s="13">
@@ -1908,16 +3092,16 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="22" t="inlineStr">
+      <c r="A16" s="23" t="inlineStr">
         <is>
           <t>TOTAL GERAL</t>
         </is>
       </c>
-      <c r="B16" s="18">
+      <c r="B16" s="20">
         <f>SUM(B4:B15)</f>
         <v/>
       </c>
-      <c r="C16" s="20">
+      <c r="C16" s="21">
         <f>SUM(C4:C15)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
📊 Dashboard Salário x Encargos (planilha + site)
- Planilha: aba Dashboard destacando Salário x Encargos (KPIs de total
  salário, total encargos e % de encargos sobre o salário) + gráfico
  pizza Salário x Encargos, além de custo por cargo e por regime.
- Site (calculadora de custo): novo painel "Salário × Encargos" com
  barras empilhadas para Simples e Presumido/Real, mostrando valor e %
  de cada parte.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/downloads/planilha-custo-empregado-gestor-certo.xlsx
+++ b/assets/downloads/planilha-custo-empregado-gestor-certo.xlsx
@@ -23,7 +23,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="R$ #,##0.00"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -70,6 +70,21 @@
       <b val="1"/>
       <color rgb="006B7A88"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001A56A5"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000C8A67"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C0392B"/>
+      <sz val="15"/>
     </font>
   </fonts>
   <fills count="8">
@@ -136,7 +151,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -150,9 +165,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -259,7 +277,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Custo por regime</a:t>
+              <a:t>Salário x Encargos</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -273,7 +291,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Dashboard'!B9</f>
+              <f>'Dashboard'!B10</f>
             </strRef>
           </tx>
           <spPr>
@@ -283,12 +301,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Dashboard'!$A$10:$A$11</f>
+              <f>'Dashboard'!$A$11:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Dashboard'!$B$10:$B$11</f>
+              <f>'Dashboard'!$B$11:$B$12</f>
             </numRef>
           </val>
         </ser>
@@ -395,6 +413,63 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
+              <a:t>Custo por regime</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <pieChart>
+        <varyColors val="1"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Dashboard'!E10</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Dashboard'!$D$11:$D$12</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Dashboard'!$E$11:$E$12</f>
+            </numRef>
+          </val>
+        </ser>
+        <firstSliceAng val="0"/>
+      </pieChart>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
               <a:t>Custo total por cargo (R$)</a:t>
             </a:r>
           </a:p>
@@ -468,10 +543,10 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>12</row>
+      <row>13</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="3240000" cy="2520000"/>
+    <ext cx="3960000" cy="2700000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -488,12 +563,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>3</col>
+      <col>0</col>
       <colOff>0</colOff>
-      <row>12</row>
+      <row>30</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="3960000" cy="2520000"/>
+    <ext cx="4320000" cy="2700000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -503,6 +578,28 @@
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>13</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3960000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -924,21 +1021,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="4" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="4" customWidth="1" min="6" max="6"/>
+    <col width="3" customWidth="1" min="6" max="6"/>
+    <col width="3" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>DASHBOARD DA FOLHA</t>
+          <t>DASHBOARD DA FOLHA — SALÁRIO x ENCARGOS</t>
         </is>
       </c>
     </row>
@@ -960,7 +1058,7 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>% médio sobre salários</t>
+          <t>Custo total / salários</t>
         </is>
       </c>
     </row>
@@ -982,50 +1080,114 @@
         <v/>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Total salário + comissões</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Total encargos + benefícios</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>Encargos sobre o salário</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10">
+        <f>(SUM('Funcionários'!D5:D34)+SUM('Funcionários'!E5:E34))</f>
+        <v/>
+      </c>
+      <c r="B7" s="11">
+        <f>SUM('Funcionários'!S5:S34)-(SUM('Funcionários'!D5:D34)+SUM('Funcionários'!E5:E34))</f>
+        <v/>
+      </c>
+      <c r="D7" s="12">
+        <f>IFERROR((SUM('Funcionários'!S5:S34)-(SUM('Funcionários'!D5:D34)+SUM('Funcionários'!E5:E34)))/(SUM('Funcionários'!D5:D34)+SUM('Funcionários'!E5:E34)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>Composição da folha</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
         <is>
           <t>Custo por regime</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>Valor/mês</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
         <is>
           <t>Regime</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="E10" s="14" t="inlineStr">
         <is>
           <t>Custo/mês</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="12" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>Salário + comissões</t>
+        </is>
+      </c>
+      <c r="B11" s="16">
+        <f>(SUM('Funcionários'!D5:D34)+SUM('Funcionários'!E5:E34))</f>
+        <v/>
+      </c>
+      <c r="D11" s="15" t="inlineStr">
         <is>
           <t>Simples</t>
         </is>
       </c>
-      <c r="B10" s="13">
+      <c r="E11" s="16">
         <f>SUMIF('Funcionários'!$C$5:$C$34,"Simples",'Funcionários'!$S$5:$S$34)</f>
         <v/>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="12" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="15" t="inlineStr">
+        <is>
+          <t>Encargos + benefícios</t>
+        </is>
+      </c>
+      <c r="B12" s="16">
+        <f>SUM('Funcionários'!S5:S34)-(SUM('Funcionários'!D5:D34)+SUM('Funcionários'!E5:E34))</f>
+        <v/>
+      </c>
+      <c r="D12" s="15" t="inlineStr">
         <is>
           <t>Presumido/Real</t>
         </is>
       </c>
-      <c r="B11" s="13">
-        <f>SUM('Funcionários'!$S$5:$S$34)-B10</f>
+      <c r="E12" s="16">
+        <f>SUM('Funcionários'!S5:S34)-E11</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1070,1783 +1232,1783 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="13" t="inlineStr">
         <is>
           <t>RAT (%):</t>
         </is>
       </c>
-      <c r="B2" s="14" t="n">
+      <c r="B2" s="17" t="n">
         <v>0.02</v>
       </c>
-      <c r="C2" s="10" t="inlineStr">
+      <c r="C2" s="13" t="inlineStr">
         <is>
           <t>Terceiros (%):</t>
         </is>
       </c>
-      <c r="D2" s="14" t="n">
+      <c r="D2" s="17" t="n">
         <v>0.058</v>
       </c>
-      <c r="F2" s="15" t="inlineStr">
+      <c r="F2" s="18" t="inlineStr">
         <is>
           <t>Amarelo = preencher · Azul = calculado</t>
         </is>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>Cargo</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>Nome</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C4" s="14" t="inlineStr">
         <is>
           <t>Regime</t>
         </is>
       </c>
-      <c r="D4" s="11" t="inlineStr">
+      <c r="D4" s="14" t="inlineStr">
         <is>
           <t>Salário</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
+      <c r="E4" s="14" t="inlineStr">
         <is>
           <t>Comissões</t>
         </is>
       </c>
-      <c r="F4" s="11" t="inlineStr">
+      <c r="F4" s="14" t="inlineStr">
         <is>
           <t>VT (mês)</t>
         </is>
       </c>
-      <c r="G4" s="11" t="inlineStr">
+      <c r="G4" s="14" t="inlineStr">
         <is>
           <t>VR (mês)</t>
         </is>
       </c>
-      <c r="H4" s="11" t="inlineStr">
+      <c r="H4" s="14" t="inlineStr">
         <is>
           <t>Desc. VR (%)</t>
         </is>
       </c>
-      <c r="I4" s="11" t="inlineStr">
+      <c r="I4" s="14" t="inlineStr">
         <is>
           <t>Plano/outros</t>
         </is>
       </c>
-      <c r="J4" s="16" t="inlineStr">
+      <c r="J4" s="19" t="inlineStr">
         <is>
           <t>INSS patr. 20%</t>
         </is>
       </c>
-      <c r="K4" s="16" t="inlineStr">
+      <c r="K4" s="19" t="inlineStr">
         <is>
           <t>RAT</t>
         </is>
       </c>
-      <c r="L4" s="16" t="inlineStr">
+      <c r="L4" s="19" t="inlineStr">
         <is>
           <t>Terceiros</t>
         </is>
       </c>
-      <c r="M4" s="16" t="inlineStr">
+      <c r="M4" s="19" t="inlineStr">
         <is>
           <t>FGTS 8%</t>
         </is>
       </c>
-      <c r="N4" s="16" t="inlineStr">
+      <c r="N4" s="19" t="inlineStr">
         <is>
           <t>Prov. 13º</t>
         </is>
       </c>
-      <c r="O4" s="16" t="inlineStr">
+      <c r="O4" s="19" t="inlineStr">
         <is>
           <t>Prov. férias+1/3</t>
         </is>
       </c>
-      <c r="P4" s="16" t="inlineStr">
+      <c r="P4" s="19" t="inlineStr">
         <is>
           <t>Multa FGTS 40%</t>
         </is>
       </c>
-      <c r="Q4" s="16" t="inlineStr">
+      <c r="Q4" s="19" t="inlineStr">
         <is>
           <t>Custo VT</t>
         </is>
       </c>
-      <c r="R4" s="16" t="inlineStr">
+      <c r="R4" s="19" t="inlineStr">
         <is>
           <t>Custo VR</t>
         </is>
       </c>
-      <c r="S4" s="16" t="inlineStr">
+      <c r="S4" s="19" t="inlineStr">
         <is>
           <t>CUSTO TOTAL</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>Vendedor</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="15" t="inlineStr">
         <is>
           <t>Ana</t>
         </is>
       </c>
-      <c r="C5" s="12" t="inlineStr">
+      <c r="C5" s="15" t="inlineStr">
         <is>
           <t>Simples</t>
         </is>
       </c>
-      <c r="D5" s="13" t="n">
+      <c r="D5" s="16" t="n">
         <v>2000</v>
       </c>
-      <c r="E5" s="13" t="n">
+      <c r="E5" s="16" t="n">
         <v>800</v>
       </c>
-      <c r="F5" s="13" t="n">
+      <c r="F5" s="16" t="n">
         <v>250</v>
       </c>
-      <c r="G5" s="13" t="n">
+      <c r="G5" s="16" t="n">
         <v>500</v>
       </c>
-      <c r="H5" s="17" t="n">
+      <c r="H5" s="20" t="n">
         <v>0.2</v>
       </c>
-      <c r="I5" s="13" t="n">
+      <c r="I5" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="J5" s="18">
+      <c r="J5" s="21">
         <f>IF(D5="","",IF(UPPER(C5)="SIMPLES",0,0.2*((D5+E5)+(D5+E5)/12+(D5+E5)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="K5" s="18">
+      <c r="K5" s="21">
         <f>IF(D5="","",IF(UPPER(C5)="SIMPLES",0,$B$2*((D5+E5)+(D5+E5)/12+(D5+E5)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="L5" s="18">
+      <c r="L5" s="21">
         <f>IF(D5="","",IF(UPPER(C5)="SIMPLES",0,$D$2*((D5+E5)+(D5+E5)/12+(D5+E5)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="M5" s="18">
+      <c r="M5" s="21">
         <f>IF(D5="","",0.08*((D5+E5)+(D5+E5)/12+(D5+E5)*4/3/12))</f>
         <v/>
       </c>
-      <c r="N5" s="18">
+      <c r="N5" s="21">
         <f>IF(D5="","",(D5+E5)/12)</f>
         <v/>
       </c>
-      <c r="O5" s="18">
+      <c r="O5" s="21">
         <f>IF(D5="","",(D5+E5)*4/3/12)</f>
         <v/>
       </c>
-      <c r="P5" s="18">
+      <c r="P5" s="21">
         <f>IF(D5="","",0.4*0.08*((D5+E5)+(D5+E5)/12+(D5+E5)*4/3/12))</f>
         <v/>
       </c>
-      <c r="Q5" s="18">
+      <c r="Q5" s="21">
         <f>IF(D5="","",F5-MIN(F5,0.06*D5))</f>
         <v/>
       </c>
-      <c r="R5" s="18">
+      <c r="R5" s="21">
         <f>IF(D5="","",G5-G5*H5)</f>
         <v/>
       </c>
-      <c r="S5" s="19">
+      <c r="S5" s="22">
         <f>IF(D5="","",D5+E5+J5+K5+L5+M5+N5+O5+P5+Q5+R5+I5)</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>Vendedor</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>Bruno</t>
         </is>
       </c>
-      <c r="C6" s="12" t="inlineStr">
+      <c r="C6" s="15" t="inlineStr">
         <is>
           <t>Simples</t>
         </is>
       </c>
-      <c r="D6" s="13" t="n">
+      <c r="D6" s="16" t="n">
         <v>2000</v>
       </c>
-      <c r="E6" s="13" t="n">
+      <c r="E6" s="16" t="n">
         <v>500</v>
       </c>
-      <c r="F6" s="13" t="n">
+      <c r="F6" s="16" t="n">
         <v>250</v>
       </c>
-      <c r="G6" s="13" t="n">
+      <c r="G6" s="16" t="n">
         <v>500</v>
       </c>
-      <c r="H6" s="17" t="n">
+      <c r="H6" s="20" t="n">
         <v>0.2</v>
       </c>
-      <c r="I6" s="13" t="n">
+      <c r="I6" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="J6" s="18">
+      <c r="J6" s="21">
         <f>IF(D6="","",IF(UPPER(C6)="SIMPLES",0,0.2*((D6+E6)+(D6+E6)/12+(D6+E6)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="K6" s="18">
+      <c r="K6" s="21">
         <f>IF(D6="","",IF(UPPER(C6)="SIMPLES",0,$B$2*((D6+E6)+(D6+E6)/12+(D6+E6)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="L6" s="18">
+      <c r="L6" s="21">
         <f>IF(D6="","",IF(UPPER(C6)="SIMPLES",0,$D$2*((D6+E6)+(D6+E6)/12+(D6+E6)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="M6" s="18">
+      <c r="M6" s="21">
         <f>IF(D6="","",0.08*((D6+E6)+(D6+E6)/12+(D6+E6)*4/3/12))</f>
         <v/>
       </c>
-      <c r="N6" s="18">
+      <c r="N6" s="21">
         <f>IF(D6="","",(D6+E6)/12)</f>
         <v/>
       </c>
-      <c r="O6" s="18">
+      <c r="O6" s="21">
         <f>IF(D6="","",(D6+E6)*4/3/12)</f>
         <v/>
       </c>
-      <c r="P6" s="18">
+      <c r="P6" s="21">
         <f>IF(D6="","",0.4*0.08*((D6+E6)+(D6+E6)/12+(D6+E6)*4/3/12))</f>
         <v/>
       </c>
-      <c r="Q6" s="18">
+      <c r="Q6" s="21">
         <f>IF(D6="","",F6-MIN(F6,0.06*D6))</f>
         <v/>
       </c>
-      <c r="R6" s="18">
+      <c r="R6" s="21">
         <f>IF(D6="","",G6-G6*H6)</f>
         <v/>
       </c>
-      <c r="S6" s="19">
+      <c r="S6" s="22">
         <f>IF(D6="","",D6+E6+J6+K6+L6+M6+N6+O6+P6+Q6+R6+I6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>Gerente</t>
         </is>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>Carla</t>
         </is>
       </c>
-      <c r="C7" s="12" t="inlineStr">
+      <c r="C7" s="15" t="inlineStr">
         <is>
           <t>Presumido</t>
         </is>
       </c>
-      <c r="D7" s="13" t="n">
+      <c r="D7" s="16" t="n">
         <v>6000</v>
       </c>
-      <c r="E7" s="13" t="n">
+      <c r="E7" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="F7" s="13" t="n">
+      <c r="F7" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="13" t="n">
+      <c r="G7" s="16" t="n">
         <v>800</v>
       </c>
-      <c r="H7" s="17" t="n">
+      <c r="H7" s="20" t="n">
         <v>0.2</v>
       </c>
-      <c r="I7" s="13" t="n">
+      <c r="I7" s="16" t="n">
         <v>500</v>
       </c>
-      <c r="J7" s="18">
+      <c r="J7" s="21">
         <f>IF(D7="","",IF(UPPER(C7)="SIMPLES",0,0.2*((D7+E7)+(D7+E7)/12+(D7+E7)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="K7" s="18">
+      <c r="K7" s="21">
         <f>IF(D7="","",IF(UPPER(C7)="SIMPLES",0,$B$2*((D7+E7)+(D7+E7)/12+(D7+E7)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="L7" s="18">
+      <c r="L7" s="21">
         <f>IF(D7="","",IF(UPPER(C7)="SIMPLES",0,$D$2*((D7+E7)+(D7+E7)/12+(D7+E7)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="M7" s="18">
+      <c r="M7" s="21">
         <f>IF(D7="","",0.08*((D7+E7)+(D7+E7)/12+(D7+E7)*4/3/12))</f>
         <v/>
       </c>
-      <c r="N7" s="18">
+      <c r="N7" s="21">
         <f>IF(D7="","",(D7+E7)/12)</f>
         <v/>
       </c>
-      <c r="O7" s="18">
+      <c r="O7" s="21">
         <f>IF(D7="","",(D7+E7)*4/3/12)</f>
         <v/>
       </c>
-      <c r="P7" s="18">
+      <c r="P7" s="21">
         <f>IF(D7="","",0.4*0.08*((D7+E7)+(D7+E7)/12+(D7+E7)*4/3/12))</f>
         <v/>
       </c>
-      <c r="Q7" s="18">
+      <c r="Q7" s="21">
         <f>IF(D7="","",F7-MIN(F7,0.06*D7))</f>
         <v/>
       </c>
-      <c r="R7" s="18">
+      <c r="R7" s="21">
         <f>IF(D7="","",G7-G7*H7)</f>
         <v/>
       </c>
-      <c r="S7" s="19">
+      <c r="S7" s="22">
         <f>IF(D7="","",D7+E7+J7+K7+L7+M7+N7+O7+P7+Q7+R7+I7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="n"/>
-      <c r="B8" s="12" t="n"/>
-      <c r="C8" s="12" t="n"/>
-      <c r="D8" s="13" t="n"/>
-      <c r="E8" s="13" t="n"/>
-      <c r="F8" s="13" t="n"/>
-      <c r="G8" s="13" t="n"/>
-      <c r="H8" s="17" t="n"/>
-      <c r="I8" s="13" t="n"/>
-      <c r="J8" s="18">
+      <c r="A8" s="15" t="n"/>
+      <c r="B8" s="15" t="n"/>
+      <c r="C8" s="15" t="n"/>
+      <c r="D8" s="16" t="n"/>
+      <c r="E8" s="16" t="n"/>
+      <c r="F8" s="16" t="n"/>
+      <c r="G8" s="16" t="n"/>
+      <c r="H8" s="20" t="n"/>
+      <c r="I8" s="16" t="n"/>
+      <c r="J8" s="21">
         <f>IF(D8="","",IF(UPPER(C8)="SIMPLES",0,0.2*((D8+E8)+(D8+E8)/12+(D8+E8)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="K8" s="18">
+      <c r="K8" s="21">
         <f>IF(D8="","",IF(UPPER(C8)="SIMPLES",0,$B$2*((D8+E8)+(D8+E8)/12+(D8+E8)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="L8" s="18">
+      <c r="L8" s="21">
         <f>IF(D8="","",IF(UPPER(C8)="SIMPLES",0,$D$2*((D8+E8)+(D8+E8)/12+(D8+E8)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="M8" s="18">
+      <c r="M8" s="21">
         <f>IF(D8="","",0.08*((D8+E8)+(D8+E8)/12+(D8+E8)*4/3/12))</f>
         <v/>
       </c>
-      <c r="N8" s="18">
+      <c r="N8" s="21">
         <f>IF(D8="","",(D8+E8)/12)</f>
         <v/>
       </c>
-      <c r="O8" s="18">
+      <c r="O8" s="21">
         <f>IF(D8="","",(D8+E8)*4/3/12)</f>
         <v/>
       </c>
-      <c r="P8" s="18">
+      <c r="P8" s="21">
         <f>IF(D8="","",0.4*0.08*((D8+E8)+(D8+E8)/12+(D8+E8)*4/3/12))</f>
         <v/>
       </c>
-      <c r="Q8" s="18">
+      <c r="Q8" s="21">
         <f>IF(D8="","",F8-MIN(F8,0.06*D8))</f>
         <v/>
       </c>
-      <c r="R8" s="18">
+      <c r="R8" s="21">
         <f>IF(D8="","",G8-G8*H8)</f>
         <v/>
       </c>
-      <c r="S8" s="19">
+      <c r="S8" s="22">
         <f>IF(D8="","",D8+E8+J8+K8+L8+M8+N8+O8+P8+Q8+R8+I8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="n"/>
-      <c r="B9" s="12" t="n"/>
-      <c r="C9" s="12" t="n"/>
-      <c r="D9" s="13" t="n"/>
-      <c r="E9" s="13" t="n"/>
-      <c r="F9" s="13" t="n"/>
-      <c r="G9" s="13" t="n"/>
-      <c r="H9" s="17" t="n"/>
-      <c r="I9" s="13" t="n"/>
-      <c r="J9" s="18">
+      <c r="A9" s="15" t="n"/>
+      <c r="B9" s="15" t="n"/>
+      <c r="C9" s="15" t="n"/>
+      <c r="D9" s="16" t="n"/>
+      <c r="E9" s="16" t="n"/>
+      <c r="F9" s="16" t="n"/>
+      <c r="G9" s="16" t="n"/>
+      <c r="H9" s="20" t="n"/>
+      <c r="I9" s="16" t="n"/>
+      <c r="J9" s="21">
         <f>IF(D9="","",IF(UPPER(C9)="SIMPLES",0,0.2*((D9+E9)+(D9+E9)/12+(D9+E9)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="K9" s="18">
+      <c r="K9" s="21">
         <f>IF(D9="","",IF(UPPER(C9)="SIMPLES",0,$B$2*((D9+E9)+(D9+E9)/12+(D9+E9)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="L9" s="18">
+      <c r="L9" s="21">
         <f>IF(D9="","",IF(UPPER(C9)="SIMPLES",0,$D$2*((D9+E9)+(D9+E9)/12+(D9+E9)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="M9" s="18">
+      <c r="M9" s="21">
         <f>IF(D9="","",0.08*((D9+E9)+(D9+E9)/12+(D9+E9)*4/3/12))</f>
         <v/>
       </c>
-      <c r="N9" s="18">
+      <c r="N9" s="21">
         <f>IF(D9="","",(D9+E9)/12)</f>
         <v/>
       </c>
-      <c r="O9" s="18">
+      <c r="O9" s="21">
         <f>IF(D9="","",(D9+E9)*4/3/12)</f>
         <v/>
       </c>
-      <c r="P9" s="18">
+      <c r="P9" s="21">
         <f>IF(D9="","",0.4*0.08*((D9+E9)+(D9+E9)/12+(D9+E9)*4/3/12))</f>
         <v/>
       </c>
-      <c r="Q9" s="18">
+      <c r="Q9" s="21">
         <f>IF(D9="","",F9-MIN(F9,0.06*D9))</f>
         <v/>
       </c>
-      <c r="R9" s="18">
+      <c r="R9" s="21">
         <f>IF(D9="","",G9-G9*H9)</f>
         <v/>
       </c>
-      <c r="S9" s="19">
+      <c r="S9" s="22">
         <f>IF(D9="","",D9+E9+J9+K9+L9+M9+N9+O9+P9+Q9+R9+I9)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="n"/>
-      <c r="B10" s="12" t="n"/>
-      <c r="C10" s="12" t="n"/>
-      <c r="D10" s="13" t="n"/>
-      <c r="E10" s="13" t="n"/>
-      <c r="F10" s="13" t="n"/>
-      <c r="G10" s="13" t="n"/>
-      <c r="H10" s="17" t="n"/>
-      <c r="I10" s="13" t="n"/>
-      <c r="J10" s="18">
+      <c r="A10" s="15" t="n"/>
+      <c r="B10" s="15" t="n"/>
+      <c r="C10" s="15" t="n"/>
+      <c r="D10" s="16" t="n"/>
+      <c r="E10" s="16" t="n"/>
+      <c r="F10" s="16" t="n"/>
+      <c r="G10" s="16" t="n"/>
+      <c r="H10" s="20" t="n"/>
+      <c r="I10" s="16" t="n"/>
+      <c r="J10" s="21">
         <f>IF(D10="","",IF(UPPER(C10)="SIMPLES",0,0.2*((D10+E10)+(D10+E10)/12+(D10+E10)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="K10" s="18">
+      <c r="K10" s="21">
         <f>IF(D10="","",IF(UPPER(C10)="SIMPLES",0,$B$2*((D10+E10)+(D10+E10)/12+(D10+E10)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="L10" s="18">
+      <c r="L10" s="21">
         <f>IF(D10="","",IF(UPPER(C10)="SIMPLES",0,$D$2*((D10+E10)+(D10+E10)/12+(D10+E10)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="M10" s="18">
+      <c r="M10" s="21">
         <f>IF(D10="","",0.08*((D10+E10)+(D10+E10)/12+(D10+E10)*4/3/12))</f>
         <v/>
       </c>
-      <c r="N10" s="18">
+      <c r="N10" s="21">
         <f>IF(D10="","",(D10+E10)/12)</f>
         <v/>
       </c>
-      <c r="O10" s="18">
+      <c r="O10" s="21">
         <f>IF(D10="","",(D10+E10)*4/3/12)</f>
         <v/>
       </c>
-      <c r="P10" s="18">
+      <c r="P10" s="21">
         <f>IF(D10="","",0.4*0.08*((D10+E10)+(D10+E10)/12+(D10+E10)*4/3/12))</f>
         <v/>
       </c>
-      <c r="Q10" s="18">
+      <c r="Q10" s="21">
         <f>IF(D10="","",F10-MIN(F10,0.06*D10))</f>
         <v/>
       </c>
-      <c r="R10" s="18">
+      <c r="R10" s="21">
         <f>IF(D10="","",G10-G10*H10)</f>
         <v/>
       </c>
-      <c r="S10" s="19">
+      <c r="S10" s="22">
         <f>IF(D10="","",D10+E10+J10+K10+L10+M10+N10+O10+P10+Q10+R10+I10)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="n"/>
-      <c r="B11" s="12" t="n"/>
-      <c r="C11" s="12" t="n"/>
-      <c r="D11" s="13" t="n"/>
-      <c r="E11" s="13" t="n"/>
-      <c r="F11" s="13" t="n"/>
-      <c r="G11" s="13" t="n"/>
-      <c r="H11" s="17" t="n"/>
-      <c r="I11" s="13" t="n"/>
-      <c r="J11" s="18">
+      <c r="A11" s="15" t="n"/>
+      <c r="B11" s="15" t="n"/>
+      <c r="C11" s="15" t="n"/>
+      <c r="D11" s="16" t="n"/>
+      <c r="E11" s="16" t="n"/>
+      <c r="F11" s="16" t="n"/>
+      <c r="G11" s="16" t="n"/>
+      <c r="H11" s="20" t="n"/>
+      <c r="I11" s="16" t="n"/>
+      <c r="J11" s="21">
         <f>IF(D11="","",IF(UPPER(C11)="SIMPLES",0,0.2*((D11+E11)+(D11+E11)/12+(D11+E11)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="K11" s="18">
+      <c r="K11" s="21">
         <f>IF(D11="","",IF(UPPER(C11)="SIMPLES",0,$B$2*((D11+E11)+(D11+E11)/12+(D11+E11)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="L11" s="18">
+      <c r="L11" s="21">
         <f>IF(D11="","",IF(UPPER(C11)="SIMPLES",0,$D$2*((D11+E11)+(D11+E11)/12+(D11+E11)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="M11" s="18">
+      <c r="M11" s="21">
         <f>IF(D11="","",0.08*((D11+E11)+(D11+E11)/12+(D11+E11)*4/3/12))</f>
         <v/>
       </c>
-      <c r="N11" s="18">
+      <c r="N11" s="21">
         <f>IF(D11="","",(D11+E11)/12)</f>
         <v/>
       </c>
-      <c r="O11" s="18">
+      <c r="O11" s="21">
         <f>IF(D11="","",(D11+E11)*4/3/12)</f>
         <v/>
       </c>
-      <c r="P11" s="18">
+      <c r="P11" s="21">
         <f>IF(D11="","",0.4*0.08*((D11+E11)+(D11+E11)/12+(D11+E11)*4/3/12))</f>
         <v/>
       </c>
-      <c r="Q11" s="18">
+      <c r="Q11" s="21">
         <f>IF(D11="","",F11-MIN(F11,0.06*D11))</f>
         <v/>
       </c>
-      <c r="R11" s="18">
+      <c r="R11" s="21">
         <f>IF(D11="","",G11-G11*H11)</f>
         <v/>
       </c>
-      <c r="S11" s="19">
+      <c r="S11" s="22">
         <f>IF(D11="","",D11+E11+J11+K11+L11+M11+N11+O11+P11+Q11+R11+I11)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="n"/>
-      <c r="B12" s="12" t="n"/>
-      <c r="C12" s="12" t="n"/>
-      <c r="D12" s="13" t="n"/>
-      <c r="E12" s="13" t="n"/>
-      <c r="F12" s="13" t="n"/>
-      <c r="G12" s="13" t="n"/>
-      <c r="H12" s="17" t="n"/>
-      <c r="I12" s="13" t="n"/>
-      <c r="J12" s="18">
+      <c r="A12" s="15" t="n"/>
+      <c r="B12" s="15" t="n"/>
+      <c r="C12" s="15" t="n"/>
+      <c r="D12" s="16" t="n"/>
+      <c r="E12" s="16" t="n"/>
+      <c r="F12" s="16" t="n"/>
+      <c r="G12" s="16" t="n"/>
+      <c r="H12" s="20" t="n"/>
+      <c r="I12" s="16" t="n"/>
+      <c r="J12" s="21">
         <f>IF(D12="","",IF(UPPER(C12)="SIMPLES",0,0.2*((D12+E12)+(D12+E12)/12+(D12+E12)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="K12" s="18">
+      <c r="K12" s="21">
         <f>IF(D12="","",IF(UPPER(C12)="SIMPLES",0,$B$2*((D12+E12)+(D12+E12)/12+(D12+E12)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="L12" s="18">
+      <c r="L12" s="21">
         <f>IF(D12="","",IF(UPPER(C12)="SIMPLES",0,$D$2*((D12+E12)+(D12+E12)/12+(D12+E12)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="M12" s="18">
+      <c r="M12" s="21">
         <f>IF(D12="","",0.08*((D12+E12)+(D12+E12)/12+(D12+E12)*4/3/12))</f>
         <v/>
       </c>
-      <c r="N12" s="18">
+      <c r="N12" s="21">
         <f>IF(D12="","",(D12+E12)/12)</f>
         <v/>
       </c>
-      <c r="O12" s="18">
+      <c r="O12" s="21">
         <f>IF(D12="","",(D12+E12)*4/3/12)</f>
         <v/>
       </c>
-      <c r="P12" s="18">
+      <c r="P12" s="21">
         <f>IF(D12="","",0.4*0.08*((D12+E12)+(D12+E12)/12+(D12+E12)*4/3/12))</f>
         <v/>
       </c>
-      <c r="Q12" s="18">
+      <c r="Q12" s="21">
         <f>IF(D12="","",F12-MIN(F12,0.06*D12))</f>
         <v/>
       </c>
-      <c r="R12" s="18">
+      <c r="R12" s="21">
         <f>IF(D12="","",G12-G12*H12)</f>
         <v/>
       </c>
-      <c r="S12" s="19">
+      <c r="S12" s="22">
         <f>IF(D12="","",D12+E12+J12+K12+L12+M12+N12+O12+P12+Q12+R12+I12)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="n"/>
-      <c r="B13" s="12" t="n"/>
-      <c r="C13" s="12" t="n"/>
-      <c r="D13" s="13" t="n"/>
-      <c r="E13" s="13" t="n"/>
-      <c r="F13" s="13" t="n"/>
-      <c r="G13" s="13" t="n"/>
-      <c r="H13" s="17" t="n"/>
-      <c r="I13" s="13" t="n"/>
-      <c r="J13" s="18">
+      <c r="A13" s="15" t="n"/>
+      <c r="B13" s="15" t="n"/>
+      <c r="C13" s="15" t="n"/>
+      <c r="D13" s="16" t="n"/>
+      <c r="E13" s="16" t="n"/>
+      <c r="F13" s="16" t="n"/>
+      <c r="G13" s="16" t="n"/>
+      <c r="H13" s="20" t="n"/>
+      <c r="I13" s="16" t="n"/>
+      <c r="J13" s="21">
         <f>IF(D13="","",IF(UPPER(C13)="SIMPLES",0,0.2*((D13+E13)+(D13+E13)/12+(D13+E13)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="K13" s="18">
+      <c r="K13" s="21">
         <f>IF(D13="","",IF(UPPER(C13)="SIMPLES",0,$B$2*((D13+E13)+(D13+E13)/12+(D13+E13)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="L13" s="18">
+      <c r="L13" s="21">
         <f>IF(D13="","",IF(UPPER(C13)="SIMPLES",0,$D$2*((D13+E13)+(D13+E13)/12+(D13+E13)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="M13" s="18">
+      <c r="M13" s="21">
         <f>IF(D13="","",0.08*((D13+E13)+(D13+E13)/12+(D13+E13)*4/3/12))</f>
         <v/>
       </c>
-      <c r="N13" s="18">
+      <c r="N13" s="21">
         <f>IF(D13="","",(D13+E13)/12)</f>
         <v/>
       </c>
-      <c r="O13" s="18">
+      <c r="O13" s="21">
         <f>IF(D13="","",(D13+E13)*4/3/12)</f>
         <v/>
       </c>
-      <c r="P13" s="18">
+      <c r="P13" s="21">
         <f>IF(D13="","",0.4*0.08*((D13+E13)+(D13+E13)/12+(D13+E13)*4/3/12))</f>
         <v/>
       </c>
-      <c r="Q13" s="18">
+      <c r="Q13" s="21">
         <f>IF(D13="","",F13-MIN(F13,0.06*D13))</f>
         <v/>
       </c>
-      <c r="R13" s="18">
+      <c r="R13" s="21">
         <f>IF(D13="","",G13-G13*H13)</f>
         <v/>
       </c>
-      <c r="S13" s="19">
+      <c r="S13" s="22">
         <f>IF(D13="","",D13+E13+J13+K13+L13+M13+N13+O13+P13+Q13+R13+I13)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="n"/>
-      <c r="B14" s="12" t="n"/>
-      <c r="C14" s="12" t="n"/>
-      <c r="D14" s="13" t="n"/>
-      <c r="E14" s="13" t="n"/>
-      <c r="F14" s="13" t="n"/>
-      <c r="G14" s="13" t="n"/>
-      <c r="H14" s="17" t="n"/>
-      <c r="I14" s="13" t="n"/>
-      <c r="J14" s="18">
+      <c r="A14" s="15" t="n"/>
+      <c r="B14" s="15" t="n"/>
+      <c r="C14" s="15" t="n"/>
+      <c r="D14" s="16" t="n"/>
+      <c r="E14" s="16" t="n"/>
+      <c r="F14" s="16" t="n"/>
+      <c r="G14" s="16" t="n"/>
+      <c r="H14" s="20" t="n"/>
+      <c r="I14" s="16" t="n"/>
+      <c r="J14" s="21">
         <f>IF(D14="","",IF(UPPER(C14)="SIMPLES",0,0.2*((D14+E14)+(D14+E14)/12+(D14+E14)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="K14" s="18">
+      <c r="K14" s="21">
         <f>IF(D14="","",IF(UPPER(C14)="SIMPLES",0,$B$2*((D14+E14)+(D14+E14)/12+(D14+E14)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="L14" s="18">
+      <c r="L14" s="21">
         <f>IF(D14="","",IF(UPPER(C14)="SIMPLES",0,$D$2*((D14+E14)+(D14+E14)/12+(D14+E14)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="M14" s="18">
+      <c r="M14" s="21">
         <f>IF(D14="","",0.08*((D14+E14)+(D14+E14)/12+(D14+E14)*4/3/12))</f>
         <v/>
       </c>
-      <c r="N14" s="18">
+      <c r="N14" s="21">
         <f>IF(D14="","",(D14+E14)/12)</f>
         <v/>
       </c>
-      <c r="O14" s="18">
+      <c r="O14" s="21">
         <f>IF(D14="","",(D14+E14)*4/3/12)</f>
         <v/>
       </c>
-      <c r="P14" s="18">
+      <c r="P14" s="21">
         <f>IF(D14="","",0.4*0.08*((D14+E14)+(D14+E14)/12+(D14+E14)*4/3/12))</f>
         <v/>
       </c>
-      <c r="Q14" s="18">
+      <c r="Q14" s="21">
         <f>IF(D14="","",F14-MIN(F14,0.06*D14))</f>
         <v/>
       </c>
-      <c r="R14" s="18">
+      <c r="R14" s="21">
         <f>IF(D14="","",G14-G14*H14)</f>
         <v/>
       </c>
-      <c r="S14" s="19">
+      <c r="S14" s="22">
         <f>IF(D14="","",D14+E14+J14+K14+L14+M14+N14+O14+P14+Q14+R14+I14)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="n"/>
-      <c r="B15" s="12" t="n"/>
-      <c r="C15" s="12" t="n"/>
-      <c r="D15" s="13" t="n"/>
-      <c r="E15" s="13" t="n"/>
-      <c r="F15" s="13" t="n"/>
-      <c r="G15" s="13" t="n"/>
-      <c r="H15" s="17" t="n"/>
-      <c r="I15" s="13" t="n"/>
-      <c r="J15" s="18">
+      <c r="A15" s="15" t="n"/>
+      <c r="B15" s="15" t="n"/>
+      <c r="C15" s="15" t="n"/>
+      <c r="D15" s="16" t="n"/>
+      <c r="E15" s="16" t="n"/>
+      <c r="F15" s="16" t="n"/>
+      <c r="G15" s="16" t="n"/>
+      <c r="H15" s="20" t="n"/>
+      <c r="I15" s="16" t="n"/>
+      <c r="J15" s="21">
         <f>IF(D15="","",IF(UPPER(C15)="SIMPLES",0,0.2*((D15+E15)+(D15+E15)/12+(D15+E15)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="K15" s="18">
+      <c r="K15" s="21">
         <f>IF(D15="","",IF(UPPER(C15)="SIMPLES",0,$B$2*((D15+E15)+(D15+E15)/12+(D15+E15)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="L15" s="18">
+      <c r="L15" s="21">
         <f>IF(D15="","",IF(UPPER(C15)="SIMPLES",0,$D$2*((D15+E15)+(D15+E15)/12+(D15+E15)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="M15" s="18">
+      <c r="M15" s="21">
         <f>IF(D15="","",0.08*((D15+E15)+(D15+E15)/12+(D15+E15)*4/3/12))</f>
         <v/>
       </c>
-      <c r="N15" s="18">
+      <c r="N15" s="21">
         <f>IF(D15="","",(D15+E15)/12)</f>
         <v/>
       </c>
-      <c r="O15" s="18">
+      <c r="O15" s="21">
         <f>IF(D15="","",(D15+E15)*4/3/12)</f>
         <v/>
       </c>
-      <c r="P15" s="18">
+      <c r="P15" s="21">
         <f>IF(D15="","",0.4*0.08*((D15+E15)+(D15+E15)/12+(D15+E15)*4/3/12))</f>
         <v/>
       </c>
-      <c r="Q15" s="18">
+      <c r="Q15" s="21">
         <f>IF(D15="","",F15-MIN(F15,0.06*D15))</f>
         <v/>
       </c>
-      <c r="R15" s="18">
+      <c r="R15" s="21">
         <f>IF(D15="","",G15-G15*H15)</f>
         <v/>
       </c>
-      <c r="S15" s="19">
+      <c r="S15" s="22">
         <f>IF(D15="","",D15+E15+J15+K15+L15+M15+N15+O15+P15+Q15+R15+I15)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="n"/>
-      <c r="B16" s="12" t="n"/>
-      <c r="C16" s="12" t="n"/>
-      <c r="D16" s="13" t="n"/>
-      <c r="E16" s="13" t="n"/>
-      <c r="F16" s="13" t="n"/>
-      <c r="G16" s="13" t="n"/>
-      <c r="H16" s="17" t="n"/>
-      <c r="I16" s="13" t="n"/>
-      <c r="J16" s="18">
+      <c r="A16" s="15" t="n"/>
+      <c r="B16" s="15" t="n"/>
+      <c r="C16" s="15" t="n"/>
+      <c r="D16" s="16" t="n"/>
+      <c r="E16" s="16" t="n"/>
+      <c r="F16" s="16" t="n"/>
+      <c r="G16" s="16" t="n"/>
+      <c r="H16" s="20" t="n"/>
+      <c r="I16" s="16" t="n"/>
+      <c r="J16" s="21">
         <f>IF(D16="","",IF(UPPER(C16)="SIMPLES",0,0.2*((D16+E16)+(D16+E16)/12+(D16+E16)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="K16" s="18">
+      <c r="K16" s="21">
         <f>IF(D16="","",IF(UPPER(C16)="SIMPLES",0,$B$2*((D16+E16)+(D16+E16)/12+(D16+E16)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="L16" s="18">
+      <c r="L16" s="21">
         <f>IF(D16="","",IF(UPPER(C16)="SIMPLES",0,$D$2*((D16+E16)+(D16+E16)/12+(D16+E16)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="M16" s="18">
+      <c r="M16" s="21">
         <f>IF(D16="","",0.08*((D16+E16)+(D16+E16)/12+(D16+E16)*4/3/12))</f>
         <v/>
       </c>
-      <c r="N16" s="18">
+      <c r="N16" s="21">
         <f>IF(D16="","",(D16+E16)/12)</f>
         <v/>
       </c>
-      <c r="O16" s="18">
+      <c r="O16" s="21">
         <f>IF(D16="","",(D16+E16)*4/3/12)</f>
         <v/>
       </c>
-      <c r="P16" s="18">
+      <c r="P16" s="21">
         <f>IF(D16="","",0.4*0.08*((D16+E16)+(D16+E16)/12+(D16+E16)*4/3/12))</f>
         <v/>
       </c>
-      <c r="Q16" s="18">
+      <c r="Q16" s="21">
         <f>IF(D16="","",F16-MIN(F16,0.06*D16))</f>
         <v/>
       </c>
-      <c r="R16" s="18">
+      <c r="R16" s="21">
         <f>IF(D16="","",G16-G16*H16)</f>
         <v/>
       </c>
-      <c r="S16" s="19">
+      <c r="S16" s="22">
         <f>IF(D16="","",D16+E16+J16+K16+L16+M16+N16+O16+P16+Q16+R16+I16)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="n"/>
-      <c r="B17" s="12" t="n"/>
-      <c r="C17" s="12" t="n"/>
-      <c r="D17" s="13" t="n"/>
-      <c r="E17" s="13" t="n"/>
-      <c r="F17" s="13" t="n"/>
-      <c r="G17" s="13" t="n"/>
-      <c r="H17" s="17" t="n"/>
-      <c r="I17" s="13" t="n"/>
-      <c r="J17" s="18">
+      <c r="A17" s="15" t="n"/>
+      <c r="B17" s="15" t="n"/>
+      <c r="C17" s="15" t="n"/>
+      <c r="D17" s="16" t="n"/>
+      <c r="E17" s="16" t="n"/>
+      <c r="F17" s="16" t="n"/>
+      <c r="G17" s="16" t="n"/>
+      <c r="H17" s="20" t="n"/>
+      <c r="I17" s="16" t="n"/>
+      <c r="J17" s="21">
         <f>IF(D17="","",IF(UPPER(C17)="SIMPLES",0,0.2*((D17+E17)+(D17+E17)/12+(D17+E17)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="K17" s="18">
+      <c r="K17" s="21">
         <f>IF(D17="","",IF(UPPER(C17)="SIMPLES",0,$B$2*((D17+E17)+(D17+E17)/12+(D17+E17)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="L17" s="18">
+      <c r="L17" s="21">
         <f>IF(D17="","",IF(UPPER(C17)="SIMPLES",0,$D$2*((D17+E17)+(D17+E17)/12+(D17+E17)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="M17" s="18">
+      <c r="M17" s="21">
         <f>IF(D17="","",0.08*((D17+E17)+(D17+E17)/12+(D17+E17)*4/3/12))</f>
         <v/>
       </c>
-      <c r="N17" s="18">
+      <c r="N17" s="21">
         <f>IF(D17="","",(D17+E17)/12)</f>
         <v/>
       </c>
-      <c r="O17" s="18">
+      <c r="O17" s="21">
         <f>IF(D17="","",(D17+E17)*4/3/12)</f>
         <v/>
       </c>
-      <c r="P17" s="18">
+      <c r="P17" s="21">
         <f>IF(D17="","",0.4*0.08*((D17+E17)+(D17+E17)/12+(D17+E17)*4/3/12))</f>
         <v/>
       </c>
-      <c r="Q17" s="18">
+      <c r="Q17" s="21">
         <f>IF(D17="","",F17-MIN(F17,0.06*D17))</f>
         <v/>
       </c>
-      <c r="R17" s="18">
+      <c r="R17" s="21">
         <f>IF(D17="","",G17-G17*H17)</f>
         <v/>
       </c>
-      <c r="S17" s="19">
+      <c r="S17" s="22">
         <f>IF(D17="","",D17+E17+J17+K17+L17+M17+N17+O17+P17+Q17+R17+I17)</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="n"/>
-      <c r="B18" s="12" t="n"/>
-      <c r="C18" s="12" t="n"/>
-      <c r="D18" s="13" t="n"/>
-      <c r="E18" s="13" t="n"/>
-      <c r="F18" s="13" t="n"/>
-      <c r="G18" s="13" t="n"/>
-      <c r="H18" s="17" t="n"/>
-      <c r="I18" s="13" t="n"/>
-      <c r="J18" s="18">
+      <c r="A18" s="15" t="n"/>
+      <c r="B18" s="15" t="n"/>
+      <c r="C18" s="15" t="n"/>
+      <c r="D18" s="16" t="n"/>
+      <c r="E18" s="16" t="n"/>
+      <c r="F18" s="16" t="n"/>
+      <c r="G18" s="16" t="n"/>
+      <c r="H18" s="20" t="n"/>
+      <c r="I18" s="16" t="n"/>
+      <c r="J18" s="21">
         <f>IF(D18="","",IF(UPPER(C18)="SIMPLES",0,0.2*((D18+E18)+(D18+E18)/12+(D18+E18)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="K18" s="18">
+      <c r="K18" s="21">
         <f>IF(D18="","",IF(UPPER(C18)="SIMPLES",0,$B$2*((D18+E18)+(D18+E18)/12+(D18+E18)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="L18" s="18">
+      <c r="L18" s="21">
         <f>IF(D18="","",IF(UPPER(C18)="SIMPLES",0,$D$2*((D18+E18)+(D18+E18)/12+(D18+E18)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="M18" s="18">
+      <c r="M18" s="21">
         <f>IF(D18="","",0.08*((D18+E18)+(D18+E18)/12+(D18+E18)*4/3/12))</f>
         <v/>
       </c>
-      <c r="N18" s="18">
+      <c r="N18" s="21">
         <f>IF(D18="","",(D18+E18)/12)</f>
         <v/>
       </c>
-      <c r="O18" s="18">
+      <c r="O18" s="21">
         <f>IF(D18="","",(D18+E18)*4/3/12)</f>
         <v/>
       </c>
-      <c r="P18" s="18">
+      <c r="P18" s="21">
         <f>IF(D18="","",0.4*0.08*((D18+E18)+(D18+E18)/12+(D18+E18)*4/3/12))</f>
         <v/>
       </c>
-      <c r="Q18" s="18">
+      <c r="Q18" s="21">
         <f>IF(D18="","",F18-MIN(F18,0.06*D18))</f>
         <v/>
       </c>
-      <c r="R18" s="18">
+      <c r="R18" s="21">
         <f>IF(D18="","",G18-G18*H18)</f>
         <v/>
       </c>
-      <c r="S18" s="19">
+      <c r="S18" s="22">
         <f>IF(D18="","",D18+E18+J18+K18+L18+M18+N18+O18+P18+Q18+R18+I18)</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="12" t="n"/>
-      <c r="B19" s="12" t="n"/>
-      <c r="C19" s="12" t="n"/>
-      <c r="D19" s="13" t="n"/>
-      <c r="E19" s="13" t="n"/>
-      <c r="F19" s="13" t="n"/>
-      <c r="G19" s="13" t="n"/>
-      <c r="H19" s="17" t="n"/>
-      <c r="I19" s="13" t="n"/>
-      <c r="J19" s="18">
+      <c r="A19" s="15" t="n"/>
+      <c r="B19" s="15" t="n"/>
+      <c r="C19" s="15" t="n"/>
+      <c r="D19" s="16" t="n"/>
+      <c r="E19" s="16" t="n"/>
+      <c r="F19" s="16" t="n"/>
+      <c r="G19" s="16" t="n"/>
+      <c r="H19" s="20" t="n"/>
+      <c r="I19" s="16" t="n"/>
+      <c r="J19" s="21">
         <f>IF(D19="","",IF(UPPER(C19)="SIMPLES",0,0.2*((D19+E19)+(D19+E19)/12+(D19+E19)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="K19" s="18">
+      <c r="K19" s="21">
         <f>IF(D19="","",IF(UPPER(C19)="SIMPLES",0,$B$2*((D19+E19)+(D19+E19)/12+(D19+E19)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="L19" s="18">
+      <c r="L19" s="21">
         <f>IF(D19="","",IF(UPPER(C19)="SIMPLES",0,$D$2*((D19+E19)+(D19+E19)/12+(D19+E19)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="M19" s="18">
+      <c r="M19" s="21">
         <f>IF(D19="","",0.08*((D19+E19)+(D19+E19)/12+(D19+E19)*4/3/12))</f>
         <v/>
       </c>
-      <c r="N19" s="18">
+      <c r="N19" s="21">
         <f>IF(D19="","",(D19+E19)/12)</f>
         <v/>
       </c>
-      <c r="O19" s="18">
+      <c r="O19" s="21">
         <f>IF(D19="","",(D19+E19)*4/3/12)</f>
         <v/>
       </c>
-      <c r="P19" s="18">
+      <c r="P19" s="21">
         <f>IF(D19="","",0.4*0.08*((D19+E19)+(D19+E19)/12+(D19+E19)*4/3/12))</f>
         <v/>
       </c>
-      <c r="Q19" s="18">
+      <c r="Q19" s="21">
         <f>IF(D19="","",F19-MIN(F19,0.06*D19))</f>
         <v/>
       </c>
-      <c r="R19" s="18">
+      <c r="R19" s="21">
         <f>IF(D19="","",G19-G19*H19)</f>
         <v/>
       </c>
-      <c r="S19" s="19">
+      <c r="S19" s="22">
         <f>IF(D19="","",D19+E19+J19+K19+L19+M19+N19+O19+P19+Q19+R19+I19)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="12" t="n"/>
-      <c r="B20" s="12" t="n"/>
-      <c r="C20" s="12" t="n"/>
-      <c r="D20" s="13" t="n"/>
-      <c r="E20" s="13" t="n"/>
-      <c r="F20" s="13" t="n"/>
-      <c r="G20" s="13" t="n"/>
-      <c r="H20" s="17" t="n"/>
-      <c r="I20" s="13" t="n"/>
-      <c r="J20" s="18">
+      <c r="A20" s="15" t="n"/>
+      <c r="B20" s="15" t="n"/>
+      <c r="C20" s="15" t="n"/>
+      <c r="D20" s="16" t="n"/>
+      <c r="E20" s="16" t="n"/>
+      <c r="F20" s="16" t="n"/>
+      <c r="G20" s="16" t="n"/>
+      <c r="H20" s="20" t="n"/>
+      <c r="I20" s="16" t="n"/>
+      <c r="J20" s="21">
         <f>IF(D20="","",IF(UPPER(C20)="SIMPLES",0,0.2*((D20+E20)+(D20+E20)/12+(D20+E20)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="K20" s="18">
+      <c r="K20" s="21">
         <f>IF(D20="","",IF(UPPER(C20)="SIMPLES",0,$B$2*((D20+E20)+(D20+E20)/12+(D20+E20)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="L20" s="18">
+      <c r="L20" s="21">
         <f>IF(D20="","",IF(UPPER(C20)="SIMPLES",0,$D$2*((D20+E20)+(D20+E20)/12+(D20+E20)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="M20" s="18">
+      <c r="M20" s="21">
         <f>IF(D20="","",0.08*((D20+E20)+(D20+E20)/12+(D20+E20)*4/3/12))</f>
         <v/>
       </c>
-      <c r="N20" s="18">
+      <c r="N20" s="21">
         <f>IF(D20="","",(D20+E20)/12)</f>
         <v/>
       </c>
-      <c r="O20" s="18">
+      <c r="O20" s="21">
         <f>IF(D20="","",(D20+E20)*4/3/12)</f>
         <v/>
       </c>
-      <c r="P20" s="18">
+      <c r="P20" s="21">
         <f>IF(D20="","",0.4*0.08*((D20+E20)+(D20+E20)/12+(D20+E20)*4/3/12))</f>
         <v/>
       </c>
-      <c r="Q20" s="18">
+      <c r="Q20" s="21">
         <f>IF(D20="","",F20-MIN(F20,0.06*D20))</f>
         <v/>
       </c>
-      <c r="R20" s="18">
+      <c r="R20" s="21">
         <f>IF(D20="","",G20-G20*H20)</f>
         <v/>
       </c>
-      <c r="S20" s="19">
+      <c r="S20" s="22">
         <f>IF(D20="","",D20+E20+J20+K20+L20+M20+N20+O20+P20+Q20+R20+I20)</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="12" t="n"/>
-      <c r="B21" s="12" t="n"/>
-      <c r="C21" s="12" t="n"/>
-      <c r="D21" s="13" t="n"/>
-      <c r="E21" s="13" t="n"/>
-      <c r="F21" s="13" t="n"/>
-      <c r="G21" s="13" t="n"/>
-      <c r="H21" s="17" t="n"/>
-      <c r="I21" s="13" t="n"/>
-      <c r="J21" s="18">
+      <c r="A21" s="15" t="n"/>
+      <c r="B21" s="15" t="n"/>
+      <c r="C21" s="15" t="n"/>
+      <c r="D21" s="16" t="n"/>
+      <c r="E21" s="16" t="n"/>
+      <c r="F21" s="16" t="n"/>
+      <c r="G21" s="16" t="n"/>
+      <c r="H21" s="20" t="n"/>
+      <c r="I21" s="16" t="n"/>
+      <c r="J21" s="21">
         <f>IF(D21="","",IF(UPPER(C21)="SIMPLES",0,0.2*((D21+E21)+(D21+E21)/12+(D21+E21)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="K21" s="18">
+      <c r="K21" s="21">
         <f>IF(D21="","",IF(UPPER(C21)="SIMPLES",0,$B$2*((D21+E21)+(D21+E21)/12+(D21+E21)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="L21" s="18">
+      <c r="L21" s="21">
         <f>IF(D21="","",IF(UPPER(C21)="SIMPLES",0,$D$2*((D21+E21)+(D21+E21)/12+(D21+E21)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="M21" s="18">
+      <c r="M21" s="21">
         <f>IF(D21="","",0.08*((D21+E21)+(D21+E21)/12+(D21+E21)*4/3/12))</f>
         <v/>
       </c>
-      <c r="N21" s="18">
+      <c r="N21" s="21">
         <f>IF(D21="","",(D21+E21)/12)</f>
         <v/>
       </c>
-      <c r="O21" s="18">
+      <c r="O21" s="21">
         <f>IF(D21="","",(D21+E21)*4/3/12)</f>
         <v/>
       </c>
-      <c r="P21" s="18">
+      <c r="P21" s="21">
         <f>IF(D21="","",0.4*0.08*((D21+E21)+(D21+E21)/12+(D21+E21)*4/3/12))</f>
         <v/>
       </c>
-      <c r="Q21" s="18">
+      <c r="Q21" s="21">
         <f>IF(D21="","",F21-MIN(F21,0.06*D21))</f>
         <v/>
       </c>
-      <c r="R21" s="18">
+      <c r="R21" s="21">
         <f>IF(D21="","",G21-G21*H21)</f>
         <v/>
       </c>
-      <c r="S21" s="19">
+      <c r="S21" s="22">
         <f>IF(D21="","",D21+E21+J21+K21+L21+M21+N21+O21+P21+Q21+R21+I21)</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="12" t="n"/>
-      <c r="B22" s="12" t="n"/>
-      <c r="C22" s="12" t="n"/>
-      <c r="D22" s="13" t="n"/>
-      <c r="E22" s="13" t="n"/>
-      <c r="F22" s="13" t="n"/>
-      <c r="G22" s="13" t="n"/>
-      <c r="H22" s="17" t="n"/>
-      <c r="I22" s="13" t="n"/>
-      <c r="J22" s="18">
+      <c r="A22" s="15" t="n"/>
+      <c r="B22" s="15" t="n"/>
+      <c r="C22" s="15" t="n"/>
+      <c r="D22" s="16" t="n"/>
+      <c r="E22" s="16" t="n"/>
+      <c r="F22" s="16" t="n"/>
+      <c r="G22" s="16" t="n"/>
+      <c r="H22" s="20" t="n"/>
+      <c r="I22" s="16" t="n"/>
+      <c r="J22" s="21">
         <f>IF(D22="","",IF(UPPER(C22)="SIMPLES",0,0.2*((D22+E22)+(D22+E22)/12+(D22+E22)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="K22" s="18">
+      <c r="K22" s="21">
         <f>IF(D22="","",IF(UPPER(C22)="SIMPLES",0,$B$2*((D22+E22)+(D22+E22)/12+(D22+E22)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="L22" s="18">
+      <c r="L22" s="21">
         <f>IF(D22="","",IF(UPPER(C22)="SIMPLES",0,$D$2*((D22+E22)+(D22+E22)/12+(D22+E22)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="M22" s="18">
+      <c r="M22" s="21">
         <f>IF(D22="","",0.08*((D22+E22)+(D22+E22)/12+(D22+E22)*4/3/12))</f>
         <v/>
       </c>
-      <c r="N22" s="18">
+      <c r="N22" s="21">
         <f>IF(D22="","",(D22+E22)/12)</f>
         <v/>
       </c>
-      <c r="O22" s="18">
+      <c r="O22" s="21">
         <f>IF(D22="","",(D22+E22)*4/3/12)</f>
         <v/>
       </c>
-      <c r="P22" s="18">
+      <c r="P22" s="21">
         <f>IF(D22="","",0.4*0.08*((D22+E22)+(D22+E22)/12+(D22+E22)*4/3/12))</f>
         <v/>
       </c>
-      <c r="Q22" s="18">
+      <c r="Q22" s="21">
         <f>IF(D22="","",F22-MIN(F22,0.06*D22))</f>
         <v/>
       </c>
-      <c r="R22" s="18">
+      <c r="R22" s="21">
         <f>IF(D22="","",G22-G22*H22)</f>
         <v/>
       </c>
-      <c r="S22" s="19">
+      <c r="S22" s="22">
         <f>IF(D22="","",D22+E22+J22+K22+L22+M22+N22+O22+P22+Q22+R22+I22)</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="12" t="n"/>
-      <c r="B23" s="12" t="n"/>
-      <c r="C23" s="12" t="n"/>
-      <c r="D23" s="13" t="n"/>
-      <c r="E23" s="13" t="n"/>
-      <c r="F23" s="13" t="n"/>
-      <c r="G23" s="13" t="n"/>
-      <c r="H23" s="17" t="n"/>
-      <c r="I23" s="13" t="n"/>
-      <c r="J23" s="18">
+      <c r="A23" s="15" t="n"/>
+      <c r="B23" s="15" t="n"/>
+      <c r="C23" s="15" t="n"/>
+      <c r="D23" s="16" t="n"/>
+      <c r="E23" s="16" t="n"/>
+      <c r="F23" s="16" t="n"/>
+      <c r="G23" s="16" t="n"/>
+      <c r="H23" s="20" t="n"/>
+      <c r="I23" s="16" t="n"/>
+      <c r="J23" s="21">
         <f>IF(D23="","",IF(UPPER(C23)="SIMPLES",0,0.2*((D23+E23)+(D23+E23)/12+(D23+E23)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="K23" s="18">
+      <c r="K23" s="21">
         <f>IF(D23="","",IF(UPPER(C23)="SIMPLES",0,$B$2*((D23+E23)+(D23+E23)/12+(D23+E23)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="L23" s="18">
+      <c r="L23" s="21">
         <f>IF(D23="","",IF(UPPER(C23)="SIMPLES",0,$D$2*((D23+E23)+(D23+E23)/12+(D23+E23)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="M23" s="18">
+      <c r="M23" s="21">
         <f>IF(D23="","",0.08*((D23+E23)+(D23+E23)/12+(D23+E23)*4/3/12))</f>
         <v/>
       </c>
-      <c r="N23" s="18">
+      <c r="N23" s="21">
         <f>IF(D23="","",(D23+E23)/12)</f>
         <v/>
       </c>
-      <c r="O23" s="18">
+      <c r="O23" s="21">
         <f>IF(D23="","",(D23+E23)*4/3/12)</f>
         <v/>
       </c>
-      <c r="P23" s="18">
+      <c r="P23" s="21">
         <f>IF(D23="","",0.4*0.08*((D23+E23)+(D23+E23)/12+(D23+E23)*4/3/12))</f>
         <v/>
       </c>
-      <c r="Q23" s="18">
+      <c r="Q23" s="21">
         <f>IF(D23="","",F23-MIN(F23,0.06*D23))</f>
         <v/>
       </c>
-      <c r="R23" s="18">
+      <c r="R23" s="21">
         <f>IF(D23="","",G23-G23*H23)</f>
         <v/>
       </c>
-      <c r="S23" s="19">
+      <c r="S23" s="22">
         <f>IF(D23="","",D23+E23+J23+K23+L23+M23+N23+O23+P23+Q23+R23+I23)</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="12" t="n"/>
-      <c r="B24" s="12" t="n"/>
-      <c r="C24" s="12" t="n"/>
-      <c r="D24" s="13" t="n"/>
-      <c r="E24" s="13" t="n"/>
-      <c r="F24" s="13" t="n"/>
-      <c r="G24" s="13" t="n"/>
-      <c r="H24" s="17" t="n"/>
-      <c r="I24" s="13" t="n"/>
-      <c r="J24" s="18">
+      <c r="A24" s="15" t="n"/>
+      <c r="B24" s="15" t="n"/>
+      <c r="C24" s="15" t="n"/>
+      <c r="D24" s="16" t="n"/>
+      <c r="E24" s="16" t="n"/>
+      <c r="F24" s="16" t="n"/>
+      <c r="G24" s="16" t="n"/>
+      <c r="H24" s="20" t="n"/>
+      <c r="I24" s="16" t="n"/>
+      <c r="J24" s="21">
         <f>IF(D24="","",IF(UPPER(C24)="SIMPLES",0,0.2*((D24+E24)+(D24+E24)/12+(D24+E24)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="K24" s="18">
+      <c r="K24" s="21">
         <f>IF(D24="","",IF(UPPER(C24)="SIMPLES",0,$B$2*((D24+E24)+(D24+E24)/12+(D24+E24)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="L24" s="18">
+      <c r="L24" s="21">
         <f>IF(D24="","",IF(UPPER(C24)="SIMPLES",0,$D$2*((D24+E24)+(D24+E24)/12+(D24+E24)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="M24" s="18">
+      <c r="M24" s="21">
         <f>IF(D24="","",0.08*((D24+E24)+(D24+E24)/12+(D24+E24)*4/3/12))</f>
         <v/>
       </c>
-      <c r="N24" s="18">
+      <c r="N24" s="21">
         <f>IF(D24="","",(D24+E24)/12)</f>
         <v/>
       </c>
-      <c r="O24" s="18">
+      <c r="O24" s="21">
         <f>IF(D24="","",(D24+E24)*4/3/12)</f>
         <v/>
       </c>
-      <c r="P24" s="18">
+      <c r="P24" s="21">
         <f>IF(D24="","",0.4*0.08*((D24+E24)+(D24+E24)/12+(D24+E24)*4/3/12))</f>
         <v/>
       </c>
-      <c r="Q24" s="18">
+      <c r="Q24" s="21">
         <f>IF(D24="","",F24-MIN(F24,0.06*D24))</f>
         <v/>
       </c>
-      <c r="R24" s="18">
+      <c r="R24" s="21">
         <f>IF(D24="","",G24-G24*H24)</f>
         <v/>
       </c>
-      <c r="S24" s="19">
+      <c r="S24" s="22">
         <f>IF(D24="","",D24+E24+J24+K24+L24+M24+N24+O24+P24+Q24+R24+I24)</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="12" t="n"/>
-      <c r="B25" s="12" t="n"/>
-      <c r="C25" s="12" t="n"/>
-      <c r="D25" s="13" t="n"/>
-      <c r="E25" s="13" t="n"/>
-      <c r="F25" s="13" t="n"/>
-      <c r="G25" s="13" t="n"/>
-      <c r="H25" s="17" t="n"/>
-      <c r="I25" s="13" t="n"/>
-      <c r="J25" s="18">
+      <c r="A25" s="15" t="n"/>
+      <c r="B25" s="15" t="n"/>
+      <c r="C25" s="15" t="n"/>
+      <c r="D25" s="16" t="n"/>
+      <c r="E25" s="16" t="n"/>
+      <c r="F25" s="16" t="n"/>
+      <c r="G25" s="16" t="n"/>
+      <c r="H25" s="20" t="n"/>
+      <c r="I25" s="16" t="n"/>
+      <c r="J25" s="21">
         <f>IF(D25="","",IF(UPPER(C25)="SIMPLES",0,0.2*((D25+E25)+(D25+E25)/12+(D25+E25)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="K25" s="18">
+      <c r="K25" s="21">
         <f>IF(D25="","",IF(UPPER(C25)="SIMPLES",0,$B$2*((D25+E25)+(D25+E25)/12+(D25+E25)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="L25" s="18">
+      <c r="L25" s="21">
         <f>IF(D25="","",IF(UPPER(C25)="SIMPLES",0,$D$2*((D25+E25)+(D25+E25)/12+(D25+E25)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="M25" s="18">
+      <c r="M25" s="21">
         <f>IF(D25="","",0.08*((D25+E25)+(D25+E25)/12+(D25+E25)*4/3/12))</f>
         <v/>
       </c>
-      <c r="N25" s="18">
+      <c r="N25" s="21">
         <f>IF(D25="","",(D25+E25)/12)</f>
         <v/>
       </c>
-      <c r="O25" s="18">
+      <c r="O25" s="21">
         <f>IF(D25="","",(D25+E25)*4/3/12)</f>
         <v/>
       </c>
-      <c r="P25" s="18">
+      <c r="P25" s="21">
         <f>IF(D25="","",0.4*0.08*((D25+E25)+(D25+E25)/12+(D25+E25)*4/3/12))</f>
         <v/>
       </c>
-      <c r="Q25" s="18">
+      <c r="Q25" s="21">
         <f>IF(D25="","",F25-MIN(F25,0.06*D25))</f>
         <v/>
       </c>
-      <c r="R25" s="18">
+      <c r="R25" s="21">
         <f>IF(D25="","",G25-G25*H25)</f>
         <v/>
       </c>
-      <c r="S25" s="19">
+      <c r="S25" s="22">
         <f>IF(D25="","",D25+E25+J25+K25+L25+M25+N25+O25+P25+Q25+R25+I25)</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="12" t="n"/>
-      <c r="B26" s="12" t="n"/>
-      <c r="C26" s="12" t="n"/>
-      <c r="D26" s="13" t="n"/>
-      <c r="E26" s="13" t="n"/>
-      <c r="F26" s="13" t="n"/>
-      <c r="G26" s="13" t="n"/>
-      <c r="H26" s="17" t="n"/>
-      <c r="I26" s="13" t="n"/>
-      <c r="J26" s="18">
+      <c r="A26" s="15" t="n"/>
+      <c r="B26" s="15" t="n"/>
+      <c r="C26" s="15" t="n"/>
+      <c r="D26" s="16" t="n"/>
+      <c r="E26" s="16" t="n"/>
+      <c r="F26" s="16" t="n"/>
+      <c r="G26" s="16" t="n"/>
+      <c r="H26" s="20" t="n"/>
+      <c r="I26" s="16" t="n"/>
+      <c r="J26" s="21">
         <f>IF(D26="","",IF(UPPER(C26)="SIMPLES",0,0.2*((D26+E26)+(D26+E26)/12+(D26+E26)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="K26" s="18">
+      <c r="K26" s="21">
         <f>IF(D26="","",IF(UPPER(C26)="SIMPLES",0,$B$2*((D26+E26)+(D26+E26)/12+(D26+E26)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="L26" s="18">
+      <c r="L26" s="21">
         <f>IF(D26="","",IF(UPPER(C26)="SIMPLES",0,$D$2*((D26+E26)+(D26+E26)/12+(D26+E26)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="M26" s="18">
+      <c r="M26" s="21">
         <f>IF(D26="","",0.08*((D26+E26)+(D26+E26)/12+(D26+E26)*4/3/12))</f>
         <v/>
       </c>
-      <c r="N26" s="18">
+      <c r="N26" s="21">
         <f>IF(D26="","",(D26+E26)/12)</f>
         <v/>
       </c>
-      <c r="O26" s="18">
+      <c r="O26" s="21">
         <f>IF(D26="","",(D26+E26)*4/3/12)</f>
         <v/>
       </c>
-      <c r="P26" s="18">
+      <c r="P26" s="21">
         <f>IF(D26="","",0.4*0.08*((D26+E26)+(D26+E26)/12+(D26+E26)*4/3/12))</f>
         <v/>
       </c>
-      <c r="Q26" s="18">
+      <c r="Q26" s="21">
         <f>IF(D26="","",F26-MIN(F26,0.06*D26))</f>
         <v/>
       </c>
-      <c r="R26" s="18">
+      <c r="R26" s="21">
         <f>IF(D26="","",G26-G26*H26)</f>
         <v/>
       </c>
-      <c r="S26" s="19">
+      <c r="S26" s="22">
         <f>IF(D26="","",D26+E26+J26+K26+L26+M26+N26+O26+P26+Q26+R26+I26)</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="12" t="n"/>
-      <c r="B27" s="12" t="n"/>
-      <c r="C27" s="12" t="n"/>
-      <c r="D27" s="13" t="n"/>
-      <c r="E27" s="13" t="n"/>
-      <c r="F27" s="13" t="n"/>
-      <c r="G27" s="13" t="n"/>
-      <c r="H27" s="17" t="n"/>
-      <c r="I27" s="13" t="n"/>
-      <c r="J27" s="18">
+      <c r="A27" s="15" t="n"/>
+      <c r="B27" s="15" t="n"/>
+      <c r="C27" s="15" t="n"/>
+      <c r="D27" s="16" t="n"/>
+      <c r="E27" s="16" t="n"/>
+      <c r="F27" s="16" t="n"/>
+      <c r="G27" s="16" t="n"/>
+      <c r="H27" s="20" t="n"/>
+      <c r="I27" s="16" t="n"/>
+      <c r="J27" s="21">
         <f>IF(D27="","",IF(UPPER(C27)="SIMPLES",0,0.2*((D27+E27)+(D27+E27)/12+(D27+E27)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="K27" s="18">
+      <c r="K27" s="21">
         <f>IF(D27="","",IF(UPPER(C27)="SIMPLES",0,$B$2*((D27+E27)+(D27+E27)/12+(D27+E27)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="L27" s="18">
+      <c r="L27" s="21">
         <f>IF(D27="","",IF(UPPER(C27)="SIMPLES",0,$D$2*((D27+E27)+(D27+E27)/12+(D27+E27)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="M27" s="18">
+      <c r="M27" s="21">
         <f>IF(D27="","",0.08*((D27+E27)+(D27+E27)/12+(D27+E27)*4/3/12))</f>
         <v/>
       </c>
-      <c r="N27" s="18">
+      <c r="N27" s="21">
         <f>IF(D27="","",(D27+E27)/12)</f>
         <v/>
       </c>
-      <c r="O27" s="18">
+      <c r="O27" s="21">
         <f>IF(D27="","",(D27+E27)*4/3/12)</f>
         <v/>
       </c>
-      <c r="P27" s="18">
+      <c r="P27" s="21">
         <f>IF(D27="","",0.4*0.08*((D27+E27)+(D27+E27)/12+(D27+E27)*4/3/12))</f>
         <v/>
       </c>
-      <c r="Q27" s="18">
+      <c r="Q27" s="21">
         <f>IF(D27="","",F27-MIN(F27,0.06*D27))</f>
         <v/>
       </c>
-      <c r="R27" s="18">
+      <c r="R27" s="21">
         <f>IF(D27="","",G27-G27*H27)</f>
         <v/>
       </c>
-      <c r="S27" s="19">
+      <c r="S27" s="22">
         <f>IF(D27="","",D27+E27+J27+K27+L27+M27+N27+O27+P27+Q27+R27+I27)</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="12" t="n"/>
-      <c r="B28" s="12" t="n"/>
-      <c r="C28" s="12" t="n"/>
-      <c r="D28" s="13" t="n"/>
-      <c r="E28" s="13" t="n"/>
-      <c r="F28" s="13" t="n"/>
-      <c r="G28" s="13" t="n"/>
-      <c r="H28" s="17" t="n"/>
-      <c r="I28" s="13" t="n"/>
-      <c r="J28" s="18">
+      <c r="A28" s="15" t="n"/>
+      <c r="B28" s="15" t="n"/>
+      <c r="C28" s="15" t="n"/>
+      <c r="D28" s="16" t="n"/>
+      <c r="E28" s="16" t="n"/>
+      <c r="F28" s="16" t="n"/>
+      <c r="G28" s="16" t="n"/>
+      <c r="H28" s="20" t="n"/>
+      <c r="I28" s="16" t="n"/>
+      <c r="J28" s="21">
         <f>IF(D28="","",IF(UPPER(C28)="SIMPLES",0,0.2*((D28+E28)+(D28+E28)/12+(D28+E28)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="K28" s="18">
+      <c r="K28" s="21">
         <f>IF(D28="","",IF(UPPER(C28)="SIMPLES",0,$B$2*((D28+E28)+(D28+E28)/12+(D28+E28)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="L28" s="18">
+      <c r="L28" s="21">
         <f>IF(D28="","",IF(UPPER(C28)="SIMPLES",0,$D$2*((D28+E28)+(D28+E28)/12+(D28+E28)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="M28" s="18">
+      <c r="M28" s="21">
         <f>IF(D28="","",0.08*((D28+E28)+(D28+E28)/12+(D28+E28)*4/3/12))</f>
         <v/>
       </c>
-      <c r="N28" s="18">
+      <c r="N28" s="21">
         <f>IF(D28="","",(D28+E28)/12)</f>
         <v/>
       </c>
-      <c r="O28" s="18">
+      <c r="O28" s="21">
         <f>IF(D28="","",(D28+E28)*4/3/12)</f>
         <v/>
       </c>
-      <c r="P28" s="18">
+      <c r="P28" s="21">
         <f>IF(D28="","",0.4*0.08*((D28+E28)+(D28+E28)/12+(D28+E28)*4/3/12))</f>
         <v/>
       </c>
-      <c r="Q28" s="18">
+      <c r="Q28" s="21">
         <f>IF(D28="","",F28-MIN(F28,0.06*D28))</f>
         <v/>
       </c>
-      <c r="R28" s="18">
+      <c r="R28" s="21">
         <f>IF(D28="","",G28-G28*H28)</f>
         <v/>
       </c>
-      <c r="S28" s="19">
+      <c r="S28" s="22">
         <f>IF(D28="","",D28+E28+J28+K28+L28+M28+N28+O28+P28+Q28+R28+I28)</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="12" t="n"/>
-      <c r="B29" s="12" t="n"/>
-      <c r="C29" s="12" t="n"/>
-      <c r="D29" s="13" t="n"/>
-      <c r="E29" s="13" t="n"/>
-      <c r="F29" s="13" t="n"/>
-      <c r="G29" s="13" t="n"/>
-      <c r="H29" s="17" t="n"/>
-      <c r="I29" s="13" t="n"/>
-      <c r="J29" s="18">
+      <c r="A29" s="15" t="n"/>
+      <c r="B29" s="15" t="n"/>
+      <c r="C29" s="15" t="n"/>
+      <c r="D29" s="16" t="n"/>
+      <c r="E29" s="16" t="n"/>
+      <c r="F29" s="16" t="n"/>
+      <c r="G29" s="16" t="n"/>
+      <c r="H29" s="20" t="n"/>
+      <c r="I29" s="16" t="n"/>
+      <c r="J29" s="21">
         <f>IF(D29="","",IF(UPPER(C29)="SIMPLES",0,0.2*((D29+E29)+(D29+E29)/12+(D29+E29)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="K29" s="18">
+      <c r="K29" s="21">
         <f>IF(D29="","",IF(UPPER(C29)="SIMPLES",0,$B$2*((D29+E29)+(D29+E29)/12+(D29+E29)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="L29" s="18">
+      <c r="L29" s="21">
         <f>IF(D29="","",IF(UPPER(C29)="SIMPLES",0,$D$2*((D29+E29)+(D29+E29)/12+(D29+E29)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="M29" s="18">
+      <c r="M29" s="21">
         <f>IF(D29="","",0.08*((D29+E29)+(D29+E29)/12+(D29+E29)*4/3/12))</f>
         <v/>
       </c>
-      <c r="N29" s="18">
+      <c r="N29" s="21">
         <f>IF(D29="","",(D29+E29)/12)</f>
         <v/>
       </c>
-      <c r="O29" s="18">
+      <c r="O29" s="21">
         <f>IF(D29="","",(D29+E29)*4/3/12)</f>
         <v/>
       </c>
-      <c r="P29" s="18">
+      <c r="P29" s="21">
         <f>IF(D29="","",0.4*0.08*((D29+E29)+(D29+E29)/12+(D29+E29)*4/3/12))</f>
         <v/>
       </c>
-      <c r="Q29" s="18">
+      <c r="Q29" s="21">
         <f>IF(D29="","",F29-MIN(F29,0.06*D29))</f>
         <v/>
       </c>
-      <c r="R29" s="18">
+      <c r="R29" s="21">
         <f>IF(D29="","",G29-G29*H29)</f>
         <v/>
       </c>
-      <c r="S29" s="19">
+      <c r="S29" s="22">
         <f>IF(D29="","",D29+E29+J29+K29+L29+M29+N29+O29+P29+Q29+R29+I29)</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="12" t="n"/>
-      <c r="B30" s="12" t="n"/>
-      <c r="C30" s="12" t="n"/>
-      <c r="D30" s="13" t="n"/>
-      <c r="E30" s="13" t="n"/>
-      <c r="F30" s="13" t="n"/>
-      <c r="G30" s="13" t="n"/>
-      <c r="H30" s="17" t="n"/>
-      <c r="I30" s="13" t="n"/>
-      <c r="J30" s="18">
+      <c r="A30" s="15" t="n"/>
+      <c r="B30" s="15" t="n"/>
+      <c r="C30" s="15" t="n"/>
+      <c r="D30" s="16" t="n"/>
+      <c r="E30" s="16" t="n"/>
+      <c r="F30" s="16" t="n"/>
+      <c r="G30" s="16" t="n"/>
+      <c r="H30" s="20" t="n"/>
+      <c r="I30" s="16" t="n"/>
+      <c r="J30" s="21">
         <f>IF(D30="","",IF(UPPER(C30)="SIMPLES",0,0.2*((D30+E30)+(D30+E30)/12+(D30+E30)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="K30" s="18">
+      <c r="K30" s="21">
         <f>IF(D30="","",IF(UPPER(C30)="SIMPLES",0,$B$2*((D30+E30)+(D30+E30)/12+(D30+E30)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="L30" s="18">
+      <c r="L30" s="21">
         <f>IF(D30="","",IF(UPPER(C30)="SIMPLES",0,$D$2*((D30+E30)+(D30+E30)/12+(D30+E30)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="M30" s="18">
+      <c r="M30" s="21">
         <f>IF(D30="","",0.08*((D30+E30)+(D30+E30)/12+(D30+E30)*4/3/12))</f>
         <v/>
       </c>
-      <c r="N30" s="18">
+      <c r="N30" s="21">
         <f>IF(D30="","",(D30+E30)/12)</f>
         <v/>
       </c>
-      <c r="O30" s="18">
+      <c r="O30" s="21">
         <f>IF(D30="","",(D30+E30)*4/3/12)</f>
         <v/>
       </c>
-      <c r="P30" s="18">
+      <c r="P30" s="21">
         <f>IF(D30="","",0.4*0.08*((D30+E30)+(D30+E30)/12+(D30+E30)*4/3/12))</f>
         <v/>
       </c>
-      <c r="Q30" s="18">
+      <c r="Q30" s="21">
         <f>IF(D30="","",F30-MIN(F30,0.06*D30))</f>
         <v/>
       </c>
-      <c r="R30" s="18">
+      <c r="R30" s="21">
         <f>IF(D30="","",G30-G30*H30)</f>
         <v/>
       </c>
-      <c r="S30" s="19">
+      <c r="S30" s="22">
         <f>IF(D30="","",D30+E30+J30+K30+L30+M30+N30+O30+P30+Q30+R30+I30)</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="12" t="n"/>
-      <c r="B31" s="12" t="n"/>
-      <c r="C31" s="12" t="n"/>
-      <c r="D31" s="13" t="n"/>
-      <c r="E31" s="13" t="n"/>
-      <c r="F31" s="13" t="n"/>
-      <c r="G31" s="13" t="n"/>
-      <c r="H31" s="17" t="n"/>
-      <c r="I31" s="13" t="n"/>
-      <c r="J31" s="18">
+      <c r="A31" s="15" t="n"/>
+      <c r="B31" s="15" t="n"/>
+      <c r="C31" s="15" t="n"/>
+      <c r="D31" s="16" t="n"/>
+      <c r="E31" s="16" t="n"/>
+      <c r="F31" s="16" t="n"/>
+      <c r="G31" s="16" t="n"/>
+      <c r="H31" s="20" t="n"/>
+      <c r="I31" s="16" t="n"/>
+      <c r="J31" s="21">
         <f>IF(D31="","",IF(UPPER(C31)="SIMPLES",0,0.2*((D31+E31)+(D31+E31)/12+(D31+E31)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="K31" s="18">
+      <c r="K31" s="21">
         <f>IF(D31="","",IF(UPPER(C31)="SIMPLES",0,$B$2*((D31+E31)+(D31+E31)/12+(D31+E31)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="L31" s="18">
+      <c r="L31" s="21">
         <f>IF(D31="","",IF(UPPER(C31)="SIMPLES",0,$D$2*((D31+E31)+(D31+E31)/12+(D31+E31)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="M31" s="18">
+      <c r="M31" s="21">
         <f>IF(D31="","",0.08*((D31+E31)+(D31+E31)/12+(D31+E31)*4/3/12))</f>
         <v/>
       </c>
-      <c r="N31" s="18">
+      <c r="N31" s="21">
         <f>IF(D31="","",(D31+E31)/12)</f>
         <v/>
       </c>
-      <c r="O31" s="18">
+      <c r="O31" s="21">
         <f>IF(D31="","",(D31+E31)*4/3/12)</f>
         <v/>
       </c>
-      <c r="P31" s="18">
+      <c r="P31" s="21">
         <f>IF(D31="","",0.4*0.08*((D31+E31)+(D31+E31)/12+(D31+E31)*4/3/12))</f>
         <v/>
       </c>
-      <c r="Q31" s="18">
+      <c r="Q31" s="21">
         <f>IF(D31="","",F31-MIN(F31,0.06*D31))</f>
         <v/>
       </c>
-      <c r="R31" s="18">
+      <c r="R31" s="21">
         <f>IF(D31="","",G31-G31*H31)</f>
         <v/>
       </c>
-      <c r="S31" s="19">
+      <c r="S31" s="22">
         <f>IF(D31="","",D31+E31+J31+K31+L31+M31+N31+O31+P31+Q31+R31+I31)</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="12" t="n"/>
-      <c r="B32" s="12" t="n"/>
-      <c r="C32" s="12" t="n"/>
-      <c r="D32" s="13" t="n"/>
-      <c r="E32" s="13" t="n"/>
-      <c r="F32" s="13" t="n"/>
-      <c r="G32" s="13" t="n"/>
-      <c r="H32" s="17" t="n"/>
-      <c r="I32" s="13" t="n"/>
-      <c r="J32" s="18">
+      <c r="A32" s="15" t="n"/>
+      <c r="B32" s="15" t="n"/>
+      <c r="C32" s="15" t="n"/>
+      <c r="D32" s="16" t="n"/>
+      <c r="E32" s="16" t="n"/>
+      <c r="F32" s="16" t="n"/>
+      <c r="G32" s="16" t="n"/>
+      <c r="H32" s="20" t="n"/>
+      <c r="I32" s="16" t="n"/>
+      <c r="J32" s="21">
         <f>IF(D32="","",IF(UPPER(C32)="SIMPLES",0,0.2*((D32+E32)+(D32+E32)/12+(D32+E32)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="K32" s="18">
+      <c r="K32" s="21">
         <f>IF(D32="","",IF(UPPER(C32)="SIMPLES",0,$B$2*((D32+E32)+(D32+E32)/12+(D32+E32)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="L32" s="18">
+      <c r="L32" s="21">
         <f>IF(D32="","",IF(UPPER(C32)="SIMPLES",0,$D$2*((D32+E32)+(D32+E32)/12+(D32+E32)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="M32" s="18">
+      <c r="M32" s="21">
         <f>IF(D32="","",0.08*((D32+E32)+(D32+E32)/12+(D32+E32)*4/3/12))</f>
         <v/>
       </c>
-      <c r="N32" s="18">
+      <c r="N32" s="21">
         <f>IF(D32="","",(D32+E32)/12)</f>
         <v/>
       </c>
-      <c r="O32" s="18">
+      <c r="O32" s="21">
         <f>IF(D32="","",(D32+E32)*4/3/12)</f>
         <v/>
       </c>
-      <c r="P32" s="18">
+      <c r="P32" s="21">
         <f>IF(D32="","",0.4*0.08*((D32+E32)+(D32+E32)/12+(D32+E32)*4/3/12))</f>
         <v/>
       </c>
-      <c r="Q32" s="18">
+      <c r="Q32" s="21">
         <f>IF(D32="","",F32-MIN(F32,0.06*D32))</f>
         <v/>
       </c>
-      <c r="R32" s="18">
+      <c r="R32" s="21">
         <f>IF(D32="","",G32-G32*H32)</f>
         <v/>
       </c>
-      <c r="S32" s="19">
+      <c r="S32" s="22">
         <f>IF(D32="","",D32+E32+J32+K32+L32+M32+N32+O32+P32+Q32+R32+I32)</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="12" t="n"/>
-      <c r="B33" s="12" t="n"/>
-      <c r="C33" s="12" t="n"/>
-      <c r="D33" s="13" t="n"/>
-      <c r="E33" s="13" t="n"/>
-      <c r="F33" s="13" t="n"/>
-      <c r="G33" s="13" t="n"/>
-      <c r="H33" s="17" t="n"/>
-      <c r="I33" s="13" t="n"/>
-      <c r="J33" s="18">
+      <c r="A33" s="15" t="n"/>
+      <c r="B33" s="15" t="n"/>
+      <c r="C33" s="15" t="n"/>
+      <c r="D33" s="16" t="n"/>
+      <c r="E33" s="16" t="n"/>
+      <c r="F33" s="16" t="n"/>
+      <c r="G33" s="16" t="n"/>
+      <c r="H33" s="20" t="n"/>
+      <c r="I33" s="16" t="n"/>
+      <c r="J33" s="21">
         <f>IF(D33="","",IF(UPPER(C33)="SIMPLES",0,0.2*((D33+E33)+(D33+E33)/12+(D33+E33)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="K33" s="18">
+      <c r="K33" s="21">
         <f>IF(D33="","",IF(UPPER(C33)="SIMPLES",0,$B$2*((D33+E33)+(D33+E33)/12+(D33+E33)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="L33" s="18">
+      <c r="L33" s="21">
         <f>IF(D33="","",IF(UPPER(C33)="SIMPLES",0,$D$2*((D33+E33)+(D33+E33)/12+(D33+E33)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="M33" s="18">
+      <c r="M33" s="21">
         <f>IF(D33="","",0.08*((D33+E33)+(D33+E33)/12+(D33+E33)*4/3/12))</f>
         <v/>
       </c>
-      <c r="N33" s="18">
+      <c r="N33" s="21">
         <f>IF(D33="","",(D33+E33)/12)</f>
         <v/>
       </c>
-      <c r="O33" s="18">
+      <c r="O33" s="21">
         <f>IF(D33="","",(D33+E33)*4/3/12)</f>
         <v/>
       </c>
-      <c r="P33" s="18">
+      <c r="P33" s="21">
         <f>IF(D33="","",0.4*0.08*((D33+E33)+(D33+E33)/12+(D33+E33)*4/3/12))</f>
         <v/>
       </c>
-      <c r="Q33" s="18">
+      <c r="Q33" s="21">
         <f>IF(D33="","",F33-MIN(F33,0.06*D33))</f>
         <v/>
       </c>
-      <c r="R33" s="18">
+      <c r="R33" s="21">
         <f>IF(D33="","",G33-G33*H33)</f>
         <v/>
       </c>
-      <c r="S33" s="19">
+      <c r="S33" s="22">
         <f>IF(D33="","",D33+E33+J33+K33+L33+M33+N33+O33+P33+Q33+R33+I33)</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="12" t="n"/>
-      <c r="B34" s="12" t="n"/>
-      <c r="C34" s="12" t="n"/>
-      <c r="D34" s="13" t="n"/>
-      <c r="E34" s="13" t="n"/>
-      <c r="F34" s="13" t="n"/>
-      <c r="G34" s="13" t="n"/>
-      <c r="H34" s="17" t="n"/>
-      <c r="I34" s="13" t="n"/>
-      <c r="J34" s="18">
+      <c r="A34" s="15" t="n"/>
+      <c r="B34" s="15" t="n"/>
+      <c r="C34" s="15" t="n"/>
+      <c r="D34" s="16" t="n"/>
+      <c r="E34" s="16" t="n"/>
+      <c r="F34" s="16" t="n"/>
+      <c r="G34" s="16" t="n"/>
+      <c r="H34" s="20" t="n"/>
+      <c r="I34" s="16" t="n"/>
+      <c r="J34" s="21">
         <f>IF(D34="","",IF(UPPER(C34)="SIMPLES",0,0.2*((D34+E34)+(D34+E34)/12+(D34+E34)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="K34" s="18">
+      <c r="K34" s="21">
         <f>IF(D34="","",IF(UPPER(C34)="SIMPLES",0,$B$2*((D34+E34)+(D34+E34)/12+(D34+E34)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="L34" s="18">
+      <c r="L34" s="21">
         <f>IF(D34="","",IF(UPPER(C34)="SIMPLES",0,$D$2*((D34+E34)+(D34+E34)/12+(D34+E34)*4/3/12)))</f>
         <v/>
       </c>
-      <c r="M34" s="18">
+      <c r="M34" s="21">
         <f>IF(D34="","",0.08*((D34+E34)+(D34+E34)/12+(D34+E34)*4/3/12))</f>
         <v/>
       </c>
-      <c r="N34" s="18">
+      <c r="N34" s="21">
         <f>IF(D34="","",(D34+E34)/12)</f>
         <v/>
       </c>
-      <c r="O34" s="18">
+      <c r="O34" s="21">
         <f>IF(D34="","",(D34+E34)*4/3/12)</f>
         <v/>
       </c>
-      <c r="P34" s="18">
+      <c r="P34" s="21">
         <f>IF(D34="","",0.4*0.08*((D34+E34)+(D34+E34)/12+(D34+E34)*4/3/12))</f>
         <v/>
       </c>
-      <c r="Q34" s="18">
+      <c r="Q34" s="21">
         <f>IF(D34="","",F34-MIN(F34,0.06*D34))</f>
         <v/>
       </c>
-      <c r="R34" s="18">
+      <c r="R34" s="21">
         <f>IF(D34="","",G34-G34*H34)</f>
         <v/>
       </c>
-      <c r="S34" s="19">
+      <c r="S34" s="22">
         <f>IF(D34="","",D34+E34+J34+K34+L34+M34+N34+O34+P34+Q34+R34+I34)</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="10" t="inlineStr"/>
-      <c r="C35" s="10" t="inlineStr">
+      <c r="B35" s="13" t="inlineStr"/>
+      <c r="C35" s="13" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="D35" s="20">
+      <c r="D35" s="23">
         <f>COUNT(D5:D34)</f>
         <v/>
       </c>
-      <c r="E35" s="21">
+      <c r="E35" s="24">
         <f>SUM(E5:E34)</f>
         <v/>
       </c>
-      <c r="I35" s="21">
+      <c r="I35" s="24">
         <f>SUM(I5:I34)</f>
         <v/>
       </c>
-      <c r="J35" s="21">
+      <c r="J35" s="24">
         <f>SUM(J5:J34)</f>
         <v/>
       </c>
-      <c r="K35" s="21">
+      <c r="K35" s="24">
         <f>SUM(K5:K34)</f>
         <v/>
       </c>
-      <c r="L35" s="21">
+      <c r="L35" s="24">
         <f>SUM(L5:L34)</f>
         <v/>
       </c>
-      <c r="M35" s="21">
+      <c r="M35" s="24">
         <f>SUM(M5:M34)</f>
         <v/>
       </c>
-      <c r="N35" s="21">
+      <c r="N35" s="24">
         <f>SUM(N5:N34)</f>
         <v/>
       </c>
-      <c r="O35" s="21">
+      <c r="O35" s="24">
         <f>SUM(O5:O34)</f>
         <v/>
       </c>
-      <c r="P35" s="21">
+      <c r="P35" s="24">
         <f>SUM(P5:P34)</f>
         <v/>
       </c>
-      <c r="Q35" s="21">
+      <c r="Q35" s="24">
         <f>SUM(Q5:Q34)</f>
         <v/>
       </c>
-      <c r="R35" s="21">
+      <c r="R35" s="24">
         <f>SUM(R5:R34)</f>
         <v/>
       </c>
-      <c r="S35" s="21">
+      <c r="S35" s="24">
         <f>SUM(S5:S34)</f>
         <v/>
       </c>
@@ -2882,226 +3044,226 @@
       </c>
     </row>
     <row r="3" ht="26" customHeight="1">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>Cargo</t>
         </is>
       </c>
-      <c r="B3" s="11" t="inlineStr">
+      <c r="B3" s="14" t="inlineStr">
         <is>
           <t>Funcionários</t>
         </is>
       </c>
-      <c r="C3" s="11" t="inlineStr">
+      <c r="C3" s="14" t="inlineStr">
         <is>
           <t>Custo total/mês</t>
         </is>
       </c>
-      <c r="D3" s="11" t="inlineStr">
+      <c r="D3" s="14" t="inlineStr">
         <is>
           <t>Custo médio</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>Vendedor</t>
         </is>
       </c>
-      <c r="B4" s="22">
+      <c r="B4" s="25">
         <f>IF(A4="","",COUNTIF('Funcionários'!$A$5:$A$34,A4))</f>
         <v/>
       </c>
-      <c r="C4" s="13">
+      <c r="C4" s="16">
         <f>IF(A4="","",SUMIF('Funcionários'!$A$5:$A$34,A4,'Funcionários'!$S$5:$S$34))</f>
         <v/>
       </c>
-      <c r="D4" s="13">
+      <c r="D4" s="16">
         <f>IF(OR(A4="",B4=0),"",C4/B4)</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>Gerente</t>
         </is>
       </c>
-      <c r="B5" s="22">
+      <c r="B5" s="25">
         <f>IF(A5="","",COUNTIF('Funcionários'!$A$5:$A$34,A5))</f>
         <v/>
       </c>
-      <c r="C5" s="13">
+      <c r="C5" s="16">
         <f>IF(A5="","",SUMIF('Funcionários'!$A$5:$A$34,A5,'Funcionários'!$S$5:$S$34))</f>
         <v/>
       </c>
-      <c r="D5" s="13">
+      <c r="D5" s="16">
         <f>IF(OR(A5="",B5=0),"",C5/B5)</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="n"/>
-      <c r="B6" s="22">
+      <c r="A6" s="15" t="n"/>
+      <c r="B6" s="25">
         <f>IF(A6="","",COUNTIF('Funcionários'!$A$5:$A$34,A6))</f>
         <v/>
       </c>
-      <c r="C6" s="13">
+      <c r="C6" s="16">
         <f>IF(A6="","",SUMIF('Funcionários'!$A$5:$A$34,A6,'Funcionários'!$S$5:$S$34))</f>
         <v/>
       </c>
-      <c r="D6" s="13">
+      <c r="D6" s="16">
         <f>IF(OR(A6="",B6=0),"",C6/B6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="n"/>
-      <c r="B7" s="22">
+      <c r="A7" s="15" t="n"/>
+      <c r="B7" s="25">
         <f>IF(A7="","",COUNTIF('Funcionários'!$A$5:$A$34,A7))</f>
         <v/>
       </c>
-      <c r="C7" s="13">
+      <c r="C7" s="16">
         <f>IF(A7="","",SUMIF('Funcionários'!$A$5:$A$34,A7,'Funcionários'!$S$5:$S$34))</f>
         <v/>
       </c>
-      <c r="D7" s="13">
+      <c r="D7" s="16">
         <f>IF(OR(A7="",B7=0),"",C7/B7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="n"/>
-      <c r="B8" s="22">
+      <c r="A8" s="15" t="n"/>
+      <c r="B8" s="25">
         <f>IF(A8="","",COUNTIF('Funcionários'!$A$5:$A$34,A8))</f>
         <v/>
       </c>
-      <c r="C8" s="13">
+      <c r="C8" s="16">
         <f>IF(A8="","",SUMIF('Funcionários'!$A$5:$A$34,A8,'Funcionários'!$S$5:$S$34))</f>
         <v/>
       </c>
-      <c r="D8" s="13">
+      <c r="D8" s="16">
         <f>IF(OR(A8="",B8=0),"",C8/B8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="n"/>
-      <c r="B9" s="22">
+      <c r="A9" s="15" t="n"/>
+      <c r="B9" s="25">
         <f>IF(A9="","",COUNTIF('Funcionários'!$A$5:$A$34,A9))</f>
         <v/>
       </c>
-      <c r="C9" s="13">
+      <c r="C9" s="16">
         <f>IF(A9="","",SUMIF('Funcionários'!$A$5:$A$34,A9,'Funcionários'!$S$5:$S$34))</f>
         <v/>
       </c>
-      <c r="D9" s="13">
+      <c r="D9" s="16">
         <f>IF(OR(A9="",B9=0),"",C9/B9)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="n"/>
-      <c r="B10" s="22">
+      <c r="A10" s="15" t="n"/>
+      <c r="B10" s="25">
         <f>IF(A10="","",COUNTIF('Funcionários'!$A$5:$A$34,A10))</f>
         <v/>
       </c>
-      <c r="C10" s="13">
+      <c r="C10" s="16">
         <f>IF(A10="","",SUMIF('Funcionários'!$A$5:$A$34,A10,'Funcionários'!$S$5:$S$34))</f>
         <v/>
       </c>
-      <c r="D10" s="13">
+      <c r="D10" s="16">
         <f>IF(OR(A10="",B10=0),"",C10/B10)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="n"/>
-      <c r="B11" s="22">
+      <c r="A11" s="15" t="n"/>
+      <c r="B11" s="25">
         <f>IF(A11="","",COUNTIF('Funcionários'!$A$5:$A$34,A11))</f>
         <v/>
       </c>
-      <c r="C11" s="13">
+      <c r="C11" s="16">
         <f>IF(A11="","",SUMIF('Funcionários'!$A$5:$A$34,A11,'Funcionários'!$S$5:$S$34))</f>
         <v/>
       </c>
-      <c r="D11" s="13">
+      <c r="D11" s="16">
         <f>IF(OR(A11="",B11=0),"",C11/B11)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="n"/>
-      <c r="B12" s="22">
+      <c r="A12" s="15" t="n"/>
+      <c r="B12" s="25">
         <f>IF(A12="","",COUNTIF('Funcionários'!$A$5:$A$34,A12))</f>
         <v/>
       </c>
-      <c r="C12" s="13">
+      <c r="C12" s="16">
         <f>IF(A12="","",SUMIF('Funcionários'!$A$5:$A$34,A12,'Funcionários'!$S$5:$S$34))</f>
         <v/>
       </c>
-      <c r="D12" s="13">
+      <c r="D12" s="16">
         <f>IF(OR(A12="",B12=0),"",C12/B12)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="n"/>
-      <c r="B13" s="22">
+      <c r="A13" s="15" t="n"/>
+      <c r="B13" s="25">
         <f>IF(A13="","",COUNTIF('Funcionários'!$A$5:$A$34,A13))</f>
         <v/>
       </c>
-      <c r="C13" s="13">
+      <c r="C13" s="16">
         <f>IF(A13="","",SUMIF('Funcionários'!$A$5:$A$34,A13,'Funcionários'!$S$5:$S$34))</f>
         <v/>
       </c>
-      <c r="D13" s="13">
+      <c r="D13" s="16">
         <f>IF(OR(A13="",B13=0),"",C13/B13)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="n"/>
-      <c r="B14" s="22">
+      <c r="A14" s="15" t="n"/>
+      <c r="B14" s="25">
         <f>IF(A14="","",COUNTIF('Funcionários'!$A$5:$A$34,A14))</f>
         <v/>
       </c>
-      <c r="C14" s="13">
+      <c r="C14" s="16">
         <f>IF(A14="","",SUMIF('Funcionários'!$A$5:$A$34,A14,'Funcionários'!$S$5:$S$34))</f>
         <v/>
       </c>
-      <c r="D14" s="13">
+      <c r="D14" s="16">
         <f>IF(OR(A14="",B14=0),"",C14/B14)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="n"/>
-      <c r="B15" s="22">
+      <c r="A15" s="15" t="n"/>
+      <c r="B15" s="25">
         <f>IF(A15="","",COUNTIF('Funcionários'!$A$5:$A$34,A15))</f>
         <v/>
       </c>
-      <c r="C15" s="13">
+      <c r="C15" s="16">
         <f>IF(A15="","",SUMIF('Funcionários'!$A$5:$A$34,A15,'Funcionários'!$S$5:$S$34))</f>
         <v/>
       </c>
-      <c r="D15" s="13">
+      <c r="D15" s="16">
         <f>IF(OR(A15="",B15=0),"",C15/B15)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="23" t="inlineStr">
+      <c r="A16" s="26" t="inlineStr">
         <is>
           <t>TOTAL GERAL</t>
         </is>
       </c>
-      <c r="B16" s="20">
+      <c r="B16" s="23">
         <f>SUM(B4:B15)</f>
         <v/>
       </c>
-      <c r="C16" s="21">
+      <c r="C16" s="24">
         <f>SUM(C4:C15)</f>
         <v/>
       </c>

</xml_diff>